<commit_message>
Corregir mapeo de posicion DC en Python, regenerar base de datos y forzar purga de cache en navegador
</commit_message>
<xml_diff>
--- a/lmi temp 9.xlsx
+++ b/lmi temp 9.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex1\Downloads\LMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E41347C0-7B64-4F37-9AE2-55B501422A05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B480AFF4-D8FF-4BD0-AC2E-3CFEB64F7D33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{37EE0A92-4687-43D8-82AB-58C1E8ACFD8D}"/>
+    <workbookView xWindow="22932" yWindow="3744" windowWidth="23256" windowHeight="12456" xr2:uid="{37EE0A92-4687-43D8-82AB-58C1E8ACFD8D}"/>
   </bookViews>
   <sheets>
     <sheet name="Registro Liga" sheetId="2" r:id="rId1"/>
@@ -3055,7 +3055,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -3075,9 +3075,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3440,27 +3441,27 @@
         <v>954</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>826</v>
+        <v>171</v>
       </c>
       <c r="C2" s="3">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="D2" s="3">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>953</v>
+        <v>947</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>794</v>
+        <v>35</v>
       </c>
       <c r="C3" s="3">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="D3" s="3">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
         <v>179</v>
@@ -3468,72 +3469,72 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>949</v>
+        <v>954</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>63</v>
+        <v>826</v>
       </c>
       <c r="C4" s="3">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D4" s="3">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
-        <v>949</v>
+        <v>137</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>62</v>
+        <v>147</v>
       </c>
       <c r="C5" s="3">
         <v>11</v>
       </c>
       <c r="D5" s="3">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>953</v>
+        <v>946</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>792</v>
+        <v>18</v>
       </c>
       <c r="C6" s="3">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="D6" s="3">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>954</v>
+        <v>950</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>815</v>
+        <v>92</v>
       </c>
       <c r="C7" s="3">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="D7" s="3">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>751</v>
+        <v>146</v>
       </c>
       <c r="C8" s="3">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D8" s="3">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -3541,52 +3542,50 @@
         <v>137</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="C9" s="3">
-        <v>11</v>
-      </c>
+        <v>141</v>
+      </c>
+      <c r="C9" s="3"/>
       <c r="D9" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>137</v>
+        <v>949</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>783</v>
+        <v>62</v>
       </c>
       <c r="C10" s="3">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D10" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="C11" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D11" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>41</v>
+        <v>152</v>
       </c>
       <c r="C12" s="3">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D12" s="3">
         <v>5</v>
@@ -3594,325 +3593,319 @@
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>96</v>
+        <v>60</v>
       </c>
       <c r="C13" s="3">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D13" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>950</v>
+        <v>954</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>97</v>
+        <v>815</v>
       </c>
       <c r="C14" s="3">
-        <v>7</v>
-      </c>
-      <c r="D14" s="3"/>
+        <v>10</v>
+      </c>
+      <c r="D14" s="3">
+        <v>4</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>946</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C15" s="3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D15" s="3">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>953</v>
+        <v>957</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="C16" s="3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D16" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>957</v>
+        <v>126</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="C17" s="3">
-        <v>6</v>
-      </c>
+        <v>130</v>
+      </c>
+      <c r="C17" s="3"/>
       <c r="D17" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C18" s="3">
-        <v>6</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="C18" s="3"/>
       <c r="D18" s="3">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>954</v>
+        <v>949</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>171</v>
+        <v>63</v>
       </c>
       <c r="C19" s="3">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D19" s="3">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
-        <v>947</v>
+        <v>137</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>35</v>
+        <v>783</v>
       </c>
       <c r="C20" s="3">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D20" s="3">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>950</v>
+        <v>946</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>82</v>
+        <v>27</v>
       </c>
       <c r="C21" s="3">
         <v>5</v>
       </c>
       <c r="D21" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>951</v>
+        <v>950</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>102</v>
+        <v>94</v>
       </c>
       <c r="C22" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D22" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>951</v>
+        <v>954</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>101</v>
+        <v>168</v>
       </c>
       <c r="C23" s="3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D23" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="C24" s="3">
-        <v>5</v>
-      </c>
-      <c r="D24" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="D24" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>947</v>
+        <v>126</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>33</v>
+        <v>133</v>
       </c>
       <c r="C25" s="3">
-        <v>5</v>
-      </c>
-      <c r="D25" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="D25" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>85</v>
+        <v>112</v>
       </c>
       <c r="C26" s="3">
-        <v>5</v>
-      </c>
-      <c r="D26" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="D26" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>137</v>
+        <v>945</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>146</v>
+        <v>3</v>
       </c>
       <c r="C27" s="3">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D27" s="3">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>946</v>
+        <v>950</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>16</v>
+        <v>93</v>
       </c>
       <c r="C28" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D28" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>946</v>
+        <v>950</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C29" s="3">
-        <v>5</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="C29" s="3"/>
       <c r="D29" s="3">
         <v>3</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C30" s="3">
-        <v>4</v>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="C30" s="3"/>
       <c r="D30" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
-        <v>945</v>
+        <v>948</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C31" s="3">
-        <v>4</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="C31" s="3"/>
       <c r="D31" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>118</v>
+        <v>945</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C32" s="3">
-        <v>4</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="C32" s="3"/>
       <c r="D32" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>946</v>
+        <v>137</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C33" s="3">
-        <v>4</v>
-      </c>
+        <v>138</v>
+      </c>
+      <c r="C33" s="3"/>
       <c r="D33" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="C34" s="3">
-        <v>4</v>
-      </c>
-      <c r="D34" s="3"/>
+        <v>140</v>
+      </c>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
-        <v>950</v>
+        <v>126</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>94</v>
+        <v>751</v>
       </c>
       <c r="C35" s="3">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D35" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
-        <v>126</v>
+        <v>950</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>134</v>
+        <v>96</v>
       </c>
       <c r="C36" s="3">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="D36" s="3">
         <v>2</v>
@@ -3920,13 +3913,13 @@
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
-        <v>947</v>
+        <v>957</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>42</v>
+        <v>159</v>
       </c>
       <c r="C37" s="3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D37" s="3">
         <v>2</v>
@@ -3934,13 +3927,13 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
-        <v>954</v>
+        <v>950</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>169</v>
+        <v>82</v>
       </c>
       <c r="C38" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D38" s="3">
         <v>2</v>
@@ -3948,13 +3941,13 @@
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
-        <v>952</v>
+        <v>951</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="C39" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D39" s="3">
         <v>2</v>
@@ -3962,66 +3955,72 @@
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
-        <v>947</v>
+        <v>951</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>36</v>
+        <v>101</v>
       </c>
       <c r="C40" s="3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D40" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>957</v>
+        <v>947</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>157</v>
+        <v>39</v>
       </c>
       <c r="C41" s="3">
-        <v>3</v>
-      </c>
-      <c r="D41" s="3"/>
+        <v>4</v>
+      </c>
+      <c r="D41" s="3">
+        <v>2</v>
+      </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
         <v>945</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C42" s="3">
-        <v>3</v>
-      </c>
-      <c r="D42" s="3"/>
+        <v>4</v>
+      </c>
+      <c r="D42" s="3">
+        <v>2</v>
+      </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>119</v>
+        <v>134</v>
       </c>
       <c r="C43" s="3">
         <v>3</v>
       </c>
-      <c r="D43" s="3"/>
+      <c r="D43" s="3">
+        <v>2</v>
+      </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
-        <v>957</v>
+        <v>947</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>158</v>
+        <v>42</v>
       </c>
       <c r="C44" s="3">
+        <v>3</v>
+      </c>
+      <c r="D44" s="3">
         <v>2</v>
-      </c>
-      <c r="D44" s="3">
-        <v>4</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
@@ -4029,27 +4028,27 @@
         <v>954</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C45" s="3">
+        <v>3</v>
+      </c>
+      <c r="D45" s="3">
         <v>2</v>
-      </c>
-      <c r="D45" s="3">
-        <v>3</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
-        <v>946</v>
+        <v>952</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>15</v>
+        <v>110</v>
       </c>
       <c r="C46" s="3">
+        <v>3</v>
+      </c>
+      <c r="D46" s="3">
         <v>2</v>
-      </c>
-      <c r="D46" s="3">
-        <v>3</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
@@ -4096,417 +4095,419 @@
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
-        <v>126</v>
+        <v>949</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>131</v>
+        <v>61</v>
       </c>
       <c r="C50" s="3">
+        <v>1</v>
+      </c>
+      <c r="D50" s="3">
         <v>2</v>
-      </c>
-      <c r="D50" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
-        <v>118</v>
+        <v>957</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>120</v>
+        <v>162</v>
       </c>
       <c r="C51" s="3">
+        <v>1</v>
+      </c>
+      <c r="D51" s="3">
         <v>2</v>
-      </c>
-      <c r="D51" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
-        <v>952</v>
+        <v>957</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>111</v>
+        <v>165</v>
       </c>
       <c r="C52" s="3">
+        <v>1</v>
+      </c>
+      <c r="D52" s="3">
         <v>2</v>
-      </c>
-      <c r="D52" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
-        <v>957</v>
+        <v>948</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>160</v>
+        <v>47</v>
       </c>
       <c r="C53" s="3">
+        <v>1</v>
+      </c>
+      <c r="D53" s="3">
         <v>2</v>
-      </c>
-      <c r="D53" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
-        <v>950</v>
+        <v>957</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>95</v>
+        <v>161</v>
       </c>
       <c r="C54" s="3">
+        <v>1</v>
+      </c>
+      <c r="D54" s="3">
         <v>2</v>
-      </c>
-      <c r="D54" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
-        <v>945</v>
+        <v>949</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>8</v>
+        <v>59</v>
       </c>
       <c r="C55" s="3">
+        <v>1</v>
+      </c>
+      <c r="D55" s="3">
         <v>2</v>
-      </c>
-      <c r="D55" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
-        <v>949</v>
+        <v>951</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="C56" s="3">
+        <v>1</v>
+      </c>
+      <c r="D56" s="3">
         <v>2</v>
-      </c>
-      <c r="D56" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
-        <v>945</v>
+        <v>948</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C57" s="3">
+        <v>45</v>
+      </c>
+      <c r="C57" s="3"/>
+      <c r="D57" s="3">
         <v>2</v>
-      </c>
-      <c r="D57" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
-        <v>137</v>
+        <v>947</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>144</v>
-      </c>
-      <c r="C58" s="3">
+        <v>37</v>
+      </c>
+      <c r="C58" s="3"/>
+      <c r="D58" s="3">
         <v>2</v>
-      </c>
-      <c r="D58" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
-        <v>952</v>
+        <v>947</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="C59" s="3">
+        <v>38</v>
+      </c>
+      <c r="C59" s="3"/>
+      <c r="D59" s="3">
         <v>2</v>
-      </c>
-      <c r="D59" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
-        <v>953</v>
+        <v>950</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="C60" s="3">
+        <v>81</v>
+      </c>
+      <c r="C60" s="3"/>
+      <c r="D60" s="3">
         <v>2</v>
       </c>
-      <c r="D60" s="3"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
-        <v>126</v>
+        <v>953</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="C61" s="3">
+        <v>802</v>
+      </c>
+      <c r="C61" s="3"/>
+      <c r="D61" s="3">
         <v>2</v>
       </c>
-      <c r="D61" s="3"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
-        <v>953</v>
+        <v>954</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>804</v>
-      </c>
-      <c r="C62" s="3">
+        <v>167</v>
+      </c>
+      <c r="C62" s="3"/>
+      <c r="D62" s="3">
         <v>2</v>
       </c>
-      <c r="D62" s="3"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
-        <v>957</v>
+        <v>945</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C63" s="3">
+        <v>610</v>
+      </c>
+      <c r="C63" s="6"/>
+      <c r="D63" s="3">
         <v>2</v>
       </c>
-      <c r="D63" s="3"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>114</v>
+        <v>794</v>
       </c>
       <c r="C64" s="3">
-        <v>2</v>
-      </c>
-      <c r="D64" s="3"/>
+        <v>15</v>
+      </c>
+      <c r="D64" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
-        <v>952</v>
+        <v>953</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>108</v>
+        <v>792</v>
       </c>
       <c r="C65" s="3">
-        <v>2</v>
-      </c>
-      <c r="D65" s="3"/>
+        <v>11</v>
+      </c>
+      <c r="D65" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
-        <v>137</v>
+        <v>948</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>142</v>
+        <v>48</v>
       </c>
       <c r="C66" s="3">
-        <v>2</v>
-      </c>
-      <c r="D66" s="3"/>
+        <v>9</v>
+      </c>
+      <c r="D66" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
-        <v>949</v>
+        <v>947</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>75</v>
+        <v>34</v>
       </c>
       <c r="C67" s="3">
-        <v>2</v>
-      </c>
-      <c r="D67" s="3"/>
+        <v>6</v>
+      </c>
+      <c r="D67" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
-        <v>950</v>
+        <v>118</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>92</v>
+        <v>125</v>
       </c>
       <c r="C68" s="3">
+        <v>4</v>
+      </c>
+      <c r="D68" s="3">
         <v>1</v>
-      </c>
-      <c r="D68" s="3">
-        <v>7</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
-        <v>949</v>
+        <v>946</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="C69" s="3">
+        <v>4</v>
+      </c>
+      <c r="D69" s="3">
         <v>1</v>
-      </c>
-      <c r="D69" s="3">
-        <v>5</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
-        <v>126</v>
+        <v>947</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>133</v>
+        <v>36</v>
       </c>
       <c r="C70" s="3">
+        <v>3</v>
+      </c>
+      <c r="D70" s="3">
         <v>1</v>
-      </c>
-      <c r="D70" s="3">
-        <v>3</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
-        <v>952</v>
+        <v>126</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>112</v>
+        <v>131</v>
       </c>
       <c r="C71" s="3">
+        <v>2</v>
+      </c>
+      <c r="D71" s="3">
         <v>1</v>
-      </c>
-      <c r="D71" s="3">
-        <v>3</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
-        <v>945</v>
+        <v>118</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>3</v>
+        <v>120</v>
       </c>
       <c r="C72" s="3">
+        <v>2</v>
+      </c>
+      <c r="D72" s="3">
         <v>1</v>
-      </c>
-      <c r="D72" s="3">
-        <v>3</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>93</v>
+        <v>111</v>
       </c>
       <c r="C73" s="3">
+        <v>2</v>
+      </c>
+      <c r="D73" s="3">
         <v>1</v>
-      </c>
-      <c r="D73" s="3">
-        <v>3</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
-        <v>949</v>
+        <v>957</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>61</v>
+        <v>160</v>
       </c>
       <c r="C74" s="3">
+        <v>2</v>
+      </c>
+      <c r="D74" s="3">
         <v>1</v>
-      </c>
-      <c r="D74" s="3">
-        <v>2</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
-        <v>957</v>
+        <v>950</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>162</v>
+        <v>95</v>
       </c>
       <c r="C75" s="3">
+        <v>2</v>
+      </c>
+      <c r="D75" s="3">
         <v>1</v>
-      </c>
-      <c r="D75" s="3">
-        <v>2</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
-        <v>957</v>
+        <v>945</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>165</v>
+        <v>8</v>
       </c>
       <c r="C76" s="3">
+        <v>2</v>
+      </c>
+      <c r="D76" s="3">
         <v>1</v>
-      </c>
-      <c r="D76" s="3">
-        <v>2</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" s="3" t="s">
-        <v>948</v>
+        <v>949</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="C77" s="3">
+        <v>2</v>
+      </c>
+      <c r="D77" s="3">
         <v>1</v>
-      </c>
-      <c r="D77" s="3">
-        <v>2</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" s="3" t="s">
-        <v>957</v>
+        <v>945</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>161</v>
+        <v>4</v>
       </c>
       <c r="C78" s="3">
+        <v>2</v>
+      </c>
+      <c r="D78" s="3">
         <v>1</v>
-      </c>
-      <c r="D78" s="3">
-        <v>2</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" s="3" t="s">
-        <v>949</v>
+        <v>137</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>59</v>
+        <v>144</v>
       </c>
       <c r="C79" s="3">
+        <v>2</v>
+      </c>
+      <c r="D79" s="3">
         <v>1</v>
-      </c>
-      <c r="D79" s="3">
-        <v>2</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="3" t="s">
-        <v>946</v>
+        <v>952</v>
       </c>
       <c r="B80" s="3" t="s">
-        <v>25</v>
+        <v>115</v>
       </c>
       <c r="C80" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D80" s="3">
         <v>1</v>
@@ -4514,10 +4515,10 @@
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
-        <v>118</v>
+        <v>946</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>122</v>
+        <v>25</v>
       </c>
       <c r="C81" s="3">
         <v>1</v>
@@ -4531,10 +4532,10 @@
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="3" t="s">
-        <v>953</v>
+        <v>118</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>153</v>
+        <v>122</v>
       </c>
       <c r="C82" s="3">
         <v>1</v>
@@ -4545,10 +4546,10 @@
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="3" t="s">
-        <v>126</v>
+        <v>953</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>128</v>
+        <v>153</v>
       </c>
       <c r="C83" s="3">
         <v>1</v>
@@ -4559,10 +4560,10 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="3" t="s">
-        <v>950</v>
+        <v>126</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>89</v>
+        <v>128</v>
       </c>
       <c r="C84" s="3">
         <v>1</v>
@@ -4573,10 +4574,10 @@
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="3" t="s">
-        <v>118</v>
+        <v>950</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>124</v>
+        <v>89</v>
       </c>
       <c r="C85" s="3">
         <v>1</v>
@@ -4587,10 +4588,10 @@
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="3" t="s">
-        <v>954</v>
+        <v>118</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>170</v>
+        <v>124</v>
       </c>
       <c r="C86" s="3">
         <v>1</v>
@@ -4601,10 +4602,10 @@
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="3" t="s">
-        <v>951</v>
+        <v>954</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>103</v>
+        <v>170</v>
       </c>
       <c r="C87" s="3">
         <v>1</v>
@@ -4618,7 +4619,7 @@
         <v>951</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C88" s="3">
         <v>1</v>
@@ -4632,13 +4633,13 @@
         <v>951</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C89" s="3">
         <v>1</v>
       </c>
       <c r="D89" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
@@ -4727,232 +4728,232 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="3" t="s">
-        <v>945</v>
+        <v>137</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>2</v>
+        <v>145</v>
       </c>
       <c r="C96" s="3">
         <v>1</v>
       </c>
-      <c r="D96" s="3"/>
+      <c r="D96" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" s="3" t="s">
-        <v>947</v>
+        <v>949</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C97" s="3">
+        <v>56</v>
+      </c>
+      <c r="C97" s="3"/>
+      <c r="D97" s="3">
         <v>1</v>
       </c>
-      <c r="D97" s="3"/>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
-        <v>945</v>
+        <v>947</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C98" s="3">
+        <v>38</v>
+      </c>
+      <c r="C98" s="3"/>
+      <c r="D98" s="3">
         <v>1</v>
       </c>
-      <c r="D98" s="3"/>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" s="3" t="s">
-        <v>952</v>
+        <v>118</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="C99" s="3">
+        <v>123</v>
+      </c>
+      <c r="C99" s="3"/>
+      <c r="D99" s="3">
         <v>1</v>
       </c>
-      <c r="D99" s="3"/>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" s="3" t="s">
-        <v>951</v>
+        <v>952</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C100" s="3">
+        <v>107</v>
+      </c>
+      <c r="C100" s="3"/>
+      <c r="D100" s="3">
         <v>1</v>
       </c>
-      <c r="D100" s="3"/>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" s="3" t="s">
-        <v>952</v>
+        <v>118</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C101" s="3">
+        <v>121</v>
+      </c>
+      <c r="C101" s="3"/>
+      <c r="D101" s="3">
         <v>1</v>
       </c>
-      <c r="D101" s="3"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" s="3" t="s">
-        <v>950</v>
+        <v>126</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C102" s="3">
+        <v>129</v>
+      </c>
+      <c r="C102" s="3"/>
+      <c r="D102" s="3">
         <v>1</v>
       </c>
-      <c r="D102" s="3"/>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" s="3" t="s">
-        <v>945</v>
+        <v>948</v>
       </c>
       <c r="B103" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="C103" s="3"/>
+      <c r="D103" s="3">
         <v>1</v>
       </c>
-      <c r="C103" s="3">
-        <v>1</v>
-      </c>
-      <c r="D103" s="3"/>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" s="3" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C104" s="3">
+        <v>31</v>
+      </c>
+      <c r="C104" s="3"/>
+      <c r="D104" s="3">
         <v>1</v>
       </c>
-      <c r="D104" s="3"/>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" s="3" t="s">
-        <v>126</v>
+        <v>953</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="C105" s="3">
+        <v>150</v>
+      </c>
+      <c r="C105" s="3"/>
+      <c r="D105" s="3">
         <v>1</v>
       </c>
-      <c r="D105" s="3"/>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" s="3" t="s">
-        <v>137</v>
+        <v>950</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C106" s="3">
+        <v>80</v>
+      </c>
+      <c r="C106" s="3"/>
+      <c r="D106" s="3">
         <v>1</v>
       </c>
-      <c r="D106" s="3"/>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" s="3" t="s">
-        <v>954</v>
+        <v>952</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="C107" s="3">
+        <v>106</v>
+      </c>
+      <c r="C107" s="3"/>
+      <c r="D107" s="3">
         <v>1</v>
       </c>
-      <c r="D107" s="3"/>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" s="3" t="s">
-        <v>954</v>
+        <v>957</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="C108" s="3">
+        <v>164</v>
+      </c>
+      <c r="C108" s="3"/>
+      <c r="D108" s="3">
         <v>1</v>
       </c>
-      <c r="D108" s="3"/>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" s="3" t="s">
-        <v>137</v>
+        <v>949</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="C109" s="3">
-        <v>1</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="C109" s="3"/>
       <c r="D109" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" s="3" t="s">
-        <v>118</v>
+        <v>951</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>738</v>
-      </c>
-      <c r="C110" s="6">
+        <v>104</v>
+      </c>
+      <c r="C110" s="3"/>
+      <c r="D110" s="3">
         <v>1</v>
       </c>
-      <c r="D110" s="6"/>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" s="3" t="s">
-        <v>945</v>
+        <v>948</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>613</v>
-      </c>
-      <c r="C111" s="3">
+        <v>49</v>
+      </c>
+      <c r="C111" s="3"/>
+      <c r="D111" s="3">
         <v>1</v>
       </c>
-      <c r="D111" s="6"/>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" s="3" t="s">
-        <v>118</v>
+        <v>947</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>724</v>
-      </c>
-      <c r="C112" s="6">
+        <v>40</v>
+      </c>
+      <c r="C112" s="3"/>
+      <c r="D112" s="3">
         <v>1</v>
       </c>
-      <c r="D112" s="6"/>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" s="3" t="s">
-        <v>126</v>
+        <v>953</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>130</v>
+        <v>154</v>
       </c>
       <c r="C113" s="3"/>
       <c r="D113" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" s="3" t="s">
-        <v>137</v>
+        <v>948</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>141</v>
+        <v>650</v>
       </c>
       <c r="C114" s="3"/>
       <c r="D114" s="3">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.3">
@@ -4960,503 +4961,516 @@
         <v>953</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>151</v>
+        <v>786</v>
       </c>
       <c r="C115" s="3"/>
       <c r="D115" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A116" s="3" t="s">
-        <v>950</v>
+        <v>949</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>77</v>
+        <v>68</v>
       </c>
       <c r="C116" s="3"/>
       <c r="D116" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" s="3" t="s">
-        <v>953</v>
+        <v>949</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>149</v>
+        <v>71</v>
       </c>
       <c r="C117" s="3"/>
       <c r="D117" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A118" s="3" t="s">
-        <v>948</v>
+        <v>137</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>50</v>
+        <v>772</v>
       </c>
       <c r="C118" s="3"/>
       <c r="D118" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A119" s="3" t="s">
-        <v>945</v>
+        <v>950</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C119" s="3"/>
+        <v>84</v>
+      </c>
+      <c r="C119" s="6"/>
       <c r="D119" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A120" s="3" t="s">
-        <v>948</v>
+        <v>118</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C120" s="3"/>
+        <v>732</v>
+      </c>
+      <c r="C120" s="6"/>
       <c r="D120" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A121" s="3" t="s">
-        <v>947</v>
+        <v>946</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C121" s="3"/>
+        <v>13</v>
+      </c>
+      <c r="C121" s="6"/>
       <c r="D121" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A122" s="3" t="s">
-        <v>947</v>
+        <v>118</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C122" s="3"/>
-      <c r="D122" s="3">
-        <v>2</v>
+        <v>737</v>
+      </c>
+      <c r="C122" s="6"/>
+      <c r="D122" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A123" s="3" t="s">
-        <v>950</v>
+        <v>118</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C123" s="3"/>
-      <c r="D123" s="3">
-        <v>2</v>
+        <v>739</v>
+      </c>
+      <c r="C123" s="6"/>
+      <c r="D123" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A124" s="3" t="s">
-        <v>137</v>
+        <v>954</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>138</v>
+        <v>172</v>
       </c>
       <c r="C124" s="3"/>
       <c r="D124" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A125" s="3" t="s">
-        <v>137</v>
+        <v>951</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C125" s="3"/>
+        <v>692</v>
+      </c>
+      <c r="C125" s="6"/>
       <c r="D125" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A126" s="3" t="s">
-        <v>953</v>
+        <v>950</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>802</v>
-      </c>
-      <c r="C126" s="3"/>
-      <c r="D126" s="3">
-        <v>2</v>
-      </c>
+        <v>97</v>
+      </c>
+      <c r="C126" s="3">
+        <v>7</v>
+      </c>
+      <c r="D126" s="3"/>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A127" s="3" t="s">
-        <v>954</v>
+        <v>948</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="C127" s="3"/>
-      <c r="D127" s="3">
-        <v>2</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C127" s="3">
+        <v>5</v>
+      </c>
+      <c r="D127" s="3"/>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A128" s="3" t="s">
-        <v>945</v>
+        <v>947</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>610</v>
-      </c>
-      <c r="C128" s="6"/>
-      <c r="D128" s="3">
-        <v>2</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="C128" s="3">
+        <v>5</v>
+      </c>
+      <c r="D128" s="3"/>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A129" s="3" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C129" s="3"/>
-      <c r="D129" s="3">
-        <v>1</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="C129" s="3">
+        <v>5</v>
+      </c>
+      <c r="D129" s="3"/>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A130" s="3" t="s">
-        <v>947</v>
+        <v>126</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C130" s="3"/>
-      <c r="D130" s="3">
-        <v>1</v>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="C130" s="3">
+        <v>4</v>
+      </c>
+      <c r="D130" s="3"/>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A131" s="3" t="s">
-        <v>118</v>
+        <v>957</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C131" s="3"/>
-      <c r="D131" s="3">
-        <v>1</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="C131" s="3">
+        <v>3</v>
+      </c>
+      <c r="D131" s="3"/>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A132" s="3" t="s">
-        <v>952</v>
+        <v>945</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="C132" s="3"/>
-      <c r="D132" s="3">
-        <v>1</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="C132" s="3">
+        <v>3</v>
+      </c>
+      <c r="D132" s="3"/>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" s="3" t="s">
         <v>118</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C133" s="3"/>
-      <c r="D133" s="3">
-        <v>1</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="C133" s="3">
+        <v>3</v>
+      </c>
+      <c r="D133" s="3"/>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A134" s="3" t="s">
-        <v>126</v>
+        <v>953</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C134" s="3"/>
-      <c r="D134" s="3">
-        <v>1</v>
-      </c>
+        <v>155</v>
+      </c>
+      <c r="C134" s="3">
+        <v>2</v>
+      </c>
+      <c r="D134" s="3"/>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A135" s="3" t="s">
-        <v>948</v>
+        <v>126</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C135" s="3"/>
-      <c r="D135" s="3">
-        <v>1</v>
-      </c>
+        <v>127</v>
+      </c>
+      <c r="C135" s="3">
+        <v>2</v>
+      </c>
+      <c r="D135" s="3"/>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A136" s="3" t="s">
-        <v>947</v>
+        <v>953</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C136" s="3"/>
-      <c r="D136" s="3">
-        <v>1</v>
-      </c>
+        <v>804</v>
+      </c>
+      <c r="C136" s="3">
+        <v>2</v>
+      </c>
+      <c r="D136" s="3"/>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A137" s="3" t="s">
-        <v>953</v>
+        <v>957</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="C137" s="3"/>
-      <c r="D137" s="3">
-        <v>1</v>
-      </c>
+        <v>166</v>
+      </c>
+      <c r="C137" s="3">
+        <v>2</v>
+      </c>
+      <c r="D137" s="3"/>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A138" s="3" t="s">
-        <v>950</v>
+        <v>952</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C138" s="3"/>
-      <c r="D138" s="3">
-        <v>1</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="C138" s="3">
+        <v>2</v>
+      </c>
+      <c r="D138" s="3"/>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A139" s="3" t="s">
         <v>952</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C139" s="1"/>
-      <c r="D139" s="1">
-        <v>1</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="C139" s="9">
+        <v>2</v>
+      </c>
+      <c r="D139" s="9"/>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A140" s="3" t="s">
-        <v>957</v>
+        <v>137</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="C140" s="1"/>
-      <c r="D140" s="1">
-        <v>1</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="C140" s="9">
+        <v>2</v>
+      </c>
+      <c r="D140" s="9"/>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A141" s="3" t="s">
         <v>949</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C141" s="1"/>
-      <c r="D141" s="1">
-        <v>1</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="C141" s="9">
+        <v>2</v>
+      </c>
+      <c r="D141" s="9"/>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A142" s="3" t="s">
-        <v>951</v>
+        <v>945</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="C142" s="1"/>
-      <c r="D142" s="1">
+        <v>2</v>
+      </c>
+      <c r="C142" s="9">
         <v>1</v>
       </c>
+      <c r="D142" s="9"/>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A143" s="3" t="s">
-        <v>948</v>
+        <v>947</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C143" s="1"/>
-      <c r="D143" s="1">
+        <v>32</v>
+      </c>
+      <c r="C143" s="9">
         <v>1</v>
       </c>
+      <c r="D143" s="9"/>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A144" s="3" t="s">
-        <v>947</v>
+        <v>945</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C144" s="1"/>
-      <c r="D144" s="1">
+        <v>0</v>
+      </c>
+      <c r="C144" s="9">
         <v>1</v>
       </c>
+      <c r="D144" s="9"/>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A145" s="3" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="C145" s="1"/>
-      <c r="D145" s="1">
+        <v>116</v>
+      </c>
+      <c r="C145" s="9">
         <v>1</v>
       </c>
+      <c r="D145" s="9"/>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A146" s="3" t="s">
-        <v>948</v>
+        <v>951</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>650</v>
-      </c>
-      <c r="C146" s="1"/>
-      <c r="D146" s="1">
+        <v>98</v>
+      </c>
+      <c r="C146" s="9">
         <v>1</v>
       </c>
+      <c r="D146" s="9"/>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A147" s="3" t="s">
-        <v>953</v>
+        <v>952</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>786</v>
-      </c>
-      <c r="C147" s="1"/>
-      <c r="D147" s="1">
+        <v>113</v>
+      </c>
+      <c r="C147" s="9">
         <v>1</v>
       </c>
+      <c r="D147" s="9"/>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A148" s="3" t="s">
-        <v>949</v>
+        <v>950</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C148" s="1"/>
-      <c r="D148" s="1">
+        <v>88</v>
+      </c>
+      <c r="C148" s="9">
         <v>1</v>
       </c>
+      <c r="D148" s="9"/>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A149" s="3" t="s">
-        <v>949</v>
+        <v>945</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C149" s="1"/>
-      <c r="D149" s="1">
         <v>1</v>
       </c>
+      <c r="C149" s="9">
+        <v>1</v>
+      </c>
+      <c r="D149" s="9"/>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A150" s="3" t="s">
-        <v>137</v>
+        <v>948</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>772</v>
-      </c>
-      <c r="C150" s="1"/>
-      <c r="D150" s="1">
+        <v>52</v>
+      </c>
+      <c r="C150" s="9">
         <v>1</v>
       </c>
+      <c r="D150" s="9"/>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A151" s="3" t="s">
-        <v>950</v>
+        <v>126</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="D151" s="1">
+        <v>135</v>
+      </c>
+      <c r="C151" s="9">
         <v>1</v>
       </c>
+      <c r="D151" s="9"/>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A152" s="3" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>732</v>
-      </c>
-      <c r="D152" s="1">
+        <v>143</v>
+      </c>
+      <c r="C152" s="9">
         <v>1</v>
       </c>
+      <c r="D152" s="9"/>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A153" s="3" t="s">
-        <v>946</v>
+        <v>954</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D153" s="1">
+        <v>173</v>
+      </c>
+      <c r="C153" s="9">
         <v>1</v>
       </c>
+      <c r="D153" s="9"/>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A154" s="3" t="s">
-        <v>118</v>
+        <v>954</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>737</v>
-      </c>
-      <c r="D154">
+        <v>174</v>
+      </c>
+      <c r="C154" s="9">
         <v>1</v>
       </c>
+      <c r="D154" s="9"/>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A155" s="3" t="s">
         <v>118</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>739</v>
-      </c>
-      <c r="D155">
+        <v>738</v>
+      </c>
+      <c r="C155" s="10">
         <v>1</v>
       </c>
+      <c r="D155" s="10"/>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A156" s="3" t="s">
-        <v>954</v>
+        <v>945</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="C156" s="1"/>
-      <c r="D156" s="1">
+        <v>613</v>
+      </c>
+      <c r="C156" s="9">
         <v>1</v>
       </c>
+      <c r="D156" s="10"/>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A157" s="3"/>
-      <c r="B157" s="3"/>
+      <c r="A157" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B157" s="3" t="s">
+        <v>724</v>
+      </c>
+      <c r="C157" s="10">
+        <v>1</v>
+      </c>
+      <c r="D157" s="10"/>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A158" s="3"/>
@@ -5469,8 +5483,6 @@
     <row r="160" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A160" s="3"/>
       <c r="B160" s="3"/>
-      <c r="C160" s="1"/>
-      <c r="D160" s="1"/>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A161" s="3"/>
@@ -5481,12 +5493,12 @@
     <row r="162" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A162" s="3"/>
       <c r="B162" s="3"/>
+      <c r="C162" s="1"/>
+      <c r="D162" s="1"/>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A163" s="3"/>
       <c r="B163" s="3"/>
-      <c r="C163" s="1"/>
-      <c r="D163" s="1"/>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A164" s="3"/>
@@ -5539,6 +5551,8 @@
     <row r="172" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A172" s="3"/>
       <c r="B172" s="3"/>
+      <c r="C172" s="1"/>
+      <c r="D172" s="1"/>
     </row>
     <row r="173" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A173" s="3"/>
@@ -5555,8 +5569,6 @@
     <row r="176" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A176" s="3"/>
       <c r="B176" s="3"/>
-      <c r="C176" s="1"/>
-      <c r="D176" s="1"/>
     </row>
     <row r="177" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A177" s="3"/>
@@ -5615,6 +5627,8 @@
     <row r="186" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A186" s="3"/>
       <c r="B186" s="3"/>
+      <c r="C186" s="1"/>
+      <c r="D186" s="1"/>
     </row>
     <row r="187" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A187" s="3"/>
@@ -5641,8 +5655,8 @@
       <c r="B192" s="3"/>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A193" s="1"/>
-      <c r="B193" s="1"/>
+      <c r="A193" s="9"/>
+      <c r="B193" s="9"/>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A194" s="1"/>
@@ -5680,6 +5694,7 @@
     <row r="202" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A202" s="1"/>
       <c r="B202" s="1"/>
+      <c r="D202" s="10"/>
     </row>
     <row r="203" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A203" s="1"/>
@@ -5693,11 +5708,13 @@
     <row r="205" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A205" s="1"/>
       <c r="B205" s="1"/>
+      <c r="C205" s="10"/>
       <c r="D205" s="8"/>
     </row>
     <row r="206" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A206" s="1"/>
       <c r="B206" s="1"/>
+      <c r="D206" s="10"/>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A207" s="1"/>
@@ -5715,26 +5732,20 @@
     <row r="210" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A210" s="1"/>
       <c r="B210" s="1"/>
+      <c r="D210" s="10"/>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A211" s="1" t="s">
-        <v>951</v>
-      </c>
-      <c r="B211" s="1" t="s">
-        <v>691</v>
-      </c>
-      <c r="C211" s="9">
-        <v>1</v>
-      </c>
+      <c r="A211" s="1"/>
+      <c r="B211" s="1"/>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A212" s="1" t="s">
         <v>951</v>
       </c>
       <c r="B212" s="1" t="s">
-        <v>692</v>
-      </c>
-      <c r="D212" s="9">
+        <v>691</v>
+      </c>
+      <c r="C212" s="1">
         <v>1</v>
       </c>
     </row>
@@ -5748,7 +5759,7 @@
       <c r="C213">
         <v>1</v>
       </c>
-      <c r="D213" s="9"/>
+      <c r="D213" s="1"/>
     </row>
     <row r="214" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A214" s="1"/>
@@ -7676,8 +7687,8 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D213" xr:uid="{3FE09B2D-DD5D-432F-829D-D273A0AAABBF}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D210">
-      <sortCondition descending="1" ref="C1:C210"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D213">
+      <sortCondition descending="1" ref="D1:D213"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>

<commit_message>
Actualizacion visual de plataforma LMI Temporada 9, brackets dinamicos desde Excel, y optimizacion de plantillas
</commit_message>
<xml_diff>
--- a/lmi temp 9.xlsx
+++ b/lmi temp 9.xlsx
@@ -8,68 +8,72 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex1\Downloads\LMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{213B9CBF-0764-447B-9647-93481520F74B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AACFE2AE-F619-4705-AB56-B8BE1EF9D3AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="3744" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{37EE0A92-4687-43D8-82AB-58C1E8ACFD8D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{37EE0A92-4687-43D8-82AB-58C1E8ACFD8D}"/>
   </bookViews>
   <sheets>
     <sheet name="Registro Liga" sheetId="2" r:id="rId1"/>
-    <sheet name="Registro Champions" sheetId="6" r:id="rId2"/>
-    <sheet name="RegistroEstelar" sheetId="7" r:id="rId3"/>
-    <sheet name="BD" sheetId="4" r:id="rId4"/>
-    <sheet name="Lista" sheetId="1" r:id="rId5"/>
+    <sheet name="ChampionsLeague" sheetId="9" r:id="rId2"/>
+    <sheet name="CopaEstelar" sheetId="8" r:id="rId3"/>
+    <sheet name="Registro Champions" sheetId="6" r:id="rId4"/>
+    <sheet name="RegistroEstelar" sheetId="7" r:id="rId5"/>
+    <sheet name="BD" sheetId="4" r:id="rId6"/>
+    <sheet name="Lista" sheetId="1" r:id="rId7"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Registro Champions'!$A$1:$D$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Registro Liga'!$A$1:$D$218</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">RegistroEstelar!$A$1:$D$1</definedName>
     <definedName name="AC_Milan">BD!$E$2:$E$24</definedName>
     <definedName name="AC_Milán">Lista!$E$2:$E$1048576</definedName>
     <definedName name="AcMilan">Lista!$E$2:$E$1048576</definedName>
-    <definedName name="Arsenal" localSheetId="3">BD!$K$2:$K$24</definedName>
+    <definedName name="Arsenal" localSheetId="5">BD!$K$2:$K$24</definedName>
     <definedName name="Arsenal">Lista!$K$2:$K$1048576</definedName>
     <definedName name="AstonVilla">Lista!$I$2:$I$1048576</definedName>
     <definedName name="Bayer_Munich">Lista!$O$2:$O$1048576</definedName>
-    <definedName name="Bayern_Leverkusen" localSheetId="3">BD!$F$2:$F$24</definedName>
+    <definedName name="Bayern_Leverkusen" localSheetId="5">BD!$F$2:$F$24</definedName>
     <definedName name="Bayern_Leverkusen">Lista!$F$2:$F$1048576</definedName>
     <definedName name="Bayern_Munich">BD!$O$2:$O$24</definedName>
-    <definedName name="Boca_Juniors" localSheetId="3">BD!$H$2:$H$24</definedName>
+    <definedName name="Boca_Juniors" localSheetId="5">BD!$H$2:$H$24</definedName>
     <definedName name="Boca_Juniors">Lista!$H$2:$H$1048576</definedName>
     <definedName name="BocaJuniors">Lista!$H$2:$H$1048576</definedName>
-    <definedName name="Como_1907" localSheetId="3">BD!$L$2:$L$24</definedName>
+    <definedName name="Como_1907" localSheetId="5">BD!$L$2:$L$24</definedName>
     <definedName name="COMO_1907">Lista!$L$2:$L$1048576</definedName>
     <definedName name="Como1907">Lista!$M$2:$M$1048576</definedName>
-    <definedName name="FC_Barcelona" localSheetId="3">BD!$C$2:$C$24</definedName>
+    <definedName name="FC_Barcelona" localSheetId="5">BD!$C$2:$C$24</definedName>
     <definedName name="FC_Barcelona">Lista!$C$2:$C$1048576</definedName>
     <definedName name="FcBarcelona">Lista!$C$2:$C$1048576</definedName>
-    <definedName name="Galatasaray" localSheetId="3">BD!$I$2:$I$24</definedName>
+    <definedName name="Galatasaray" localSheetId="5">BD!$I$2:$I$24</definedName>
     <definedName name="GALATASARAY">Lista!$I$2:$I$1048576</definedName>
-    <definedName name="Hellas_Verona" localSheetId="3">BD!$N$2:$N$24</definedName>
+    <definedName name="Hellas_Verona" localSheetId="5">BD!$N$2:$N$24</definedName>
     <definedName name="Hellas_Verona">Lista!$N$2:$N$1048576</definedName>
-    <definedName name="Inter_de_Milan" localSheetId="3">BD!$A$2:$A$24</definedName>
+    <definedName name="Inter_de_Milan" localSheetId="5">BD!$A$2:$A$24</definedName>
     <definedName name="Inter_de_Milan">Lista!$A$2:$A$1048576</definedName>
     <definedName name="InterMilan">Lista!$A$2:$A$1048576</definedName>
     <definedName name="Leverkusen">Lista!$F$2:$F$1048576</definedName>
-    <definedName name="Manchester_United" localSheetId="3">BD!$P$2:$P$24</definedName>
+    <definedName name="Manchester_United" localSheetId="5">BD!$P$2:$P$24</definedName>
     <definedName name="Manchester_United">Lista!$P$2:$P$1048576</definedName>
-    <definedName name="Melbourne_City" localSheetId="3">BD!$Q$2:$Q$24</definedName>
+    <definedName name="Melbourne_City" localSheetId="5">BD!$Q$2:$Q$24</definedName>
     <definedName name="Melbourne_City">Lista!$Q$2:$Q$1048576</definedName>
     <definedName name="PARIS_SAINT___GERMAIN">Lista!$J$2:$J$1048576</definedName>
-    <definedName name="PSG" localSheetId="3">BD!$J$2:$J$24</definedName>
+    <definedName name="PSG" localSheetId="5">BD!$J$2:$J$24</definedName>
     <definedName name="PSG">Lista!$K$2:$K$1048576</definedName>
-    <definedName name="RB_Leipzig" localSheetId="3">BD!$G$2:$G$24</definedName>
+    <definedName name="RB_Leipzig" localSheetId="5">BD!$G$2:$G$24</definedName>
     <definedName name="RB_LEIPZIG">Lista!$G$2:$G$1048576</definedName>
     <definedName name="RBLeipzig">Lista!$G$2:$G$1048576</definedName>
-    <definedName name="Real_Madrid" localSheetId="3">BD!$B$2:$B$24</definedName>
+    <definedName name="Real_Madrid" localSheetId="5">BD!$B$2:$B$24</definedName>
     <definedName name="Real_Madrid">Lista!$B$2:$B$1048576</definedName>
     <definedName name="RealMadrid">Lista!$B$2:$B$1048576</definedName>
     <definedName name="Sparta">Lista!$P$2:$P$1048576</definedName>
-    <definedName name="Terengganu_FC" localSheetId="3">BD!$D$2:$D$24</definedName>
+    <definedName name="Terengganu_FC" localSheetId="5">BD!$D$2:$D$24</definedName>
     <definedName name="Terengganu_FC">Lista!$D$2:$D$1048576</definedName>
     <definedName name="Terrengganu">Lista!$D$2:$D$1048576</definedName>
     <definedName name="Tottenham">Lista!$O$2:$O$1048576</definedName>
-    <definedName name="Tottenham_Hotspur" localSheetId="3">BD!$M$2:$M$24</definedName>
+    <definedName name="Tottenham_Hotspur" localSheetId="5">BD!$M$2:$M$24</definedName>
     <definedName name="Tottenham_Hotspur">Lista!$M$2:$M$1048576</definedName>
     <definedName name="United">Lista!$N$2:$N$1048576</definedName>
-    <definedName name="Wrexham" localSheetId="3">BD!$R$2:$R$24</definedName>
+    <definedName name="Wrexham" localSheetId="5">BD!$R$2:$R$24</definedName>
     <definedName name="WREXHAM">Lista!$R$2:$R$1048576</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -96,7 +100,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1012" uniqueCount="774">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1191" uniqueCount="798">
   <si>
     <t xml:space="preserve">Alessandro Bastoni  </t>
   </si>
@@ -2418,6 +2422,78 @@
   </si>
   <si>
     <t>Manchester_United</t>
+  </si>
+  <si>
+    <t>Fase</t>
+  </si>
+  <si>
+    <t>Equipo 1</t>
+  </si>
+  <si>
+    <t>Goles 1</t>
+  </si>
+  <si>
+    <t>Equipo 2</t>
+  </si>
+  <si>
+    <t>Goles 2</t>
+  </si>
+  <si>
+    <t>Estado</t>
+  </si>
+  <si>
+    <t>Cuartos 1</t>
+  </si>
+  <si>
+    <t>Cuartos 2</t>
+  </si>
+  <si>
+    <t>Cuartos 3</t>
+  </si>
+  <si>
+    <t>Cuartos 4</t>
+  </si>
+  <si>
+    <t>Semifinal 1</t>
+  </si>
+  <si>
+    <t>Semifinal 2</t>
+  </si>
+  <si>
+    <t>Final</t>
+  </si>
+  <si>
+    <t>2 (2)</t>
+  </si>
+  <si>
+    <t>Finalizado</t>
+  </si>
+  <si>
+    <t>Terengganu</t>
+  </si>
+  <si>
+    <t>2 (4)</t>
+  </si>
+  <si>
+    <t>Bayern_Munich</t>
+  </si>
+  <si>
+    <t>Watkins</t>
+  </si>
+  <si>
+    <t>del Piero</t>
+  </si>
+  <si>
+    <t>Rafael Leão</t>
+  </si>
+  <si>
+    <t>modric</t>
+  </si>
+  <si>
+    <t>diaby</t>
+  </si>
+  <si>
+    <t>Richarlison</t>
   </si>
 </sst>
 </file>
@@ -2500,7 +2576,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2524,9 +2600,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2889,27 +2962,27 @@
         <v>771</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>711</v>
+        <v>171</v>
       </c>
       <c r="C2" s="3">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D2" s="3">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
-        <v>770</v>
+        <v>764</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>679</v>
+        <v>35</v>
       </c>
       <c r="C3" s="3">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="D3" s="3">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s">
         <v>179</v>
@@ -2917,16 +2990,16 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
-        <v>766</v>
+        <v>771</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>63</v>
+        <v>711</v>
       </c>
       <c r="C4" s="3">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D4" s="3">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -2934,52 +3007,52 @@
         <v>137</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>668</v>
+        <v>147</v>
       </c>
       <c r="C5" s="3">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D5" s="3">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>766</v>
+        <v>764</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>62</v>
+        <v>41</v>
       </c>
       <c r="C6" s="3">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="D6" s="3">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>771</v>
+        <v>763</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>700</v>
+        <v>18</v>
       </c>
       <c r="C7" s="3">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D7" s="3">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>137</v>
+        <v>767</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>147</v>
+        <v>92</v>
       </c>
       <c r="C8" s="3">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D8" s="3">
         <v>7</v>
@@ -2990,151 +3063,149 @@
         <v>770</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>677</v>
+        <v>152</v>
       </c>
       <c r="C9" s="3">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D9" s="3">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>636</v>
+        <v>146</v>
       </c>
       <c r="C10" s="3">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D10" s="3">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>767</v>
+        <v>137</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="C11" s="3">
-        <v>9</v>
-      </c>
+        <v>141</v>
+      </c>
+      <c r="C11" s="3"/>
       <c r="D11" s="3">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
-        <v>765</v>
+        <v>766</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="C12" s="3">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D12" s="3">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
-        <v>764</v>
+        <v>771</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>41</v>
+        <v>700</v>
       </c>
       <c r="C13" s="3">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D13" s="3">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
-        <v>770</v>
+        <v>766</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>152</v>
+        <v>60</v>
       </c>
       <c r="C14" s="3">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D14" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
-        <v>767</v>
+        <v>126</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="C15" s="3">
-        <v>7</v>
-      </c>
-      <c r="D15" s="3"/>
+        <v>130</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3">
+        <v>5</v>
+      </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
-        <v>763</v>
+        <v>766</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="C16" s="3">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="D16" s="3">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
-        <v>137</v>
+        <v>771</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>146</v>
+        <v>169</v>
       </c>
       <c r="C17" s="3">
         <v>6</v>
       </c>
       <c r="D17" s="3">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
-        <v>773</v>
+        <v>763</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>159</v>
+        <v>16</v>
       </c>
       <c r="C18" s="3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D18" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
-        <v>768</v>
+        <v>773</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>101</v>
+        <v>158</v>
       </c>
       <c r="C19" s="3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D19" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -3142,10 +3213,10 @@
         <v>771</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C20" s="3">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D20" s="3">
         <v>4</v>
@@ -3153,69 +3224,67 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C21" s="3">
-        <v>6</v>
-      </c>
+        <v>151</v>
+      </c>
+      <c r="C21" s="3"/>
       <c r="D21" s="3">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
-        <v>764</v>
+        <v>137</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>36</v>
+        <v>668</v>
       </c>
       <c r="C22" s="3">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D22" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
-        <v>771</v>
+        <v>767</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>171</v>
+        <v>96</v>
       </c>
       <c r="C23" s="3">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D23" s="3">
-        <v>11</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
-        <v>764</v>
+        <v>763</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="C24" s="3">
         <v>5</v>
       </c>
       <c r="D24" s="3">
-        <v>10</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>27</v>
+        <v>94</v>
       </c>
       <c r="C25" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D25" s="3">
         <v>3</v>
@@ -3223,201 +3292,193 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
-        <v>767</v>
+        <v>763</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>82</v>
+        <v>15</v>
       </c>
       <c r="C26" s="3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D26" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>102</v>
+        <v>93</v>
       </c>
       <c r="C27" s="3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D27" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>46</v>
+        <v>109</v>
       </c>
       <c r="C28" s="3">
-        <v>5</v>
-      </c>
-      <c r="D28" s="3"/>
+        <v>2</v>
+      </c>
+      <c r="D28" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
-        <v>764</v>
+        <v>126</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>33</v>
+        <v>133</v>
       </c>
       <c r="C29" s="3">
-        <v>5</v>
-      </c>
-      <c r="D29" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="D29" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
-        <v>767</v>
+        <v>769</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>85</v>
+        <v>112</v>
       </c>
       <c r="C30" s="3">
-        <v>5</v>
-      </c>
-      <c r="D30" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="D30" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
-        <v>126</v>
+        <v>762</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>132</v>
+        <v>3</v>
       </c>
       <c r="C31" s="3">
-        <v>5</v>
-      </c>
-      <c r="D31" s="3"/>
+        <v>1</v>
+      </c>
+      <c r="D31" s="3">
+        <v>3</v>
+      </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>763</v>
+        <v>767</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C32" s="3">
-        <v>4</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="C32" s="3"/>
       <c r="D32" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C33" s="3">
-        <v>4</v>
-      </c>
+        <v>149</v>
+      </c>
+      <c r="C33" s="3"/>
       <c r="D33" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C34" s="3">
-        <v>4</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="C34" s="3"/>
       <c r="D34" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
-        <v>769</v>
+        <v>762</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="C35" s="3">
-        <v>4</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="C35" s="3"/>
       <c r="D35" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="C36" s="3">
-        <v>4</v>
-      </c>
+        <v>138</v>
+      </c>
+      <c r="C36" s="3"/>
       <c r="D36" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
-        <v>763</v>
+        <v>137</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="C37" s="3">
-        <v>4</v>
-      </c>
+        <v>140</v>
+      </c>
+      <c r="C37" s="3"/>
       <c r="D37" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="C38" s="3">
-        <v>3</v>
-      </c>
+        <v>38</v>
+      </c>
+      <c r="C38" s="3"/>
       <c r="D38" s="3">
         <v>3</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="C39" s="3">
+        <v>617</v>
+      </c>
+      <c r="C39" s="6"/>
+      <c r="D39" s="3">
         <v>3</v>
-      </c>
-      <c r="D39" s="3">
-        <v>2</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
-        <v>764</v>
+        <v>126</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>42</v>
+        <v>636</v>
       </c>
       <c r="C40" s="3">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D40" s="3">
         <v>2</v>
@@ -3425,13 +3486,13 @@
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>769</v>
+        <v>773</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>114</v>
+        <v>159</v>
       </c>
       <c r="C41" s="3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D41" s="3">
         <v>2</v>
@@ -3439,13 +3500,13 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
-        <v>118</v>
+        <v>768</v>
       </c>
       <c r="B42" s="3" t="s">
-        <v>120</v>
+        <v>101</v>
       </c>
       <c r="C42" s="3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D42" s="3">
         <v>2</v>
@@ -3453,122 +3514,128 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
-        <v>118</v>
+        <v>767</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>122</v>
+        <v>82</v>
       </c>
       <c r="C43" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D43" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
-        <v>118</v>
+        <v>768</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>624</v>
-      </c>
-      <c r="C44" s="6">
-        <v>3</v>
-      </c>
-      <c r="D44" s="6">
-        <v>1</v>
+        <v>102</v>
+      </c>
+      <c r="C44" s="3">
+        <v>5</v>
+      </c>
+      <c r="D44" s="3">
+        <v>2</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
-        <v>773</v>
+        <v>764</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>157</v>
+        <v>39</v>
       </c>
       <c r="C45" s="3">
-        <v>3</v>
-      </c>
-      <c r="D45" s="3"/>
+        <v>4</v>
+      </c>
+      <c r="D45" s="3">
+        <v>2</v>
+      </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
         <v>762</v>
       </c>
       <c r="B46" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C46" s="3">
-        <v>3</v>
-      </c>
-      <c r="D46" s="3"/>
+        <v>4</v>
+      </c>
+      <c r="D46" s="3">
+        <v>2</v>
+      </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
-        <v>118</v>
+        <v>769</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="C47" s="3">
-        <v>3</v>
-      </c>
-      <c r="D47" s="3"/>
+        <v>4</v>
+      </c>
+      <c r="D47" s="3">
+        <v>2</v>
+      </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
-        <v>773</v>
+        <v>126</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>158</v>
+        <v>134</v>
       </c>
       <c r="C48" s="3">
+        <v>3</v>
+      </c>
+      <c r="D48" s="3">
         <v>2</v>
-      </c>
-      <c r="D48" s="3">
-        <v>4</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
-        <v>771</v>
+        <v>764</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>168</v>
+        <v>42</v>
       </c>
       <c r="C49" s="3">
+        <v>3</v>
+      </c>
+      <c r="D49" s="3">
         <v>2</v>
-      </c>
-      <c r="D49" s="3">
-        <v>4</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>15</v>
+        <v>114</v>
       </c>
       <c r="C50" s="3">
+        <v>3</v>
+      </c>
+      <c r="D50" s="3">
         <v>2</v>
-      </c>
-      <c r="D50" s="3">
-        <v>3</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
-        <v>767</v>
+        <v>118</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>93</v>
+        <v>120</v>
       </c>
       <c r="C51" s="3">
+        <v>3</v>
+      </c>
+      <c r="D51" s="3">
         <v>2</v>
-      </c>
-      <c r="D51" s="3">
-        <v>3</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
@@ -3590,38 +3657,38 @@
         <v>769</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C53" s="3">
         <v>2</v>
       </c>
       <c r="D53" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
-        <v>126</v>
+        <v>770</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>131</v>
+        <v>153</v>
       </c>
       <c r="C54" s="3">
         <v>2</v>
       </c>
       <c r="D54" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
-        <v>769</v>
+        <v>766</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>111</v>
+        <v>61</v>
       </c>
       <c r="C55" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D55" s="3">
         <v>2</v>
@@ -3632,343 +3699,347 @@
         <v>773</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C56" s="3">
+        <v>1</v>
+      </c>
+      <c r="D56" s="3">
         <v>2</v>
-      </c>
-      <c r="D56" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
-        <v>767</v>
+        <v>773</v>
       </c>
       <c r="B57" s="3" t="s">
-        <v>95</v>
+        <v>165</v>
       </c>
       <c r="C57" s="3">
+        <v>1</v>
+      </c>
+      <c r="D57" s="3">
         <v>2</v>
-      </c>
-      <c r="D57" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>8</v>
+        <v>47</v>
       </c>
       <c r="C58" s="3">
+        <v>1</v>
+      </c>
+      <c r="D58" s="3">
         <v>2</v>
-      </c>
-      <c r="D58" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
-        <v>766</v>
+        <v>773</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>70</v>
+        <v>161</v>
       </c>
       <c r="C59" s="3">
+        <v>1</v>
+      </c>
+      <c r="D59" s="3">
         <v>2</v>
-      </c>
-      <c r="D59" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>4</v>
+        <v>59</v>
       </c>
       <c r="C60" s="3">
+        <v>1</v>
+      </c>
+      <c r="D60" s="3">
         <v>2</v>
-      </c>
-      <c r="D60" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
-        <v>137</v>
+        <v>768</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>144</v>
+        <v>99</v>
       </c>
       <c r="C61" s="3">
+        <v>1</v>
+      </c>
+      <c r="D61" s="3">
         <v>2</v>
-      </c>
-      <c r="D61" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
-        <v>769</v>
+        <v>767</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>115</v>
+        <v>83</v>
       </c>
       <c r="C62" s="3">
+        <v>1</v>
+      </c>
+      <c r="D62" s="3">
         <v>2</v>
-      </c>
-      <c r="D62" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
-        <v>770</v>
+        <v>118</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="C63" s="3">
-        <v>2</v>
-      </c>
-      <c r="D63" s="3">
+        <v>623</v>
+      </c>
+      <c r="C63" s="6">
+        <v>1</v>
+      </c>
+      <c r="D63" s="6">
         <v>2</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
-        <v>771</v>
+        <v>765</v>
       </c>
       <c r="B64" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="C64" s="3">
+        <v>45</v>
+      </c>
+      <c r="C64" s="3"/>
+      <c r="D64" s="3">
         <v>2</v>
-      </c>
-      <c r="D64" s="3">
-        <v>1</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
-        <v>770</v>
+        <v>764</v>
       </c>
       <c r="B65" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="C65" s="3">
+        <v>37</v>
+      </c>
+      <c r="C65" s="3"/>
+      <c r="D65" s="3">
         <v>2</v>
       </c>
-      <c r="D65" s="3"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
-        <v>126</v>
+        <v>767</v>
       </c>
       <c r="B66" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="C66" s="3">
+        <v>81</v>
+      </c>
+      <c r="C66" s="3"/>
+      <c r="D66" s="3">
         <v>2</v>
       </c>
-      <c r="D66" s="3"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
         <v>770</v>
       </c>
       <c r="B67" s="3" t="s">
-        <v>689</v>
-      </c>
-      <c r="C67" s="3">
+        <v>687</v>
+      </c>
+      <c r="C67" s="3"/>
+      <c r="D67" s="3">
         <v>2</v>
       </c>
-      <c r="D67" s="3"/>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
-        <v>773</v>
+        <v>771</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C68" s="3">
+        <v>167</v>
+      </c>
+      <c r="C68" s="3"/>
+      <c r="D68" s="3">
         <v>2</v>
       </c>
-      <c r="D68" s="3"/>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
-        <v>769</v>
+        <v>762</v>
       </c>
       <c r="B69" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C69" s="3">
+        <v>516</v>
+      </c>
+      <c r="C69" s="6"/>
+      <c r="D69" s="3">
         <v>2</v>
       </c>
-      <c r="D69" s="3"/>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
-        <v>769</v>
+        <v>118</v>
       </c>
       <c r="B70" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="C70" s="3">
+        <v>121</v>
+      </c>
+      <c r="C70" s="3"/>
+      <c r="D70" s="3">
         <v>2</v>
       </c>
-      <c r="D70" s="3"/>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
-        <v>137</v>
+        <v>770</v>
       </c>
       <c r="B71" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="C71" s="3">
+        <v>150</v>
+      </c>
+      <c r="C71" s="3"/>
+      <c r="D71" s="3">
         <v>2</v>
       </c>
-      <c r="D71" s="3"/>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
-        <v>766</v>
+        <v>770</v>
       </c>
       <c r="B72" s="3" t="s">
-        <v>75</v>
+        <v>679</v>
       </c>
       <c r="C72" s="3">
-        <v>2</v>
-      </c>
-      <c r="D72" s="3"/>
+        <v>16</v>
+      </c>
+      <c r="D72" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
-        <v>126</v>
+        <v>770</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>135</v>
+        <v>677</v>
       </c>
       <c r="C73" s="3">
-        <v>2</v>
-      </c>
-      <c r="D73" s="3"/>
+        <v>11</v>
+      </c>
+      <c r="D73" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
-        <v>118</v>
+        <v>765</v>
       </c>
       <c r="B74" s="3" t="s">
-        <v>609</v>
-      </c>
-      <c r="C74" s="6">
-        <v>2</v>
-      </c>
-      <c r="D74" s="6">
+        <v>48</v>
+      </c>
+      <c r="C74" s="3">
+        <v>9</v>
+      </c>
+      <c r="D74" s="3">
         <v>1</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
-        <v>126</v>
+        <v>764</v>
       </c>
       <c r="B75" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="C75" s="11">
-        <v>2</v>
-      </c>
-      <c r="D75" s="6"/>
+        <v>34</v>
+      </c>
+      <c r="C75" s="3">
+        <v>6</v>
+      </c>
+      <c r="D75" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
-        <v>767</v>
+        <v>764</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>92</v>
+        <v>36</v>
       </c>
       <c r="C76" s="3">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D76" s="3">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77" s="3" t="s">
-        <v>766</v>
+        <v>118</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>60</v>
+        <v>125</v>
       </c>
       <c r="C77" s="3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D77" s="3">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78" s="3" t="s">
-        <v>126</v>
+        <v>763</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>133</v>
+        <v>19</v>
       </c>
       <c r="C78" s="3">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D78" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79" s="3" t="s">
-        <v>769</v>
+        <v>118</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>112</v>
+        <v>122</v>
       </c>
       <c r="C79" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D79" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80" s="3" t="s">
-        <v>762</v>
+        <v>118</v>
       </c>
       <c r="B80" s="3" t="s">
+        <v>624</v>
+      </c>
+      <c r="C80" s="6">
         <v>3</v>
       </c>
-      <c r="C80" s="3">
-        <v>1</v>
-      </c>
-      <c r="D80" s="3">
-        <v>3</v>
+      <c r="D80" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
-        <v>766</v>
+        <v>126</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>61</v>
+        <v>131</v>
       </c>
       <c r="C81" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D81" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E81" t="s">
         <v>179</v>
@@ -3979,94 +4050,94 @@
         <v>773</v>
       </c>
       <c r="B82" s="3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C82" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D82" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="3" t="s">
-        <v>773</v>
+        <v>767</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>165</v>
+        <v>95</v>
       </c>
       <c r="C83" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D83" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="3" t="s">
-        <v>765</v>
+        <v>762</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="C84" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D84" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="3" t="s">
-        <v>773</v>
+        <v>766</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>161</v>
+        <v>70</v>
       </c>
       <c r="C85" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D85" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="3" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>59</v>
+        <v>4</v>
       </c>
       <c r="C86" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D86" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="3" t="s">
-        <v>768</v>
+        <v>137</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>99</v>
+        <v>144</v>
       </c>
       <c r="C87" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D87" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" s="3" t="s">
-        <v>763</v>
+        <v>769</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>25</v>
+        <v>115</v>
       </c>
       <c r="C88" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D88" s="3">
         <v>1</v>
@@ -4074,13 +4145,13 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" s="3" t="s">
-        <v>126</v>
+        <v>771</v>
       </c>
       <c r="B89" s="3" t="s">
-        <v>128</v>
+        <v>170</v>
       </c>
       <c r="C89" s="3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D89" s="3">
         <v>1</v>
@@ -4088,24 +4159,24 @@
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" s="3" t="s">
-        <v>767</v>
+        <v>118</v>
       </c>
       <c r="B90" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C90" s="3">
-        <v>1</v>
-      </c>
-      <c r="D90" s="3">
+        <v>609</v>
+      </c>
+      <c r="C90" s="6">
+        <v>2</v>
+      </c>
+      <c r="D90" s="6">
         <v>1</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" s="3" t="s">
-        <v>118</v>
+        <v>763</v>
       </c>
       <c r="B91" s="3" t="s">
-        <v>124</v>
+        <v>25</v>
       </c>
       <c r="C91" s="3">
         <v>1</v>
@@ -4116,10 +4187,10 @@
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" s="3" t="s">
-        <v>768</v>
+        <v>126</v>
       </c>
       <c r="B92" s="3" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="C92" s="3">
         <v>1</v>
@@ -4130,10 +4201,10 @@
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" s="3" t="s">
-        <v>768</v>
+        <v>767</v>
       </c>
       <c r="B93" s="3" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="C93" s="3">
         <v>1</v>
@@ -4144,10 +4215,10 @@
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" s="3" t="s">
-        <v>765</v>
+        <v>118</v>
       </c>
       <c r="B94" s="3" t="s">
-        <v>43</v>
+        <v>124</v>
       </c>
       <c r="C94" s="3">
         <v>1</v>
@@ -4158,10 +4229,10 @@
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" s="3" t="s">
-        <v>765</v>
+        <v>768</v>
       </c>
       <c r="B95" s="3" t="s">
-        <v>44</v>
+        <v>103</v>
       </c>
       <c r="C95" s="3">
         <v>1</v>
@@ -4172,26 +4243,26 @@
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="3" t="s">
-        <v>767</v>
+        <v>768</v>
       </c>
       <c r="B96" s="3" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="C96" s="3">
         <v>1</v>
       </c>
       <c r="D96" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97" s="3" t="s">
-        <v>771</v>
+        <v>765</v>
       </c>
       <c r="B97" s="3" t="s">
-        <v>710</v>
-      </c>
-      <c r="C97" s="6">
+        <v>43</v>
+      </c>
+      <c r="C97" s="3">
         <v>1</v>
       </c>
       <c r="D97" s="3">
@@ -4200,10 +4271,10 @@
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
-        <v>137</v>
+        <v>765</v>
       </c>
       <c r="B98" s="3" t="s">
-        <v>139</v>
+        <v>44</v>
       </c>
       <c r="C98" s="3">
         <v>1</v>
@@ -4214,12 +4285,12 @@
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99" s="3" t="s">
-        <v>768</v>
+        <v>771</v>
       </c>
       <c r="B99" s="3" t="s">
-        <v>575</v>
-      </c>
-      <c r="C99" s="3">
+        <v>710</v>
+      </c>
+      <c r="C99" s="6">
         <v>1</v>
       </c>
       <c r="D99" s="3">
@@ -4231,7 +4302,7 @@
         <v>137</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="C100" s="3">
         <v>1</v>
@@ -4242,10 +4313,10 @@
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" s="3" t="s">
-        <v>764</v>
+        <v>768</v>
       </c>
       <c r="B101" s="3" t="s">
-        <v>38</v>
+        <v>575</v>
       </c>
       <c r="C101" s="3">
         <v>1</v>
@@ -4256,10 +4327,10 @@
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" s="3" t="s">
-        <v>771</v>
+        <v>137</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>172</v>
+        <v>145</v>
       </c>
       <c r="C102" s="3">
         <v>1</v>
@@ -4270,256 +4341,258 @@
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" s="3" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="B103" s="3" t="s">
-        <v>2</v>
+        <v>38</v>
       </c>
       <c r="C103" s="3">
         <v>1</v>
       </c>
-      <c r="D103" s="3"/>
+      <c r="D103" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" s="3" t="s">
-        <v>764</v>
+        <v>771</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>32</v>
+        <v>172</v>
       </c>
       <c r="C104" s="3">
         <v>1</v>
       </c>
-      <c r="D104" s="3"/>
+      <c r="D104" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" s="3" t="s">
-        <v>762</v>
+        <v>766</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C105" s="3">
-        <v>1</v>
-      </c>
-      <c r="D105" s="3"/>
+        <v>56</v>
+      </c>
+      <c r="C105" s="3"/>
+      <c r="D105" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" s="3" t="s">
-        <v>769</v>
+        <v>118</v>
       </c>
       <c r="B106" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="C106" s="3">
-        <v>1</v>
-      </c>
-      <c r="D106" s="3"/>
+        <v>123</v>
+      </c>
+      <c r="C106" s="3"/>
+      <c r="D106" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" s="3" t="s">
-        <v>768</v>
+        <v>769</v>
       </c>
       <c r="B107" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C107" s="3">
-        <v>1</v>
-      </c>
-      <c r="D107" s="3"/>
+        <v>107</v>
+      </c>
+      <c r="C107" s="3"/>
+      <c r="D107" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" s="3" t="s">
-        <v>769</v>
+        <v>126</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C108" s="3">
-        <v>1</v>
-      </c>
-      <c r="D108" s="3"/>
+        <v>129</v>
+      </c>
+      <c r="C108" s="3"/>
+      <c r="D108" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" s="3" t="s">
-        <v>767</v>
+        <v>765</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C109" s="3">
-        <v>1</v>
-      </c>
-      <c r="D109" s="3"/>
+        <v>51</v>
+      </c>
+      <c r="C109" s="3"/>
+      <c r="D109" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" s="3" t="s">
-        <v>762</v>
+        <v>764</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C110" s="3">
-        <v>1</v>
-      </c>
-      <c r="D110" s="3"/>
+        <v>31</v>
+      </c>
+      <c r="C110" s="3"/>
+      <c r="D110" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" s="3" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C111" s="3">
-        <v>1</v>
-      </c>
-      <c r="D111" s="3"/>
+        <v>80</v>
+      </c>
+      <c r="C111" s="3"/>
+      <c r="D111" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" s="3" t="s">
-        <v>137</v>
+        <v>769</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C112" s="3">
-        <v>1</v>
-      </c>
-      <c r="D112" s="3"/>
+        <v>106</v>
+      </c>
+      <c r="C112" s="3"/>
+      <c r="D112" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" s="3" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="C113" s="3">
-        <v>1</v>
-      </c>
-      <c r="D113" s="3"/>
+        <v>164</v>
+      </c>
+      <c r="C113" s="3"/>
+      <c r="D113" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" s="3" t="s">
-        <v>771</v>
+        <v>766</v>
       </c>
       <c r="B114" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="C114" s="3">
-        <v>1</v>
-      </c>
-      <c r="D114" s="3"/>
+        <v>66</v>
+      </c>
+      <c r="C114" s="3"/>
+      <c r="D114" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" s="3" t="s">
-        <v>118</v>
+        <v>768</v>
       </c>
       <c r="B115" s="3" t="s">
-        <v>623</v>
-      </c>
-      <c r="C115" s="6">
-        <v>1</v>
-      </c>
-      <c r="D115" s="6">
-        <v>2</v>
+        <v>104</v>
+      </c>
+      <c r="C115" s="3"/>
+      <c r="D115" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A116" s="3" t="s">
-        <v>762</v>
+        <v>765</v>
       </c>
       <c r="B116" s="3" t="s">
-        <v>519</v>
-      </c>
-      <c r="C116" s="3">
-        <v>1</v>
-      </c>
-      <c r="D116" s="6"/>
+        <v>49</v>
+      </c>
+      <c r="C116" s="3"/>
+      <c r="D116" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" s="3" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
       <c r="B117" s="3" t="s">
-        <v>576</v>
-      </c>
-      <c r="C117" s="3">
-        <v>1</v>
-      </c>
-      <c r="D117" s="6"/>
+        <v>40</v>
+      </c>
+      <c r="C117" s="3"/>
+      <c r="D117" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A118" s="3" t="s">
-        <v>764</v>
+        <v>770</v>
       </c>
       <c r="B118" s="3" t="s">
-        <v>549</v>
-      </c>
-      <c r="C118" s="6">
-        <v>1</v>
-      </c>
-      <c r="D118" s="3"/>
+        <v>154</v>
+      </c>
+      <c r="C118" s="3"/>
+      <c r="D118" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A119" s="3" t="s">
-        <v>770</v>
+        <v>765</v>
       </c>
       <c r="B119" s="3" t="s">
-        <v>686</v>
-      </c>
-      <c r="C119" s="6">
-        <v>1</v>
-      </c>
-      <c r="D119" s="6"/>
+        <v>555</v>
+      </c>
+      <c r="C119" s="3"/>
+      <c r="D119" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A120" s="3" t="s">
-        <v>118</v>
+        <v>770</v>
       </c>
       <c r="B120" s="3" t="s">
-        <v>625</v>
-      </c>
-      <c r="C120" s="6">
-        <v>1</v>
-      </c>
-      <c r="D120" s="6"/>
+        <v>671</v>
+      </c>
+      <c r="C120" s="3"/>
+      <c r="D120" s="3">
+        <v>1</v>
+      </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A121" s="3" t="s">
-        <v>137</v>
+        <v>766</v>
       </c>
       <c r="B121" s="3" t="s">
-        <v>141</v>
+        <v>68</v>
       </c>
       <c r="C121" s="3"/>
       <c r="D121" s="3">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A122" s="3" t="s">
-        <v>126</v>
+        <v>766</v>
       </c>
       <c r="B122" s="3" t="s">
-        <v>130</v>
+        <v>71</v>
       </c>
       <c r="C122" s="3"/>
       <c r="D122" s="3">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A123" s="3" t="s">
-        <v>770</v>
+        <v>137</v>
       </c>
       <c r="B123" s="3" t="s">
-        <v>151</v>
+        <v>657</v>
       </c>
       <c r="C123" s="3"/>
       <c r="D123" s="3">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.3">
@@ -4527,476 +4600,492 @@
         <v>767</v>
       </c>
       <c r="B124" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="C124" s="3"/>
+        <v>84</v>
+      </c>
+      <c r="C124" s="6"/>
       <c r="D124" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A125" s="3" t="s">
-        <v>770</v>
+        <v>763</v>
       </c>
       <c r="B125" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="C125" s="3"/>
+        <v>13</v>
+      </c>
+      <c r="C125" s="6"/>
       <c r="D125" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A126" s="3" t="s">
-        <v>765</v>
+        <v>118</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="C126" s="3"/>
-      <c r="D126" s="3">
-        <v>3</v>
+        <v>622</v>
+      </c>
+      <c r="C126" s="6"/>
+      <c r="D126" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A127" s="3" t="s">
-        <v>762</v>
+        <v>768</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C127" s="3"/>
+        <v>577</v>
+      </c>
+      <c r="C127" s="6"/>
       <c r="D127" s="3">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A128" s="3" t="s">
-        <v>137</v>
+        <v>771</v>
       </c>
       <c r="B128" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="C128" s="3"/>
-      <c r="D128" s="3">
-        <v>3</v>
+        <v>709</v>
+      </c>
+      <c r="C128" s="6"/>
+      <c r="D128" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A129" s="3" t="s">
-        <v>137</v>
+        <v>118</v>
       </c>
       <c r="B129" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C129" s="3"/>
-      <c r="D129" s="3">
-        <v>3</v>
+        <v>618</v>
+      </c>
+      <c r="C129" s="6"/>
+      <c r="D129" s="6">
+        <v>1</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A130" s="3" t="s">
-        <v>765</v>
+        <v>767</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C130" s="3"/>
-      <c r="D130" s="3">
-        <v>2</v>
-      </c>
+        <v>97</v>
+      </c>
+      <c r="C130" s="3">
+        <v>7</v>
+      </c>
+      <c r="D130" s="3"/>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A131" s="3" t="s">
-        <v>764</v>
+        <v>765</v>
       </c>
       <c r="B131" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="C131" s="3"/>
-      <c r="D131" s="3">
-        <v>2</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C131" s="3">
+        <v>5</v>
+      </c>
+      <c r="D131" s="3"/>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A132" s="3" t="s">
         <v>764</v>
       </c>
       <c r="B132" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="C132" s="3"/>
-      <c r="D132" s="3">
-        <v>3</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="C132" s="3">
+        <v>5</v>
+      </c>
+      <c r="D132" s="3"/>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" s="3" t="s">
         <v>767</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="C133" s="3"/>
-      <c r="D133" s="3">
-        <v>2</v>
-      </c>
+        <v>85</v>
+      </c>
+      <c r="C133" s="3">
+        <v>5</v>
+      </c>
+      <c r="D133" s="3"/>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A134" s="3" t="s">
-        <v>770</v>
+        <v>126</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>687</v>
-      </c>
-      <c r="C134" s="3"/>
-      <c r="D134" s="3">
-        <v>2</v>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="C134" s="3">
+        <v>5</v>
+      </c>
+      <c r="D134" s="3"/>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A135" s="3" t="s">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="C135" s="3"/>
-      <c r="D135" s="3">
-        <v>2</v>
-      </c>
+        <v>157</v>
+      </c>
+      <c r="C135" s="3">
+        <v>3</v>
+      </c>
+      <c r="D135" s="3"/>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A136" s="3" t="s">
         <v>762</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>516</v>
-      </c>
-      <c r="C136" s="6"/>
-      <c r="D136" s="3">
-        <v>2</v>
-      </c>
+        <v>7</v>
+      </c>
+      <c r="C136" s="3">
+        <v>3</v>
+      </c>
+      <c r="D136" s="3"/>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A137" s="3" t="s">
-        <v>766</v>
+        <v>118</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C137" s="3"/>
-      <c r="D137" s="3">
-        <v>1</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="C137" s="3">
+        <v>3</v>
+      </c>
+      <c r="D137" s="3"/>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A138" s="3" t="s">
-        <v>118</v>
+        <v>770</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="C138" s="3"/>
-      <c r="D138" s="3">
-        <v>1</v>
-      </c>
+        <v>155</v>
+      </c>
+      <c r="C138" s="3">
+        <v>2</v>
+      </c>
+      <c r="D138" s="3"/>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A139" s="3" t="s">
-        <v>769</v>
+        <v>126</v>
       </c>
       <c r="B139" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="C139" s="9"/>
-      <c r="D139" s="9">
-        <v>1</v>
-      </c>
+        <v>127</v>
+      </c>
+      <c r="C139" s="9">
+        <v>2</v>
+      </c>
+      <c r="D139" s="9"/>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A140" s="3" t="s">
-        <v>118</v>
+        <v>770</v>
       </c>
       <c r="B140" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="C140" s="9"/>
-      <c r="D140" s="9">
+        <v>689</v>
+      </c>
+      <c r="C140" s="9">
         <v>2</v>
       </c>
+      <c r="D140" s="9"/>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A141" s="3" t="s">
-        <v>126</v>
+        <v>773</v>
       </c>
       <c r="B141" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="C141" s="9"/>
-      <c r="D141" s="9">
-        <v>1</v>
-      </c>
+        <v>166</v>
+      </c>
+      <c r="C141" s="9">
+        <v>2</v>
+      </c>
+      <c r="D141" s="9"/>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A142" s="3" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="B142" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C142" s="9"/>
-      <c r="D142" s="9">
-        <v>1</v>
-      </c>
+        <v>114</v>
+      </c>
+      <c r="C142" s="9">
+        <v>2</v>
+      </c>
+      <c r="D142" s="9"/>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A143" s="3" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B143" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="C143" s="9"/>
-      <c r="D143" s="9">
-        <v>1</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="C143" s="9">
+        <v>2</v>
+      </c>
+      <c r="D143" s="9"/>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A144" s="3" t="s">
-        <v>770</v>
+        <v>137</v>
       </c>
       <c r="B144" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="C144" s="9"/>
-      <c r="D144" s="9">
+        <v>142</v>
+      </c>
+      <c r="C144" s="9">
         <v>2</v>
       </c>
+      <c r="D144" s="9"/>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A145" s="3" t="s">
-        <v>767</v>
+        <v>766</v>
       </c>
       <c r="B145" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C145" s="9"/>
-      <c r="D145" s="9">
-        <v>1</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="C145" s="9">
+        <v>2</v>
+      </c>
+      <c r="D145" s="9"/>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A146" s="3" t="s">
-        <v>769</v>
+        <v>126</v>
       </c>
       <c r="B146" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="C146" s="9"/>
-      <c r="D146" s="9">
-        <v>1</v>
-      </c>
+        <v>135</v>
+      </c>
+      <c r="C146" s="9">
+        <v>2</v>
+      </c>
+      <c r="D146" s="9"/>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A147" s="3" t="s">
-        <v>773</v>
+        <v>126</v>
       </c>
       <c r="B147" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="C147" s="9"/>
-      <c r="D147" s="9">
-        <v>1</v>
-      </c>
+        <v>136</v>
+      </c>
+      <c r="C147" s="9">
+        <v>2</v>
+      </c>
+      <c r="D147" s="10"/>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A148" s="3" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="B148" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C148" s="9"/>
-      <c r="D148" s="9">
-        <v>1</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="C148" s="9">
+        <v>1</v>
+      </c>
+      <c r="D148" s="9"/>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A149" s="3" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
       <c r="B149" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="C149" s="9"/>
-      <c r="D149" s="9">
-        <v>1</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="C149" s="9">
+        <v>1</v>
+      </c>
+      <c r="D149" s="9"/>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A150" s="3" t="s">
-        <v>765</v>
+        <v>762</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C150" s="9"/>
-      <c r="D150" s="9">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="C150" s="9">
+        <v>1</v>
+      </c>
+      <c r="D150" s="9"/>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A151" s="3" t="s">
-        <v>764</v>
+        <v>769</v>
       </c>
       <c r="B151" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C151" s="9"/>
-      <c r="D151" s="9">
-        <v>1</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="C151" s="9">
+        <v>1</v>
+      </c>
+      <c r="D151" s="9"/>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A152" s="3" t="s">
-        <v>770</v>
+        <v>768</v>
       </c>
       <c r="B152" s="3" t="s">
-        <v>154</v>
-      </c>
-      <c r="C152" s="9"/>
-      <c r="D152" s="9">
-        <v>1</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="C152" s="9">
+        <v>1</v>
+      </c>
+      <c r="D152" s="9"/>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A153" s="3" t="s">
-        <v>765</v>
+        <v>769</v>
       </c>
       <c r="B153" s="3" t="s">
-        <v>555</v>
-      </c>
-      <c r="C153" s="9"/>
-      <c r="D153" s="9">
-        <v>1</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="C153" s="9">
+        <v>1</v>
+      </c>
+      <c r="D153" s="9"/>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A154" s="3" t="s">
-        <v>770</v>
+        <v>767</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>671</v>
-      </c>
-      <c r="C154" s="9"/>
-      <c r="D154" s="9">
-        <v>1</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="C154" s="9">
+        <v>1</v>
+      </c>
+      <c r="D154" s="9"/>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A155" s="3" t="s">
-        <v>766</v>
+        <v>762</v>
       </c>
       <c r="B155" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C155" s="9"/>
-      <c r="D155" s="9">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="C155" s="9">
+        <v>1</v>
+      </c>
+      <c r="D155" s="9"/>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A156" s="3" t="s">
-        <v>766</v>
+        <v>765</v>
       </c>
       <c r="B156" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="C156" s="9"/>
-      <c r="D156" s="9">
-        <v>1</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="C156" s="9">
+        <v>1</v>
+      </c>
+      <c r="D156" s="9"/>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A157" s="3" t="s">
         <v>137</v>
       </c>
       <c r="B157" s="3" t="s">
-        <v>657</v>
-      </c>
-      <c r="C157" s="9"/>
-      <c r="D157" s="9">
-        <v>1</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="C157" s="9">
+        <v>1</v>
+      </c>
+      <c r="D157" s="9"/>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A158" s="3" t="s">
-        <v>767</v>
+        <v>771</v>
       </c>
       <c r="B158" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="C158" s="10"/>
-      <c r="D158" s="9">
-        <v>1</v>
-      </c>
+        <v>173</v>
+      </c>
+      <c r="C158" s="9">
+        <v>1</v>
+      </c>
+      <c r="D158" s="9"/>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A159" s="3" t="s">
-        <v>118</v>
+        <v>771</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>617</v>
-      </c>
-      <c r="C159" s="10"/>
-      <c r="D159" s="9">
-        <v>3</v>
-      </c>
+        <v>174</v>
+      </c>
+      <c r="C159" s="9">
+        <v>1</v>
+      </c>
+      <c r="D159" s="9"/>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A160" s="3" t="s">
-        <v>763</v>
+        <v>762</v>
       </c>
       <c r="B160" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C160" s="10"/>
-      <c r="D160" s="9">
-        <v>1</v>
-      </c>
+        <v>519</v>
+      </c>
+      <c r="C160" s="9">
+        <v>1</v>
+      </c>
+      <c r="D160" s="10"/>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A161" s="3" t="s">
-        <v>118</v>
+        <v>768</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>622</v>
-      </c>
-      <c r="C161" s="10"/>
-      <c r="D161" s="10">
-        <v>1</v>
-      </c>
+        <v>576</v>
+      </c>
+      <c r="C161" s="9">
+        <v>1</v>
+      </c>
+      <c r="D161" s="10"/>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A162" s="3" t="s">
-        <v>768</v>
+        <v>764</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>577</v>
-      </c>
-      <c r="C162" s="10"/>
-      <c r="D162" s="9">
-        <v>1</v>
-      </c>
+        <v>549</v>
+      </c>
+      <c r="C162" s="10">
+        <v>1</v>
+      </c>
+      <c r="D162" s="9"/>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A163" s="3"/>
-      <c r="B163" s="3"/>
+      <c r="A163" s="3" t="s">
+        <v>770</v>
+      </c>
+      <c r="B163" s="3" t="s">
+        <v>686</v>
+      </c>
+      <c r="C163" s="10">
+        <v>1</v>
+      </c>
+      <c r="D163" s="10"/>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A164" s="3"/>
-      <c r="B164" s="3"/>
+      <c r="A164" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="B164" s="3" t="s">
+        <v>625</v>
+      </c>
+      <c r="C164" s="10">
+        <v>1</v>
+      </c>
+      <c r="D164" s="10"/>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A165" s="3"/>
@@ -5005,18 +5094,16 @@
     <row r="166" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A166" s="3"/>
       <c r="B166" s="3"/>
-      <c r="C166" s="1"/>
-      <c r="D166" s="1"/>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A167" s="3"/>
       <c r="B167" s="3"/>
-      <c r="C167" s="1"/>
-      <c r="D167" s="1"/>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A168" s="3"/>
       <c r="B168" s="3"/>
+      <c r="C168" s="1"/>
+      <c r="D168" s="1"/>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A169" s="3"/>
@@ -5027,8 +5114,6 @@
     <row r="170" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A170" s="3"/>
       <c r="B170" s="3"/>
-      <c r="C170" s="1"/>
-      <c r="D170" s="1"/>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A171" s="3"/>
@@ -5075,10 +5160,14 @@
     <row r="178" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A178" s="3"/>
       <c r="B178" s="3"/>
+      <c r="C178" s="1"/>
+      <c r="D178" s="1"/>
     </row>
     <row r="179" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A179" s="3"/>
       <c r="B179" s="3"/>
+      <c r="C179" s="1"/>
+      <c r="D179" s="1"/>
     </row>
     <row r="180" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A180" s="3"/>
@@ -5091,14 +5180,10 @@
     <row r="182" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A182" s="3"/>
       <c r="B182" s="3"/>
-      <c r="C182" s="1"/>
-      <c r="D182" s="1"/>
     </row>
     <row r="183" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A183" s="3"/>
       <c r="B183" s="3"/>
-      <c r="C183" s="1"/>
-      <c r="D183" s="1"/>
     </row>
     <row r="184" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A184" s="3"/>
@@ -5151,26 +5236,30 @@
     <row r="192" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A192" s="3"/>
       <c r="B192" s="3"/>
+      <c r="C192" s="1"/>
+      <c r="D192" s="1"/>
     </row>
     <row r="193" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A193" s="9"/>
       <c r="B193" s="9"/>
+      <c r="C193" s="1"/>
+      <c r="D193" s="1"/>
     </row>
     <row r="194" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A194" s="9"/>
       <c r="B194" s="9"/>
     </row>
     <row r="195" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A195" s="9"/>
-      <c r="B195" s="9"/>
+      <c r="A195" s="1"/>
+      <c r="B195" s="1"/>
     </row>
     <row r="196" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A196" s="9"/>
-      <c r="B196" s="9"/>
+      <c r="A196" s="1"/>
+      <c r="B196" s="1"/>
     </row>
     <row r="197" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A197" s="9"/>
-      <c r="B197" s="9"/>
+      <c r="A197" s="1"/>
+      <c r="B197" s="1"/>
     </row>
     <row r="198" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A198" s="1"/>
@@ -5196,6 +5285,7 @@
     <row r="203" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A203" s="1"/>
       <c r="B203" s="1"/>
+      <c r="D203" s="10"/>
     </row>
     <row r="204" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A204" s="1"/>
@@ -5210,11 +5300,12 @@
     <row r="206" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A206" s="1"/>
       <c r="B206" s="1"/>
-      <c r="D206" s="10"/>
+      <c r="C206" s="10"/>
     </row>
     <row r="207" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A207" s="1"/>
       <c r="B207" s="1"/>
+      <c r="D207" s="10"/>
     </row>
     <row r="208" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A208" s="1"/>
@@ -5223,17 +5314,16 @@
     <row r="209" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A209" s="1"/>
       <c r="B209" s="1"/>
-      <c r="C209" s="10"/>
       <c r="D209" s="7"/>
     </row>
     <row r="210" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A210" s="1"/>
       <c r="B210" s="1"/>
-      <c r="D210" s="10"/>
     </row>
     <row r="211" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A211" s="1"/>
       <c r="B211" s="1"/>
+      <c r="D211" s="10"/>
     </row>
     <row r="212" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A212" s="1"/>
@@ -5246,7 +5336,6 @@
     <row r="214" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A214" s="1"/>
       <c r="B214" s="1"/>
-      <c r="D214" s="10"/>
     </row>
     <row r="215" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A215" s="1"/>
@@ -5257,26 +5346,12 @@
       <c r="B216" s="1"/>
     </row>
     <row r="217" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A217" s="1" t="s">
-        <v>771</v>
-      </c>
-      <c r="B217" s="1" t="s">
-        <v>709</v>
-      </c>
-      <c r="D217">
-        <v>1</v>
-      </c>
+      <c r="A217" s="1"/>
+      <c r="B217" s="1"/>
     </row>
     <row r="218" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A218" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="B218" s="1" t="s">
-        <v>618</v>
-      </c>
-      <c r="D218">
-        <v>1</v>
-      </c>
+      <c r="A218" s="1"/>
+      <c r="B218" s="1"/>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A219" s="1"/>
@@ -7185,7 +7260,7 @@
   </sheetData>
   <autoFilter ref="A1:D218" xr:uid="{3FE09B2D-DD5D-432F-829D-D273A0AAABBF}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D218">
-      <sortCondition descending="1" ref="C1:C218"/>
+      <sortCondition descending="1" ref="D1:D218"/>
     </sortState>
   </autoFilter>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -7197,7 +7272,7 @@
           <x14:formula1>
             <xm:f>BD!$A$1:$R$1</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A694</xm:sqref>
+          <xm:sqref>A3:A694 A2</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9EE7BA2F-C3BE-496B-873D-B1336765EE7C}">
           <x14:formula1>
@@ -7212,9 +7287,220 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{842C90A5-6A1D-4160-BB44-4221CCA559CB}">
+  <dimension ref="A1:F1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>774</v>
+      </c>
+      <c r="B1" t="s">
+        <v>775</v>
+      </c>
+      <c r="C1" t="s">
+        <v>776</v>
+      </c>
+      <c r="D1" t="s">
+        <v>777</v>
+      </c>
+      <c r="E1" t="s">
+        <v>778</v>
+      </c>
+      <c r="F1" t="s">
+        <v>779</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{262348FF-AB45-42AC-90D8-2B26510033C5}">
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>774</v>
+      </c>
+      <c r="B1" t="s">
+        <v>775</v>
+      </c>
+      <c r="C1" t="s">
+        <v>776</v>
+      </c>
+      <c r="D1" t="s">
+        <v>777</v>
+      </c>
+      <c r="E1" t="s">
+        <v>778</v>
+      </c>
+      <c r="F1" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>780</v>
+      </c>
+      <c r="B2" t="s">
+        <v>277</v>
+      </c>
+      <c r="C2">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
+        <v>759</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>781</v>
+      </c>
+      <c r="B3" t="s">
+        <v>789</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>462</v>
+      </c>
+      <c r="E3">
+        <v>5</v>
+      </c>
+      <c r="F3" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>782</v>
+      </c>
+      <c r="B4" t="s">
+        <v>251</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>118</v>
+      </c>
+      <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>783</v>
+      </c>
+      <c r="B5" t="s">
+        <v>126</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5" t="s">
+        <v>760</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>784</v>
+      </c>
+      <c r="B6" t="s">
+        <v>277</v>
+      </c>
+      <c r="C6" t="s">
+        <v>790</v>
+      </c>
+      <c r="D6" t="s">
+        <v>462</v>
+      </c>
+      <c r="E6" t="s">
+        <v>787</v>
+      </c>
+      <c r="F6" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>785</v>
+      </c>
+      <c r="B7" t="s">
+        <v>251</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>760</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>786</v>
+      </c>
+      <c r="B8" t="s">
+        <v>277</v>
+      </c>
+      <c r="C8">
+        <v>6</v>
+      </c>
+      <c r="D8" t="s">
+        <v>760</v>
+      </c>
+      <c r="E8">
+        <v>7</v>
+      </c>
+      <c r="F8" t="s">
+        <v>788</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2AAEF23-A1DA-4A41-B7F8-AB0D6A4CA83C}">
   <dimension ref="A1:D400"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
@@ -7231,87 +7517,181 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="6"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
+      <c r="A2" s="6" t="s">
+        <v>766</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="6">
+        <v>16</v>
+      </c>
+      <c r="D2" s="6">
+        <v>11</v>
+      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
+      <c r="A3" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3" s="6">
+        <v>21</v>
+      </c>
+      <c r="D3" s="6">
+        <v>10</v>
+      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="6"/>
-      <c r="B4" s="6"/>
+      <c r="A4" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>542</v>
+      </c>
       <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
+      <c r="D4" s="6">
+        <v>9</v>
+      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
+      <c r="A5" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>667</v>
+      </c>
       <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
+      <c r="D5" s="6">
+        <v>9</v>
+      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
+      <c r="A6" s="6" t="s">
+        <v>766</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="6">
+        <v>15</v>
+      </c>
+      <c r="D6" s="6">
+        <v>5</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
+      <c r="A7" s="6" t="s">
+        <v>772</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>733</v>
+      </c>
+      <c r="C7" s="6">
+        <v>11</v>
+      </c>
+      <c r="D7" s="6">
+        <v>5</v>
+      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
+      <c r="A8" s="6" t="s">
+        <v>771</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>711</v>
+      </c>
+      <c r="C8" s="6">
+        <v>10</v>
+      </c>
+      <c r="D8" s="6">
+        <v>5</v>
+      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
+      <c r="A9" s="6" t="s">
+        <v>762</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>515</v>
+      </c>
       <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
+      <c r="D9" s="6">
+        <v>5</v>
+      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
+      <c r="A10" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>632</v>
+      </c>
       <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
+      <c r="D10" s="6">
+        <v>5</v>
+      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="6"/>
-      <c r="B11" s="6"/>
+      <c r="A11" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>666</v>
+      </c>
       <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
+      <c r="D11" s="6">
+        <v>5</v>
+      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="6"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
+      <c r="A12" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="6">
+        <v>11</v>
+      </c>
       <c r="D12" s="6"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="6"/>
-      <c r="B13" s="6"/>
-      <c r="C13" s="6"/>
+      <c r="A13" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>679</v>
+      </c>
+      <c r="C13" s="6">
+        <v>10</v>
+      </c>
       <c r="D13" s="6"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="6"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
+      <c r="A14" s="6" t="s">
+        <v>762</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>520</v>
+      </c>
+      <c r="C14" s="6">
+        <v>9</v>
+      </c>
       <c r="D14" s="6"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="6"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
+      <c r="A15" s="6" t="s">
+        <v>768</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>568</v>
+      </c>
+      <c r="C15" s="6">
+        <v>9</v>
+      </c>
       <c r="D15" s="6"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -9625,6 +10005,11 @@
       <c r="D400" s="6"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D1" xr:uid="{D2AAEF23-A1DA-4A41-B7F8-AB0D6A4CA83C}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D15">
+      <sortCondition descending="1" ref="D1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
@@ -9633,7 +10018,7 @@
           <x14:formula1>
             <xm:f>BD!$A$1:$R$1</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A400</xm:sqref>
+          <xm:sqref>A3:A400 A2</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{5721DBA4-3C7D-4FF6-A482-EFB850BFBEAB}">
           <x14:formula1>
@@ -9647,10 +10032,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC46A619-F66E-4911-BB8B-97411CA835E7}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D56"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
@@ -9666,12 +10057,705 @@
         <v>178</v>
       </c>
     </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="6" t="s">
+        <v>771</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>711</v>
+      </c>
+      <c r="C2" s="6">
+        <v>2</v>
+      </c>
+      <c r="D2" s="6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="C3" s="6">
+        <v>2</v>
+      </c>
+      <c r="D3" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>540</v>
+      </c>
+      <c r="C4" s="6">
+        <v>1</v>
+      </c>
+      <c r="D4" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C5" s="6">
+        <v>1</v>
+      </c>
+      <c r="D5" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>551</v>
+      </c>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8" s="6">
+        <v>6</v>
+      </c>
+      <c r="D8" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>689</v>
+      </c>
+      <c r="C9" s="6">
+        <v>4</v>
+      </c>
+      <c r="D9" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="6" t="s">
+        <v>771</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>699</v>
+      </c>
+      <c r="C10" s="6">
+        <v>3</v>
+      </c>
+      <c r="D10" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>771</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>701</v>
+      </c>
+      <c r="C11" s="6">
+        <v>2</v>
+      </c>
+      <c r="D11" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>559</v>
+      </c>
+      <c r="C12" s="6">
+        <v>2</v>
+      </c>
+      <c r="D12" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="6" t="s">
+        <v>768</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>570</v>
+      </c>
+      <c r="C13" s="6">
+        <v>1</v>
+      </c>
+      <c r="D13" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>541</v>
+      </c>
+      <c r="C14" s="6">
+        <v>1</v>
+      </c>
+      <c r="D14" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>614</v>
+      </c>
+      <c r="C15" s="6">
+        <v>1</v>
+      </c>
+      <c r="D15" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>624</v>
+      </c>
+      <c r="C16" s="6">
+        <v>1</v>
+      </c>
+      <c r="D16" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>610</v>
+      </c>
+      <c r="C17" s="6">
+        <v>1</v>
+      </c>
+      <c r="D17" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>552</v>
+      </c>
+      <c r="C18" s="6">
+        <v>1</v>
+      </c>
+      <c r="D18" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>678</v>
+      </c>
+      <c r="C19" s="6">
+        <v>1</v>
+      </c>
+      <c r="D19" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="6" t="s">
+        <v>768</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>575</v>
+      </c>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>768</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>565</v>
+      </c>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="6" t="s">
+        <v>791</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>795</v>
+      </c>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="6" t="s">
+        <v>791</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>796</v>
+      </c>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="6" t="s">
+        <v>791</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>797</v>
+      </c>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>675</v>
+      </c>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="6" t="s">
+        <v>766</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" s="6"/>
+      <c r="D27" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>644</v>
+      </c>
+      <c r="C28" s="6"/>
+      <c r="D28" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C29" s="6"/>
+      <c r="D29" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="6" t="s">
+        <v>771</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>696</v>
+      </c>
+      <c r="C30" s="6"/>
+      <c r="D30" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C31" s="6"/>
+      <c r="D31" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C32" s="6"/>
+      <c r="D32" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>688</v>
+      </c>
+      <c r="C33" s="6"/>
+      <c r="D33" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="6" t="s">
+        <v>771</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>700</v>
+      </c>
+      <c r="C34" s="6">
+        <v>4</v>
+      </c>
+      <c r="D34" s="6"/>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="6" t="s">
+        <v>768</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>567</v>
+      </c>
+      <c r="C35" s="6">
+        <v>3</v>
+      </c>
+      <c r="D35" s="6"/>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="6" t="s">
+        <v>791</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>792</v>
+      </c>
+      <c r="C36" s="6">
+        <v>2</v>
+      </c>
+      <c r="D36" s="6"/>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>554</v>
+      </c>
+      <c r="C37" s="6">
+        <v>2</v>
+      </c>
+      <c r="D37" s="6"/>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>679</v>
+      </c>
+      <c r="C38" s="6">
+        <v>2</v>
+      </c>
+      <c r="D38" s="6"/>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>558</v>
+      </c>
+      <c r="C39" s="6">
+        <v>2</v>
+      </c>
+      <c r="D39" s="6"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>542</v>
+      </c>
+      <c r="C40" s="6">
+        <v>2</v>
+      </c>
+      <c r="D40" s="6"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="s">
+        <v>764</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>543</v>
+      </c>
+      <c r="C41" s="6">
+        <v>2</v>
+      </c>
+      <c r="D41" s="6"/>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>686</v>
+      </c>
+      <c r="C42" s="6">
+        <v>2</v>
+      </c>
+      <c r="D42" s="6"/>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="s">
+        <v>791</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>793</v>
+      </c>
+      <c r="C43" s="6">
+        <v>1</v>
+      </c>
+      <c r="D43" s="6"/>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="6" t="s">
+        <v>769</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>589</v>
+      </c>
+      <c r="C44" s="6">
+        <v>1</v>
+      </c>
+      <c r="D44" s="6"/>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" s="6" t="s">
+        <v>766</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C45" s="6">
+        <v>1</v>
+      </c>
+      <c r="D45" s="6"/>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>636</v>
+      </c>
+      <c r="C46" s="6">
+        <v>1</v>
+      </c>
+      <c r="D46" s="6"/>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="C47" s="6">
+        <v>1</v>
+      </c>
+      <c r="D47" s="6"/>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>677</v>
+      </c>
+      <c r="C48" s="6">
+        <v>1</v>
+      </c>
+      <c r="D48" s="6"/>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
+        <v>771</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>698</v>
+      </c>
+      <c r="C49" s="6">
+        <v>1</v>
+      </c>
+      <c r="D49" s="6"/>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" s="6" t="s">
+        <v>765</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>794</v>
+      </c>
+      <c r="C50" s="6">
+        <v>1</v>
+      </c>
+      <c r="D50" s="6"/>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="B51" s="6" t="s">
+        <v>687</v>
+      </c>
+      <c r="C51" s="6">
+        <v>1</v>
+      </c>
+      <c r="D51" s="6"/>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="C52" s="6">
+        <v>1</v>
+      </c>
+      <c r="D52" s="6"/>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="B53" s="6" t="s">
+        <v>690</v>
+      </c>
+      <c r="C53" s="6">
+        <v>1</v>
+      </c>
+      <c r="D53" s="6"/>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" s="6" t="s">
+        <v>767</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C54" s="6">
+        <v>1</v>
+      </c>
+      <c r="D54" s="6"/>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" s="6" t="s">
+        <v>770</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>685</v>
+      </c>
+      <c r="C55" s="6">
+        <v>1</v>
+      </c>
+      <c r="D55" s="6"/>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" s="6" t="s">
+        <v>765</v>
+      </c>
+      <c r="B56" s="6"/>
+      <c r="C56" s="6"/>
+      <c r="D56" s="6"/>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:D1" xr:uid="{EC46A619-F66E-4911-BB8B-97411CA835E7}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D56">
+      <sortCondition descending="1" ref="D1"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8766A35D-A2D5-46F6-9349-21CBEF25DC17}">
   <dimension ref="A1:R24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -10848,7 +11932,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{212B8270-F54B-455C-9F1F-A00A4AC2D0B9}">
   <dimension ref="A1:AN24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
Correccion de logotipos, jugadores fantasma y mapeo de estadisticas
</commit_message>
<xml_diff>
--- a/lmi temp 9.xlsx
+++ b/lmi temp 9.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex1\Downloads\LMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4F7C750-5CC6-4F28-B51B-9EEC880D7F8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{162831FF-7276-4DAD-A5B2-85E60E29AAB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="3744" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{37EE0A92-4687-43D8-82AB-58C1E8ACFD8D}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{37EE0A92-4687-43D8-82AB-58C1E8ACFD8D}"/>
   </bookViews>
   <sheets>
     <sheet name="Registro Liga" sheetId="2" r:id="rId1"/>
@@ -23,7 +23,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Registro Champions'!$A$1:$D$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Registro Liga'!$A$1:$D$218</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Registro Liga'!$A$1:$D$220</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">RegistroEstelar!$A$1:$D$1</definedName>
     <definedName name="AC_Milan">BD!$E$2:$E$24</definedName>
     <definedName name="AC_Milán">Lista!$E$2:$E$1048576</definedName>
@@ -100,7 +100,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1277" uniqueCount="881">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1307" uniqueCount="882">
   <si>
     <t xml:space="preserve">Alessandro Bastoni  </t>
   </si>
@@ -2743,6 +2743,9 @@
   </si>
   <si>
     <t>DC Benjamin Šeško</t>
+  </si>
+  <si>
+    <t>Por jugar</t>
   </si>
 </sst>
 </file>
@@ -2851,7 +2854,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2878,6 +2881,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3214,6 +3220,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FE09B2D-DD5D-432F-829D-D273A0AAABBF}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:E694"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3237,7 +3244,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>771</v>
       </c>
@@ -3251,7 +3258,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>764</v>
       </c>
@@ -3262,13 +3269,13 @@
         <v>5</v>
       </c>
       <c r="D3" s="3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E3" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>771</v>
       </c>
@@ -3282,7 +3289,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>137</v>
       </c>
@@ -3296,7 +3303,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>764</v>
       </c>
@@ -3304,13 +3311,13 @@
         <v>41</v>
       </c>
       <c r="C6" s="3">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D6" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>763</v>
       </c>
@@ -3324,7 +3331,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>767</v>
       </c>
@@ -3338,7 +3345,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>770</v>
       </c>
@@ -3352,7 +3359,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>137</v>
       </c>
@@ -3366,7 +3373,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>137</v>
       </c>
@@ -3378,7 +3385,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>766</v>
       </c>
@@ -3392,7 +3399,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>771</v>
       </c>
@@ -3406,7 +3413,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>766</v>
       </c>
@@ -3420,7 +3427,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>126</v>
       </c>
@@ -3432,7 +3439,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>766</v>
       </c>
@@ -3446,7 +3453,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>771</v>
       </c>
@@ -3460,7 +3467,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>763</v>
       </c>
@@ -3474,7 +3481,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>773</v>
       </c>
@@ -3488,7 +3495,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>771</v>
       </c>
@@ -3502,7 +3509,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>770</v>
       </c>
@@ -3514,7 +3521,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>137</v>
       </c>
@@ -3528,7 +3535,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>767</v>
       </c>
@@ -3542,7 +3549,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>763</v>
       </c>
@@ -3556,7 +3563,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>767</v>
       </c>
@@ -3570,7 +3577,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>763</v>
       </c>
@@ -3584,7 +3591,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>767</v>
       </c>
@@ -3612,7 +3619,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>126</v>
       </c>
@@ -3637,10 +3644,10 @@
         <v>1</v>
       </c>
       <c r="D30" s="3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>762</v>
       </c>
@@ -3654,7 +3661,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>767</v>
       </c>
@@ -3666,7 +3673,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
         <v>770</v>
       </c>
@@ -3678,7 +3685,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
         <v>765</v>
       </c>
@@ -3690,7 +3697,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
         <v>762</v>
       </c>
@@ -3702,7 +3709,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>137</v>
       </c>
@@ -3714,7 +3721,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>137</v>
       </c>
@@ -3726,7 +3733,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
         <v>764</v>
       </c>
@@ -3750,7 +3757,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
         <v>126</v>
       </c>
@@ -3764,7 +3771,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
         <v>773</v>
       </c>
@@ -3778,7 +3785,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
         <v>768</v>
       </c>
@@ -3792,7 +3799,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
         <v>767</v>
       </c>
@@ -3806,7 +3813,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
         <v>768</v>
       </c>
@@ -3817,10 +3824,10 @@
         <v>5</v>
       </c>
       <c r="D44" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
         <v>764</v>
       </c>
@@ -3834,7 +3841,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
         <v>762</v>
       </c>
@@ -3862,7 +3869,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>126</v>
       </c>
@@ -3876,7 +3883,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
         <v>764</v>
       </c>
@@ -3898,10 +3905,10 @@
         <v>114</v>
       </c>
       <c r="C50" s="3">
+        <v>5</v>
+      </c>
+      <c r="D50" s="3">
         <v>3</v>
-      </c>
-      <c r="D50" s="3">
-        <v>2</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
@@ -3918,7 +3925,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
         <v>773</v>
       </c>
@@ -3940,13 +3947,13 @@
         <v>111</v>
       </c>
       <c r="C53" s="3">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D53" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
         <v>770</v>
       </c>
@@ -3960,7 +3967,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
         <v>766</v>
       </c>
@@ -3974,7 +3981,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
         <v>773</v>
       </c>
@@ -3988,7 +3995,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
         <v>773</v>
       </c>
@@ -4002,7 +4009,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
         <v>765</v>
       </c>
@@ -4016,7 +4023,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
         <v>773</v>
       </c>
@@ -4030,7 +4037,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
         <v>766</v>
       </c>
@@ -4044,7 +4051,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
         <v>768</v>
       </c>
@@ -4058,7 +4065,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
         <v>767</v>
       </c>
@@ -4086,7 +4093,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
         <v>765</v>
       </c>
@@ -4098,7 +4105,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
         <v>764</v>
       </c>
@@ -4110,7 +4117,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
         <v>767</v>
       </c>
@@ -4122,7 +4129,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
         <v>770</v>
       </c>
@@ -4134,7 +4141,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
         <v>771</v>
       </c>
@@ -4146,7 +4153,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
         <v>762</v>
       </c>
@@ -4170,7 +4177,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
         <v>770</v>
       </c>
@@ -4182,7 +4189,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
         <v>770</v>
       </c>
@@ -4196,7 +4203,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
         <v>770</v>
       </c>
@@ -4210,7 +4217,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
         <v>765</v>
       </c>
@@ -4224,7 +4231,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
         <v>764</v>
       </c>
@@ -4238,7 +4245,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
         <v>764</v>
       </c>
@@ -4266,7 +4273,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78" s="3" t="s">
         <v>763</v>
       </c>
@@ -4308,7 +4315,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
         <v>126</v>
       </c>
@@ -4325,7 +4332,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82" s="3" t="s">
         <v>773</v>
       </c>
@@ -4339,7 +4346,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83" s="3" t="s">
         <v>767</v>
       </c>
@@ -4353,7 +4360,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84" s="3" t="s">
         <v>762</v>
       </c>
@@ -4367,7 +4374,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85" s="3" t="s">
         <v>766</v>
       </c>
@@ -4381,7 +4388,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86" s="3" t="s">
         <v>762</v>
       </c>
@@ -4395,7 +4402,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87" s="3" t="s">
         <v>137</v>
       </c>
@@ -4423,7 +4430,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89" s="3" t="s">
         <v>771</v>
       </c>
@@ -4445,13 +4452,13 @@
         <v>609</v>
       </c>
       <c r="C90" s="6">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D90" s="6">
         <v>1</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91" s="3" t="s">
         <v>763</v>
       </c>
@@ -4465,7 +4472,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92" s="3" t="s">
         <v>126</v>
       </c>
@@ -4479,7 +4486,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93" s="3" t="s">
         <v>767</v>
       </c>
@@ -4507,7 +4514,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95" s="3" t="s">
         <v>768</v>
       </c>
@@ -4515,13 +4522,13 @@
         <v>103</v>
       </c>
       <c r="C95" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D95" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:5" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96" s="3" t="s">
         <v>768</v>
       </c>
@@ -4535,7 +4542,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97" s="3" t="s">
         <v>765</v>
       </c>
@@ -4549,7 +4556,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
         <v>765</v>
       </c>
@@ -4563,7 +4570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99" s="3" t="s">
         <v>771</v>
       </c>
@@ -4577,7 +4584,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" s="3" t="s">
         <v>137</v>
       </c>
@@ -4591,7 +4598,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" s="3" t="s">
         <v>768</v>
       </c>
@@ -4605,7 +4612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" s="3" t="s">
         <v>137</v>
       </c>
@@ -4619,7 +4626,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" s="3" t="s">
         <v>764</v>
       </c>
@@ -4633,7 +4640,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" s="3" t="s">
         <v>771</v>
       </c>
@@ -4647,7 +4654,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" s="3" t="s">
         <v>766</v>
       </c>
@@ -4683,7 +4690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" s="3" t="s">
         <v>126</v>
       </c>
@@ -4695,7 +4702,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" s="3" t="s">
         <v>765</v>
       </c>
@@ -4707,7 +4714,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" s="3" t="s">
         <v>764</v>
       </c>
@@ -4719,7 +4726,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" s="3" t="s">
         <v>767</v>
       </c>
@@ -4743,7 +4750,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A113" s="3" t="s">
         <v>773</v>
       </c>
@@ -4755,7 +4762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A114" s="3" t="s">
         <v>766</v>
       </c>
@@ -4767,7 +4774,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A115" s="3" t="s">
         <v>768</v>
       </c>
@@ -4779,7 +4786,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A116" s="3" t="s">
         <v>765</v>
       </c>
@@ -4791,7 +4798,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A117" s="3" t="s">
         <v>764</v>
       </c>
@@ -4803,7 +4810,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A118" s="3" t="s">
         <v>770</v>
       </c>
@@ -4815,7 +4822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A119" s="3" t="s">
         <v>765</v>
       </c>
@@ -4827,7 +4834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A120" s="3" t="s">
         <v>770</v>
       </c>
@@ -4839,7 +4846,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A121" s="3" t="s">
         <v>766</v>
       </c>
@@ -4851,7 +4858,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A122" s="3" t="s">
         <v>766</v>
       </c>
@@ -4863,7 +4870,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A123" s="3" t="s">
         <v>137</v>
       </c>
@@ -4875,7 +4882,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="124" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A124" s="3" t="s">
         <v>767</v>
       </c>
@@ -4887,7 +4894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A125" s="3" t="s">
         <v>763</v>
       </c>
@@ -4911,7 +4918,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A127" s="3" t="s">
         <v>768</v>
       </c>
@@ -4923,7 +4930,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A128" s="3" t="s">
         <v>771</v>
       </c>
@@ -4944,10 +4951,10 @@
       </c>
       <c r="C129" s="6"/>
       <c r="D129" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="130" spans="1:4" x14ac:dyDescent="0.3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="130" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A130" s="3" t="s">
         <v>767</v>
       </c>
@@ -4959,7 +4966,7 @@
       </c>
       <c r="D130" s="3"/>
     </row>
-    <row r="131" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A131" s="3" t="s">
         <v>765</v>
       </c>
@@ -4971,7 +4978,7 @@
       </c>
       <c r="D131" s="3"/>
     </row>
-    <row r="132" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A132" s="3" t="s">
         <v>764</v>
       </c>
@@ -4983,7 +4990,7 @@
       </c>
       <c r="D132" s="3"/>
     </row>
-    <row r="133" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A133" s="3" t="s">
         <v>767</v>
       </c>
@@ -4995,7 +5002,7 @@
       </c>
       <c r="D133" s="3"/>
     </row>
-    <row r="134" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A134" s="3" t="s">
         <v>126</v>
       </c>
@@ -5007,7 +5014,7 @@
       </c>
       <c r="D134" s="3"/>
     </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A135" s="3" t="s">
         <v>773</v>
       </c>
@@ -5019,7 +5026,7 @@
       </c>
       <c r="D135" s="3"/>
     </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A136" s="3" t="s">
         <v>762</v>
       </c>
@@ -5043,7 +5050,7 @@
       </c>
       <c r="D137" s="3"/>
     </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A138" s="3" t="s">
         <v>770</v>
       </c>
@@ -5055,7 +5062,7 @@
       </c>
       <c r="D138" s="3"/>
     </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A139" s="3" t="s">
         <v>126</v>
       </c>
@@ -5067,7 +5074,7 @@
       </c>
       <c r="D139" s="1"/>
     </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A140" s="3" t="s">
         <v>770</v>
       </c>
@@ -5079,7 +5086,7 @@
       </c>
       <c r="D140" s="1"/>
     </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A141" s="3" t="s">
         <v>773</v>
       </c>
@@ -5092,15 +5099,9 @@
       <c r="D141" s="1"/>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A142" s="3" t="s">
-        <v>769</v>
-      </c>
-      <c r="B142" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="C142" s="1">
-        <v>2</v>
-      </c>
+      <c r="A142" s="3"/>
+      <c r="B142" s="3"/>
+      <c r="C142" s="1"/>
       <c r="D142" s="1"/>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.3">
@@ -5111,11 +5112,11 @@
         <v>108</v>
       </c>
       <c r="C143" s="1">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D143" s="1"/>
     </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A144" s="3" t="s">
         <v>137</v>
       </c>
@@ -5127,7 +5128,7 @@
       </c>
       <c r="D144" s="1"/>
     </row>
-    <row r="145" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A145" s="3" t="s">
         <v>766</v>
       </c>
@@ -5139,7 +5140,7 @@
       </c>
       <c r="D145" s="1"/>
     </row>
-    <row r="146" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A146" s="3" t="s">
         <v>126</v>
       </c>
@@ -5151,7 +5152,7 @@
       </c>
       <c r="D146" s="1"/>
     </row>
-    <row r="147" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A147" s="3" t="s">
         <v>126</v>
       </c>
@@ -5162,7 +5163,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="148" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A148" s="3" t="s">
         <v>762</v>
       </c>
@@ -5174,7 +5175,7 @@
       </c>
       <c r="D148" s="1"/>
     </row>
-    <row r="149" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A149" s="3" t="s">
         <v>764</v>
       </c>
@@ -5186,7 +5187,7 @@
       </c>
       <c r="D149" s="1"/>
     </row>
-    <row r="150" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A150" s="3" t="s">
         <v>762</v>
       </c>
@@ -5210,7 +5211,7 @@
       </c>
       <c r="D151" s="1"/>
     </row>
-    <row r="152" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A152" s="3" t="s">
         <v>768</v>
       </c>
@@ -5234,7 +5235,7 @@
       </c>
       <c r="D153" s="1"/>
     </row>
-    <row r="154" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A154" s="3" t="s">
         <v>767</v>
       </c>
@@ -5246,7 +5247,7 @@
       </c>
       <c r="D154" s="1"/>
     </row>
-    <row r="155" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A155" s="3" t="s">
         <v>762</v>
       </c>
@@ -5258,7 +5259,7 @@
       </c>
       <c r="D155" s="1"/>
     </row>
-    <row r="156" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A156" s="3" t="s">
         <v>765</v>
       </c>
@@ -5270,7 +5271,7 @@
       </c>
       <c r="D156" s="1"/>
     </row>
-    <row r="157" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A157" s="3" t="s">
         <v>137</v>
       </c>
@@ -5282,7 +5283,7 @@
       </c>
       <c r="D157" s="1"/>
     </row>
-    <row r="158" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A158" s="3" t="s">
         <v>771</v>
       </c>
@@ -5294,7 +5295,7 @@
       </c>
       <c r="D158" s="1"/>
     </row>
-    <row r="159" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A159" s="3" t="s">
         <v>771</v>
       </c>
@@ -5306,7 +5307,7 @@
       </c>
       <c r="D159" s="1"/>
     </row>
-    <row r="160" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A160" s="3" t="s">
         <v>762</v>
       </c>
@@ -5317,7 +5318,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A161" s="3" t="s">
         <v>768</v>
       </c>
@@ -5328,7 +5329,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A162" s="3" t="s">
         <v>764</v>
       </c>
@@ -5340,7 +5341,7 @@
       </c>
       <c r="D162" s="1"/>
     </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A163" s="3" t="s">
         <v>770</v>
       </c>
@@ -5362,275 +5363,289 @@
         <v>1</v>
       </c>
     </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A165" s="3"/>
       <c r="B165" s="3"/>
     </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A166" s="3"/>
       <c r="B166" s="3"/>
     </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A167" s="3"/>
       <c r="B167" s="3"/>
     </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A168" s="3"/>
       <c r="B168" s="3"/>
       <c r="C168" s="1"/>
       <c r="D168" s="1"/>
     </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A169" s="3"/>
       <c r="B169" s="3"/>
       <c r="C169" s="1"/>
       <c r="D169" s="1"/>
     </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A170" s="3"/>
       <c r="B170" s="3"/>
     </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A171" s="3"/>
       <c r="B171" s="3"/>
       <c r="C171" s="1"/>
       <c r="D171" s="1"/>
     </row>
-    <row r="172" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A172" s="3"/>
       <c r="B172" s="3"/>
       <c r="C172" s="1"/>
       <c r="D172" s="1"/>
     </row>
-    <row r="173" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A173" s="3"/>
       <c r="B173" s="3"/>
       <c r="C173" s="1"/>
       <c r="D173" s="1"/>
     </row>
-    <row r="174" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A174" s="3"/>
       <c r="B174" s="3"/>
       <c r="C174" s="1"/>
       <c r="D174" s="1"/>
     </row>
-    <row r="175" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A175" s="3"/>
       <c r="B175" s="3"/>
       <c r="C175" s="1"/>
       <c r="D175" s="1"/>
     </row>
-    <row r="176" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A176" s="3"/>
       <c r="B176" s="3"/>
       <c r="C176" s="1"/>
       <c r="D176" s="1"/>
     </row>
-    <row r="177" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A177" s="3"/>
       <c r="B177" s="3"/>
       <c r="C177" s="1"/>
       <c r="D177" s="1"/>
     </row>
-    <row r="178" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A178" s="3"/>
       <c r="B178" s="3"/>
       <c r="C178" s="1"/>
       <c r="D178" s="1"/>
     </row>
-    <row r="179" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A179" s="3"/>
       <c r="B179" s="3"/>
       <c r="C179" s="1"/>
       <c r="D179" s="1"/>
     </row>
-    <row r="180" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A180" s="3"/>
       <c r="B180" s="3"/>
     </row>
-    <row r="181" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A181" s="3"/>
       <c r="B181" s="3"/>
     </row>
-    <row r="182" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A182" s="3"/>
       <c r="B182" s="3"/>
     </row>
-    <row r="183" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A183" s="3"/>
       <c r="B183" s="3"/>
     </row>
-    <row r="184" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A184" s="3"/>
       <c r="B184" s="3"/>
       <c r="C184" s="1"/>
       <c r="D184" s="1"/>
     </row>
-    <row r="185" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A185" s="3"/>
       <c r="B185" s="3"/>
       <c r="C185" s="1"/>
       <c r="D185" s="1"/>
     </row>
-    <row r="186" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A186" s="3"/>
       <c r="B186" s="3"/>
       <c r="C186" s="1"/>
       <c r="D186" s="1"/>
     </row>
-    <row r="187" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A187" s="3"/>
       <c r="B187" s="3"/>
       <c r="C187" s="1"/>
       <c r="D187" s="1"/>
     </row>
-    <row r="188" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A188" s="3"/>
       <c r="B188" s="3"/>
       <c r="C188" s="1"/>
       <c r="D188" s="1"/>
     </row>
-    <row r="189" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A189" s="3"/>
       <c r="B189" s="3"/>
       <c r="C189" s="1"/>
       <c r="D189" s="1"/>
     </row>
-    <row r="190" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A190" s="3"/>
       <c r="B190" s="3"/>
       <c r="C190" s="1"/>
       <c r="D190" s="1"/>
     </row>
-    <row r="191" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A191" s="3"/>
       <c r="B191" s="3"/>
       <c r="C191" s="1"/>
       <c r="D191" s="1"/>
     </row>
-    <row r="192" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A192" s="3"/>
       <c r="B192" s="3"/>
       <c r="C192" s="1"/>
       <c r="D192" s="1"/>
     </row>
-    <row r="193" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A193" s="1"/>
       <c r="B193" s="1"/>
       <c r="C193" s="1"/>
       <c r="D193" s="1"/>
     </row>
-    <row r="194" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A194" s="1"/>
       <c r="B194" s="1"/>
     </row>
-    <row r="195" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A195" s="1"/>
       <c r="B195" s="1"/>
     </row>
-    <row r="196" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A196" s="1"/>
       <c r="B196" s="1"/>
     </row>
-    <row r="197" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A197" s="1"/>
       <c r="B197" s="1"/>
     </row>
-    <row r="198" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A198" s="1"/>
       <c r="B198" s="1"/>
     </row>
-    <row r="199" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A199" s="1"/>
       <c r="B199" s="1"/>
     </row>
-    <row r="200" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A200" s="1"/>
       <c r="B200" s="1"/>
     </row>
-    <row r="201" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A201" s="1"/>
       <c r="B201" s="1"/>
       <c r="D201" s="7"/>
     </row>
-    <row r="202" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A202" s="1"/>
       <c r="B202" s="1"/>
     </row>
-    <row r="203" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A203" s="1"/>
       <c r="B203" s="1"/>
     </row>
-    <row r="204" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A204" s="1"/>
       <c r="B204" s="1"/>
       <c r="C204" s="7"/>
     </row>
-    <row r="205" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A205" s="1"/>
       <c r="B205" s="1"/>
       <c r="D205" s="8"/>
     </row>
-    <row r="206" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A206" s="1"/>
       <c r="B206" s="1"/>
     </row>
-    <row r="207" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A207" s="1"/>
       <c r="B207" s="1"/>
     </row>
-    <row r="208" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A208" s="1"/>
       <c r="B208" s="1"/>
     </row>
-    <row r="209" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A209" s="1"/>
       <c r="B209" s="1"/>
       <c r="D209" s="7"/>
     </row>
-    <row r="210" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A210" s="1"/>
       <c r="B210" s="1"/>
     </row>
-    <row r="211" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A211" s="1"/>
       <c r="B211" s="1"/>
     </row>
-    <row r="212" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A212" s="1"/>
       <c r="B212" s="1"/>
     </row>
-    <row r="213" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A213" s="1"/>
       <c r="B213" s="1"/>
     </row>
-    <row r="214" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A214" s="1"/>
       <c r="B214" s="1"/>
     </row>
-    <row r="215" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A215" s="1"/>
       <c r="B215" s="1"/>
     </row>
-    <row r="216" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A216" s="1"/>
       <c r="B216" s="1"/>
     </row>
-    <row r="217" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A217" s="1"/>
       <c r="B217" s="1"/>
     </row>
-    <row r="218" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A218" s="1"/>
       <c r="B218" s="1"/>
     </row>
     <row r="219" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A219" s="1"/>
-      <c r="B219" s="1"/>
+      <c r="A219" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="B219" s="1" t="s">
+        <v>595</v>
+      </c>
+      <c r="C219" s="12">
+        <v>1</v>
+      </c>
     </row>
     <row r="220" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A220" s="1"/>
-      <c r="B220" s="1"/>
+      <c r="A220" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="B220" s="1" t="s">
+        <v>585</v>
+      </c>
+      <c r="D220">
+        <v>1</v>
+      </c>
     </row>
     <row r="221" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A221" s="1"/>
@@ -7529,7 +7544,13 @@
       <c r="B694" s="1"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D218" xr:uid="{3FE09B2D-DD5D-432F-829D-D273A0AAABBF}">
+  <autoFilter ref="A1:D220" xr:uid="{3FE09B2D-DD5D-432F-829D-D273A0AAABBF}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="Boca_Juniors"/>
+        <filter val="Galatasaray"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D218">
       <sortCondition descending="1" ref="D1:D218"/>
     </sortState>
@@ -7559,8 +7580,12 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{842C90A5-6A1D-4160-BB44-4221CCA559CB}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -7580,6 +7605,140 @@
       </c>
       <c r="F1" t="s">
         <v>779</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>780</v>
+      </c>
+      <c r="B2" t="s">
+        <v>251</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>253</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>781</v>
+      </c>
+      <c r="B3" t="s">
+        <v>463</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>277</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>782</v>
+      </c>
+      <c r="B4" t="s">
+        <v>462</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>126</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>783</v>
+      </c>
+      <c r="B5" t="s">
+        <v>180</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>760</v>
+      </c>
+      <c r="E5">
+        <v>3</v>
+      </c>
+      <c r="F5" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>784</v>
+      </c>
+      <c r="B6" t="s">
+        <v>277</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>251</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>785</v>
+      </c>
+      <c r="B7" t="s">
+        <v>126</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7" t="s">
+        <v>760</v>
+      </c>
+      <c r="E7">
+        <v>3</v>
+      </c>
+      <c r="F7" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>786</v>
+      </c>
+      <c r="B8" t="s">
+        <v>760</v>
+      </c>
+      <c r="D8" t="s">
+        <v>277</v>
+      </c>
+      <c r="F8" t="s">
+        <v>881</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corregir mapeo dinamico de cabeceras de Clubes y sincronizar presupuestos
</commit_message>
<xml_diff>
--- a/lmi temp 9.xlsx
+++ b/lmi temp 9.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex1\Downloads\LMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{291956E7-BF86-426E-A323-BF6F76A69A3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFE2F89F-F13F-47A8-8A3B-E8232BBF7A8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="3744" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1447" uniqueCount="958">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1397" uniqueCount="952">
   <si>
     <t>Equipo</t>
   </si>
@@ -2745,48 +2745,21 @@
     <t>Presupuesto Inicial</t>
   </si>
   <si>
-    <t>Color Primario</t>
-  </si>
-  <si>
-    <t>Color Secundario</t>
-  </si>
-  <si>
-    <t>Degradado Fondo</t>
-  </si>
-  <si>
     <t>Logo</t>
   </si>
   <si>
-    <t>Nota Cambio Leyenda</t>
-  </si>
-  <si>
-    <t>Nota Eliminar Leyenda</t>
-  </si>
-  <si>
     <t>INT</t>
   </si>
   <si>
     <t>Director Técnico</t>
   </si>
   <si>
-    <t>#004789</t>
-  </si>
-  <si>
-    <t>#ffffff</t>
-  </si>
-  <si>
-    <t>linear-gradient(135deg, #0b0e15 0%, #161f30 100%)</t>
-  </si>
-  <si>
     <t>Logos Equipos/intermilan.webp</t>
   </si>
   <si>
     <t>REA</t>
   </si>
   <si>
-    <t>#000000</t>
-  </si>
-  <si>
     <t>Logos Equipos/realmadrid.webp</t>
   </si>
   <si>
@@ -2956,6 +2929,15 @@
   </si>
   <si>
     <t>Racecourse Ground</t>
+  </si>
+  <si>
+    <t>CT Strahinja Pavlović</t>
+  </si>
+  <si>
+    <t>ED Ismaila Sarr</t>
+  </si>
+  <si>
+    <t>CT Aymeric Laporte</t>
   </si>
 </sst>
 </file>
@@ -13681,7 +13663,9 @@
       <c r="N20" s="3" t="s">
         <v>820</v>
       </c>
-      <c r="O20" s="3"/>
+      <c r="O20" s="3" t="s">
+        <v>949</v>
+      </c>
       <c r="P20" s="3"/>
       <c r="Q20" s="3"/>
       <c r="R20" s="3" t="s">
@@ -13731,7 +13715,9 @@
       <c r="N21" s="3" t="s">
         <v>835</v>
       </c>
-      <c r="O21" s="3"/>
+      <c r="O21" s="3" t="s">
+        <v>950</v>
+      </c>
       <c r="P21" s="3"/>
       <c r="Q21" s="3"/>
       <c r="R21" s="3" t="s">
@@ -13781,7 +13767,9 @@
       <c r="N22" s="3" t="s">
         <v>850</v>
       </c>
-      <c r="O22" s="3"/>
+      <c r="O22" s="3" t="s">
+        <v>951</v>
+      </c>
       <c r="P22" s="3"/>
       <c r="Q22" s="3"/>
       <c r="R22" s="3" t="s">
@@ -13895,24 +13883,19 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="14.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="43.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="31.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.5546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -13934,34 +13917,19 @@
       <c r="G1" t="s">
         <v>887</v>
       </c>
-      <c r="H1" t="s">
-        <v>888</v>
-      </c>
-      <c r="I1" t="s">
-        <v>889</v>
-      </c>
-      <c r="J1" t="s">
-        <v>890</v>
-      </c>
-      <c r="K1" t="s">
-        <v>891</v>
-      </c>
-      <c r="L1" t="s">
-        <v>892</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>198</v>
       </c>
       <c r="B2" t="s">
-        <v>893</v>
+        <v>888</v>
       </c>
       <c r="C2" t="s">
-        <v>943</v>
+        <v>934</v>
       </c>
       <c r="D2" t="s">
-        <v>929</v>
+        <v>920</v>
       </c>
       <c r="E2">
         <v>100000000</v>
@@ -13970,30 +13938,21 @@
         <v>1259000000</v>
       </c>
       <c r="G2" t="s">
-        <v>895</v>
-      </c>
-      <c r="H2" t="s">
-        <v>896</v>
-      </c>
-      <c r="I2" t="s">
-        <v>897</v>
-      </c>
-      <c r="J2" t="s">
-        <v>898</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+        <v>890</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>516</v>
       </c>
       <c r="B3" t="s">
-        <v>899</v>
+        <v>891</v>
       </c>
       <c r="C3" t="s">
-        <v>944</v>
+        <v>935</v>
       </c>
       <c r="D3" t="s">
-        <v>930</v>
+        <v>921</v>
       </c>
       <c r="E3">
         <v>100000000</v>
@@ -14002,30 +13961,21 @@
         <v>191000000</v>
       </c>
       <c r="G3" t="s">
-        <v>900</v>
-      </c>
-      <c r="H3" t="s">
-        <v>896</v>
-      </c>
-      <c r="I3" t="s">
-        <v>897</v>
-      </c>
-      <c r="J3" t="s">
-        <v>901</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+        <v>892</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>189</v>
       </c>
       <c r="B4" t="s">
-        <v>902</v>
+        <v>893</v>
       </c>
       <c r="C4" t="s">
-        <v>945</v>
+        <v>936</v>
       </c>
       <c r="D4" t="s">
-        <v>931</v>
+        <v>922</v>
       </c>
       <c r="E4">
         <v>100000000</v>
@@ -14034,30 +13984,21 @@
         <v>2097000000</v>
       </c>
       <c r="G4" t="s">
-        <v>895</v>
-      </c>
-      <c r="H4" t="s">
-        <v>896</v>
-      </c>
-      <c r="I4" t="s">
-        <v>897</v>
-      </c>
-      <c r="J4" t="s">
-        <v>903</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+        <v>894</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>517</v>
       </c>
       <c r="B5" t="s">
-        <v>904</v>
+        <v>895</v>
       </c>
       <c r="C5" t="s">
-        <v>946</v>
+        <v>937</v>
       </c>
       <c r="D5" t="s">
-        <v>894</v>
+        <v>889</v>
       </c>
       <c r="E5">
         <v>100000000</v>
@@ -14066,30 +14007,21 @@
         <v>300000000</v>
       </c>
       <c r="G5" t="s">
-        <v>895</v>
-      </c>
-      <c r="H5" t="s">
         <v>896</v>
       </c>
-      <c r="I5" t="s">
-        <v>897</v>
-      </c>
-      <c r="J5" t="s">
-        <v>905</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>190</v>
       </c>
       <c r="B6" t="s">
-        <v>906</v>
+        <v>897</v>
       </c>
       <c r="C6" t="s">
-        <v>943</v>
+        <v>934</v>
       </c>
       <c r="D6" t="s">
-        <v>932</v>
+        <v>923</v>
       </c>
       <c r="E6">
         <v>100000000</v>
@@ -14098,30 +14030,21 @@
         <v>251000000</v>
       </c>
       <c r="G6" t="s">
-        <v>895</v>
-      </c>
-      <c r="H6" t="s">
-        <v>896</v>
-      </c>
-      <c r="I6" t="s">
-        <v>897</v>
-      </c>
-      <c r="J6" t="s">
-        <v>907</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+        <v>898</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>194</v>
       </c>
       <c r="B7" t="s">
-        <v>908</v>
+        <v>899</v>
       </c>
       <c r="C7" t="s">
-        <v>947</v>
+        <v>938</v>
       </c>
       <c r="D7" t="s">
-        <v>933</v>
+        <v>924</v>
       </c>
       <c r="E7">
         <v>100000000</v>
@@ -14130,30 +14053,21 @@
         <v>1265000000</v>
       </c>
       <c r="G7" t="s">
-        <v>895</v>
-      </c>
-      <c r="H7" t="s">
-        <v>896</v>
-      </c>
-      <c r="I7" t="s">
-        <v>897</v>
-      </c>
-      <c r="J7" t="s">
-        <v>909</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+        <v>900</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>204</v>
       </c>
       <c r="B8" t="s">
-        <v>910</v>
+        <v>901</v>
       </c>
       <c r="C8" t="s">
-        <v>948</v>
+        <v>939</v>
       </c>
       <c r="D8" t="s">
-        <v>934</v>
+        <v>925</v>
       </c>
       <c r="E8">
         <v>100000000</v>
@@ -14162,30 +14076,21 @@
         <v>300000000</v>
       </c>
       <c r="G8" t="s">
-        <v>895</v>
-      </c>
-      <c r="H8" t="s">
-        <v>896</v>
-      </c>
-      <c r="I8" t="s">
-        <v>897</v>
-      </c>
-      <c r="J8" t="s">
-        <v>911</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>518</v>
       </c>
       <c r="B9" t="s">
-        <v>912</v>
+        <v>903</v>
       </c>
       <c r="C9" t="s">
-        <v>949</v>
+        <v>940</v>
       </c>
       <c r="D9" t="s">
-        <v>935</v>
+        <v>926</v>
       </c>
       <c r="E9">
         <v>100000000</v>
@@ -14194,30 +14099,21 @@
         <v>921000000</v>
       </c>
       <c r="G9" t="s">
-        <v>895</v>
-      </c>
-      <c r="H9" t="s">
-        <v>896</v>
-      </c>
-      <c r="I9" t="s">
-        <v>897</v>
-      </c>
-      <c r="J9" t="s">
-        <v>913</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>54</v>
       </c>
       <c r="B10" t="s">
-        <v>914</v>
+        <v>905</v>
       </c>
       <c r="C10" t="s">
-        <v>950</v>
+        <v>941</v>
       </c>
       <c r="D10" t="s">
-        <v>936</v>
+        <v>927</v>
       </c>
       <c r="E10">
         <v>100000000</v>
@@ -14226,19 +14122,10 @@
         <v>205000000</v>
       </c>
       <c r="G10" t="s">
-        <v>895</v>
-      </c>
-      <c r="H10" t="s">
-        <v>896</v>
-      </c>
-      <c r="I10" t="s">
-        <v>897</v>
-      </c>
-      <c r="J10" t="s">
-        <v>915</v>
-      </c>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+        <v>906</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -14246,10 +14133,10 @@
         <v>25</v>
       </c>
       <c r="C11" t="s">
-        <v>951</v>
+        <v>942</v>
       </c>
       <c r="D11" t="s">
-        <v>937</v>
+        <v>928</v>
       </c>
       <c r="E11">
         <v>100000000</v>
@@ -14258,30 +14145,21 @@
         <v>433000000</v>
       </c>
       <c r="G11" t="s">
-        <v>895</v>
-      </c>
-      <c r="H11" t="s">
-        <v>896</v>
-      </c>
-      <c r="I11" t="s">
-        <v>897</v>
-      </c>
-      <c r="J11" t="s">
-        <v>916</v>
-      </c>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>917</v>
+        <v>908</v>
       </c>
       <c r="C12" t="s">
-        <v>952</v>
+        <v>943</v>
       </c>
       <c r="D12" t="s">
-        <v>894</v>
+        <v>889</v>
       </c>
       <c r="E12">
         <v>100000000</v>
@@ -14290,30 +14168,21 @@
         <v>300000000</v>
       </c>
       <c r="G12" t="s">
-        <v>895</v>
-      </c>
-      <c r="H12" t="s">
-        <v>896</v>
-      </c>
-      <c r="I12" t="s">
-        <v>897</v>
-      </c>
-      <c r="J12" t="s">
-        <v>918</v>
-      </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+        <v>909</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>199</v>
       </c>
       <c r="B13" t="s">
-        <v>919</v>
+        <v>910</v>
       </c>
       <c r="C13" t="s">
-        <v>953</v>
+        <v>944</v>
       </c>
       <c r="D13" t="s">
-        <v>938</v>
+        <v>929</v>
       </c>
       <c r="E13">
         <v>100000000</v>
@@ -14322,30 +14191,21 @@
         <v>1732000000</v>
       </c>
       <c r="G13" t="s">
-        <v>895</v>
-      </c>
-      <c r="H13" t="s">
-        <v>896</v>
-      </c>
-      <c r="I13" t="s">
-        <v>897</v>
-      </c>
-      <c r="J13" t="s">
-        <v>920</v>
-      </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+        <v>911</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>196</v>
       </c>
       <c r="B14" t="s">
-        <v>921</v>
+        <v>912</v>
       </c>
       <c r="C14" t="s">
-        <v>954</v>
+        <v>945</v>
       </c>
       <c r="D14" t="s">
-        <v>939</v>
+        <v>930</v>
       </c>
       <c r="E14">
         <v>100000000</v>
@@ -14354,30 +14214,21 @@
         <v>106000000</v>
       </c>
       <c r="G14" t="s">
-        <v>895</v>
-      </c>
-      <c r="H14" t="s">
-        <v>896</v>
-      </c>
-      <c r="I14" t="s">
-        <v>897</v>
-      </c>
-      <c r="J14" t="s">
-        <v>922</v>
-      </c>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>193</v>
       </c>
       <c r="B15" t="s">
-        <v>923</v>
+        <v>914</v>
       </c>
       <c r="C15" t="s">
-        <v>955</v>
+        <v>946</v>
       </c>
       <c r="D15" t="s">
-        <v>940</v>
+        <v>931</v>
       </c>
       <c r="E15">
         <v>100000000</v>
@@ -14386,30 +14237,21 @@
         <v>300000000</v>
       </c>
       <c r="G15" t="s">
-        <v>895</v>
-      </c>
-      <c r="H15" t="s">
-        <v>896</v>
-      </c>
-      <c r="I15" t="s">
-        <v>897</v>
-      </c>
-      <c r="J15" t="s">
-        <v>924</v>
-      </c>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+        <v>915</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>519</v>
       </c>
       <c r="B16" t="s">
-        <v>925</v>
+        <v>916</v>
       </c>
       <c r="C16" t="s">
-        <v>956</v>
+        <v>947</v>
       </c>
       <c r="D16" t="s">
-        <v>942</v>
+        <v>933</v>
       </c>
       <c r="E16">
         <v>100000000</v>
@@ -14418,30 +14260,21 @@
         <v>300000000</v>
       </c>
       <c r="G16" t="s">
-        <v>895</v>
-      </c>
-      <c r="H16" t="s">
-        <v>896</v>
-      </c>
-      <c r="I16" t="s">
-        <v>897</v>
-      </c>
-      <c r="J16" t="s">
-        <v>926</v>
-      </c>
-    </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>250</v>
       </c>
       <c r="B17" t="s">
-        <v>927</v>
+        <v>918</v>
       </c>
       <c r="C17" t="s">
-        <v>957</v>
+        <v>948</v>
       </c>
       <c r="D17" t="s">
-        <v>941</v>
+        <v>932</v>
       </c>
       <c r="E17">
         <v>100000000</v>
@@ -14450,16 +14283,7 @@
         <v>300000000</v>
       </c>
       <c r="G17" t="s">
-        <v>895</v>
-      </c>
-      <c r="H17" t="s">
-        <v>896</v>
-      </c>
-      <c r="I17" t="s">
-        <v>897</v>
-      </c>
-      <c r="J17" t="s">
-        <v>928</v>
+        <v>919</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Conclusión de Temporada 9 y adición de Atlético de Madrid (17 equipos)
</commit_message>
<xml_diff>
--- a/lmi temp 9.xlsx
+++ b/lmi temp 9.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex1\Downloads\LMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D0F0073-D0F0-4BCF-B708-907E7BD55C8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB10F719-EDF4-4F33-B664-DBFDE771809E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1399" uniqueCount="957">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1424" uniqueCount="980">
   <si>
     <t>Equipo</t>
   </si>
@@ -900,9 +900,6 @@
     <t>Final</t>
   </si>
   <si>
-    <t>Por jugar</t>
-  </si>
-  <si>
     <t>Terengganu</t>
   </si>
   <si>
@@ -2760,9 +2757,6 @@
     <t>Etihad Stadium</t>
   </si>
   <si>
-    <t>Logos Equipos/city.webp</t>
-  </si>
-  <si>
     <t>LI Alejandro Balde</t>
   </si>
   <si>
@@ -2953,6 +2947,81 @@
   </si>
   <si>
     <t>DC Gonzalo García</t>
+  </si>
+  <si>
+    <t>Atletico de Madrid</t>
+  </si>
+  <si>
+    <t>PT Luis Malagon</t>
+  </si>
+  <si>
+    <t>LD Jonathan Clauss</t>
+  </si>
+  <si>
+    <t>LD Mateo Ponte</t>
+  </si>
+  <si>
+    <t>LI Salvador Reyes</t>
+  </si>
+  <si>
+    <t>CT Stefan de Vrij</t>
+  </si>
+  <si>
+    <t>CT Perr Schuurs</t>
+  </si>
+  <si>
+    <t>CT Rafael Márquez</t>
+  </si>
+  <si>
+    <t>CT Jesús Orozco</t>
+  </si>
+  <si>
+    <t>MCD Mateo Kovacic</t>
+  </si>
+  <si>
+    <t>MP Calvin Stengs</t>
+  </si>
+  <si>
+    <t>ED Angel Correa</t>
+  </si>
+  <si>
+    <t>ED Roberto Alvarado</t>
+  </si>
+  <si>
+    <t>EI Brian Rodríguez</t>
+  </si>
+  <si>
+    <t>ID Alex Zendejas</t>
+  </si>
+  <si>
+    <t>ID Samuel Chukwueze</t>
+  </si>
+  <si>
+    <t>SD Yoshinori Muto</t>
+  </si>
+  <si>
+    <t>DC Martin Terrier</t>
+  </si>
+  <si>
+    <t>DC Álvaro Morata</t>
+  </si>
+  <si>
+    <t>DC Tammy Abraham</t>
+  </si>
+  <si>
+    <t>ATM</t>
+  </si>
+  <si>
+    <t>Cívitas Metropolitano</t>
+  </si>
+  <si>
+    <t>Fernando</t>
+  </si>
+  <si>
+    <t>Logos Equipos/manchestercity.png</t>
+  </si>
+  <si>
+    <t>Logos Equipos/atleticomadrid.webp</t>
   </si>
 </sst>
 </file>
@@ -7912,11 +7981,17 @@
       <c r="B8" t="s">
         <v>56</v>
       </c>
+      <c r="C8">
+        <v>3</v>
+      </c>
       <c r="D8" t="s">
         <v>28</v>
       </c>
+      <c r="E8">
+        <v>4</v>
+      </c>
       <c r="F8" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -7978,7 +8053,7 @@
         <v>266</v>
       </c>
       <c r="B3" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -8041,13 +8116,13 @@
         <v>28</v>
       </c>
       <c r="C6" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D6" t="s">
         <v>61</v>
       </c>
       <c r="E6" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F6" t="s">
         <v>265</v>
@@ -8156,7 +8231,7 @@
         <v>86</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="6">
@@ -8168,7 +8243,7 @@
         <v>52</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C5" s="6"/>
       <c r="D5" s="6">
@@ -8191,10 +8266,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>278</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>279</v>
       </c>
       <c r="C7" s="6">
         <v>11</v>
@@ -8222,7 +8297,7 @@
         <v>121</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C9" s="6"/>
       <c r="D9" s="6">
@@ -8234,7 +8309,7 @@
         <v>48</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="6">
@@ -8246,7 +8321,7 @@
         <v>52</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C11" s="6"/>
       <c r="D11" s="6">
@@ -8282,7 +8357,7 @@
         <v>121</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="C14" s="6">
         <v>9</v>
@@ -8294,7 +8369,7 @@
         <v>134</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C15" s="6">
         <v>9</v>
@@ -10679,7 +10754,7 @@
         <v>86</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C4" s="6">
         <v>1</v>
@@ -10707,7 +10782,7 @@
         <v>86</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="6">
@@ -10759,7 +10834,7 @@
         <v>84</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C10" s="6">
         <v>3</v>
@@ -10773,7 +10848,7 @@
         <v>84</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C11" s="6">
         <v>2</v>
@@ -10787,7 +10862,7 @@
         <v>93</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="C12" s="6">
         <v>2</v>
@@ -10801,7 +10876,7 @@
         <v>134</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C13" s="6">
         <v>1</v>
@@ -10815,7 +10890,7 @@
         <v>86</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C14" s="6">
         <v>1</v>
@@ -10829,7 +10904,7 @@
         <v>43</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C15" s="6">
         <v>1</v>
@@ -10857,7 +10932,7 @@
         <v>43</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="C17" s="6">
         <v>1</v>
@@ -10871,7 +10946,7 @@
         <v>86</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C18" s="6">
         <v>1</v>
@@ -10885,7 +10960,7 @@
         <v>95</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C19" s="6">
         <v>1</v>
@@ -10911,7 +10986,7 @@
         <v>134</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="6">
@@ -10920,10 +10995,10 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="B22" s="6" t="s">
         <v>297</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>298</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="6">
@@ -10932,10 +11007,10 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="6" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="C23" s="6"/>
       <c r="D23" s="6">
@@ -10944,10 +11019,10 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="6" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="6">
@@ -10959,7 +11034,7 @@
         <v>95</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="6">
@@ -10971,7 +11046,7 @@
         <v>93</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="6">
@@ -10995,7 +11070,7 @@
         <v>48</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="6">
@@ -11019,7 +11094,7 @@
         <v>84</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="6">
@@ -11055,7 +11130,7 @@
         <v>95</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C33" s="6"/>
       <c r="D33" s="6">
@@ -11079,7 +11154,7 @@
         <v>134</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="C35" s="6">
         <v>3</v>
@@ -11088,10 +11163,10 @@
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="6" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C36" s="6">
         <v>2</v>
@@ -11103,7 +11178,7 @@
         <v>86</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C37" s="6">
         <v>2</v>
@@ -11127,7 +11202,7 @@
         <v>93</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="C39" s="6">
         <v>2</v>
@@ -11139,7 +11214,7 @@
         <v>86</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C40" s="6">
         <v>2</v>
@@ -11151,7 +11226,7 @@
         <v>86</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C41" s="6">
         <v>2</v>
@@ -11172,10 +11247,10 @@
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="6" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C43" s="6">
         <v>1</v>
@@ -11187,7 +11262,7 @@
         <v>117</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C44" s="6">
         <v>1</v>
@@ -11247,7 +11322,7 @@
         <v>84</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="C49" s="6">
         <v>1</v>
@@ -11259,7 +11334,7 @@
         <v>125</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C50" s="6">
         <v>1</v>
@@ -11295,7 +11370,7 @@
         <v>95</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C53" s="6">
         <v>1</v>
@@ -11319,7 +11394,7 @@
         <v>95</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C55" s="6">
         <v>1</v>
@@ -11405,13 +11480,13 @@
         <v>84</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="N1" s="3" t="s">
         <v>107</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>888</v>
+        <v>887</v>
       </c>
       <c r="P1" s="3" t="s">
         <v>76</v>
@@ -11419,302 +11494,302 @@
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="B2" s="5" t="s">
         <v>317</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="9" t="s">
         <v>318</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="D2" s="10" t="s">
         <v>319</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="E2" s="5" t="s">
         <v>320</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>322</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>325</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>327</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="M2" s="11" t="s">
         <v>328</v>
       </c>
-      <c r="M2" s="11" t="s">
+      <c r="N2" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" s="3" t="s">
+        <v>867</v>
+      </c>
+      <c r="P2" s="3" t="s">
         <v>330</v>
-      </c>
-      <c r="O2" s="3" t="s">
-        <v>868</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>332</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="9" t="s">
         <v>333</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="10" t="s">
         <v>334</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>335</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>123</v>
       </c>
       <c r="F3" s="3" t="s">
+        <v>335</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>341</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="M3" s="11" t="s">
         <v>342</v>
       </c>
-      <c r="M3" s="11" t="s">
+      <c r="N3" s="3" t="s">
+        <v>859</v>
+      </c>
+      <c r="O3" s="3" t="s">
+        <v>868</v>
+      </c>
+      <c r="P3" s="3" t="s">
         <v>343</v>
-      </c>
-      <c r="N3" s="3" t="s">
-        <v>860</v>
-      </c>
-      <c r="O3" s="3" t="s">
-        <v>869</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>345</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="9" t="s">
         <v>346</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="D4" s="10" t="s">
         <v>347</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="E4" s="5" t="s">
         <v>348</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="F4" s="3" t="s">
         <v>349</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>350</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
         <v>352</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>353</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>354</v>
       </c>
       <c r="K4" s="3" t="s">
         <v>212</v>
       </c>
       <c r="L4" s="3" t="s">
+        <v>354</v>
+      </c>
+      <c r="M4" s="11" t="s">
         <v>355</v>
       </c>
-      <c r="M4" s="11" t="s">
+      <c r="N4" s="3" t="s">
         <v>356</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="O4" s="3" t="s">
+        <v>869</v>
+      </c>
+      <c r="P4" s="3" t="s">
         <v>357</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>870</v>
-      </c>
-      <c r="P4" s="3" t="s">
-        <v>358</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>359</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="9" t="s">
         <v>360</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>361</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>197</v>
       </c>
       <c r="E5" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>362</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>363</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>257</v>
       </c>
       <c r="H5" s="3" t="s">
+        <v>363</v>
+      </c>
+      <c r="I5" s="3" t="s">
         <v>364</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="J5" s="3" t="s">
         <v>365</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="K5" s="3" t="s">
         <v>366</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="L5" s="3" t="s">
         <v>367</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="M5" s="11" t="s">
         <v>368</v>
       </c>
-      <c r="M5" s="11" t="s">
+      <c r="N5" s="3" t="s">
         <v>369</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="O5" s="3" t="s">
+        <v>870</v>
+      </c>
+      <c r="P5" s="3" t="s">
         <v>370</v>
-      </c>
-      <c r="O5" s="3" t="s">
-        <v>871</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B6" s="5" t="s">
         <v>217</v>
       </c>
       <c r="C6" s="9" t="s">
+        <v>372</v>
+      </c>
+      <c r="D6" s="10" t="s">
         <v>373</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="E6" s="5" t="s">
         <v>374</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="F6" s="3" t="s">
         <v>375</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="H6" s="3" t="s">
         <v>377</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="I6" s="3" t="s">
         <v>378</v>
       </c>
-      <c r="I6" s="3" t="s">
+      <c r="J6" s="3" t="s">
         <v>379</v>
       </c>
-      <c r="J6" s="3" t="s">
+      <c r="K6" s="3" t="s">
         <v>380</v>
       </c>
-      <c r="K6" s="3" t="s">
+      <c r="L6" s="3" t="s">
         <v>381</v>
       </c>
-      <c r="L6" s="3" t="s">
+      <c r="M6" s="11" t="s">
         <v>382</v>
       </c>
-      <c r="M6" s="11" t="s">
+      <c r="N6" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="N6" s="3" t="s">
+      <c r="O6" s="3" t="s">
+        <v>871</v>
+      </c>
+      <c r="P6" s="3" t="s">
         <v>384</v>
-      </c>
-      <c r="O6" s="3" t="s">
-        <v>872</v>
-      </c>
-      <c r="P6" s="3" t="s">
-        <v>385</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="C7" s="9" t="s">
         <v>386</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="D7" s="10" t="s">
         <v>387</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>388</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>203</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>183</v>
       </c>
       <c r="I7" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="J7" s="3" t="s">
         <v>390</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="K7" s="3" t="s">
         <v>391</v>
       </c>
-      <c r="K7" s="3" t="s">
+      <c r="L7" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="M7" s="11" t="s">
         <v>392</v>
       </c>
-      <c r="L7" s="3" t="s">
-        <v>304</v>
-      </c>
-      <c r="M7" s="11" t="s">
+      <c r="N7" s="3" t="s">
         <v>393</v>
       </c>
-      <c r="N7" s="3" t="s">
+      <c r="O7" s="3" t="s">
+        <v>872</v>
+      </c>
+      <c r="P7" s="3" t="s">
         <v>394</v>
-      </c>
-      <c r="O7" s="3" t="s">
-        <v>873</v>
-      </c>
-      <c r="P7" s="3" t="s">
-        <v>395</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
@@ -11725,107 +11800,107 @@
         <v>115</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>153</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F8" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>397</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="H8" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="J8" s="3" t="s">
         <v>398</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>293</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="J8" s="3" t="s">
+      <c r="K8" s="3" t="s">
+        <v>300</v>
+      </c>
+      <c r="L8" s="3" t="s">
         <v>399</v>
       </c>
-      <c r="K8" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="L8" s="3" t="s">
+      <c r="M8" s="11" t="s">
         <v>400</v>
       </c>
-      <c r="M8" s="11" t="s">
+      <c r="N8" s="3" t="s">
+        <v>860</v>
+      </c>
+      <c r="O8" s="3" t="s">
+        <v>873</v>
+      </c>
+      <c r="P8" s="3" t="s">
         <v>401</v>
-      </c>
-      <c r="N8" s="3" t="s">
-        <v>861</v>
-      </c>
-      <c r="O8" s="3" t="s">
-        <v>874</v>
-      </c>
-      <c r="P8" s="3" t="s">
-        <v>402</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="B9" s="5" t="s">
         <v>106</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>102</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G9" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>405</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="L9" s="3" t="s">
         <v>312</v>
       </c>
-      <c r="H9" s="3" t="s">
-        <v>404</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>405</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>406</v>
-      </c>
-      <c r="K9" s="3" t="s">
+      <c r="M9" s="11" t="s">
         <v>407</v>
       </c>
-      <c r="L9" s="3" t="s">
-        <v>313</v>
-      </c>
-      <c r="M9" s="11" t="s">
+      <c r="N9" s="3" t="s">
         <v>408</v>
       </c>
-      <c r="N9" s="3" t="s">
+      <c r="O9" s="3" t="s">
+        <v>874</v>
+      </c>
+      <c r="P9" s="3" t="s">
         <v>409</v>
-      </c>
-      <c r="O9" s="3" t="s">
-        <v>875</v>
-      </c>
-      <c r="P9" s="3" t="s">
-        <v>410</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
+        <v>410</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="B10" s="5" t="s">
-        <v>412</v>
-      </c>
       <c r="C10" s="9" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>148</v>
@@ -11834,37 +11909,37 @@
         <v>155</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G10" s="3" t="s">
+        <v>412</v>
+      </c>
+      <c r="H10" s="3" t="s">
         <v>413</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="I10" s="3" t="s">
         <v>414</v>
       </c>
-      <c r="I10" s="3" t="s">
+      <c r="J10" s="3" t="s">
         <v>415</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>416</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>166</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="M10" s="11" t="s">
+        <v>416</v>
+      </c>
+      <c r="N10" s="3" t="s">
         <v>417</v>
       </c>
-      <c r="N10" s="3" t="s">
+      <c r="O10" s="3" t="s">
+        <v>875</v>
+      </c>
+      <c r="P10" s="3" t="s">
         <v>418</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>876</v>
-      </c>
-      <c r="P10" s="3" t="s">
-        <v>419</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.3">
@@ -11875,7 +11950,7 @@
         <v>92</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>100</v>
@@ -11884,48 +11959,48 @@
         <v>216</v>
       </c>
       <c r="F11" s="3" t="s">
+        <v>419</v>
+      </c>
+      <c r="G11" s="3" t="s">
         <v>420</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="H11" s="3" t="s">
         <v>421</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="I11" s="3" t="s">
         <v>422</v>
-      </c>
-      <c r="I11" s="3" t="s">
-        <v>423</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>215</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>101</v>
       </c>
       <c r="M11" s="11" t="s">
+        <v>423</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>861</v>
+      </c>
+      <c r="O11" s="3" t="s">
+        <v>876</v>
+      </c>
+      <c r="P11" s="3" t="s">
         <v>424</v>
-      </c>
-      <c r="N11" s="3" t="s">
-        <v>862</v>
-      </c>
-      <c r="O11" s="3" t="s">
-        <v>877</v>
-      </c>
-      <c r="P11" s="3" t="s">
-        <v>425</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="B12" s="5" t="s">
         <v>171</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>104</v>
@@ -11934,148 +12009,148 @@
         <v>225</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="I12" s="3" t="s">
         <v>132</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
       <c r="K12" s="3" t="s">
         <v>165</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="M12" s="11" t="s">
+        <v>427</v>
+      </c>
+      <c r="N12" s="3" t="s">
+        <v>862</v>
+      </c>
+      <c r="O12" s="3" t="s">
+        <v>877</v>
+      </c>
+      <c r="P12" s="3" t="s">
         <v>428</v>
-      </c>
-      <c r="N12" s="3" t="s">
-        <v>863</v>
-      </c>
-      <c r="O12" s="3" t="s">
-        <v>878</v>
-      </c>
-      <c r="P12" s="3" t="s">
-        <v>429</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>430</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="9" t="s">
         <v>431</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="D13" s="10" t="s">
         <v>432</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="E13" s="5" t="s">
         <v>433</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="F13" s="3" t="s">
         <v>434</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>435</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="H13" s="3" t="s">
         <v>436</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="I13" s="3" t="s">
         <v>437</v>
       </c>
-      <c r="I13" s="3" t="s">
+      <c r="J13" s="3" t="s">
         <v>438</v>
       </c>
-      <c r="J13" s="3" t="s">
+      <c r="K13" s="3" t="s">
         <v>439</v>
       </c>
-      <c r="K13" s="3" t="s">
+      <c r="L13" s="3" t="s">
         <v>440</v>
       </c>
-      <c r="L13" s="3" t="s">
+      <c r="M13" s="11" t="s">
         <v>441</v>
       </c>
-      <c r="M13" s="11" t="s">
+      <c r="N13" s="3" t="s">
+        <v>863</v>
+      </c>
+      <c r="O13" s="3" t="s">
+        <v>878</v>
+      </c>
+      <c r="P13" s="3" t="s">
         <v>442</v>
-      </c>
-      <c r="N13" s="3" t="s">
-        <v>864</v>
-      </c>
-      <c r="O13" s="3" t="s">
-        <v>879</v>
-      </c>
-      <c r="P13" s="3" t="s">
-        <v>443</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
+        <v>443</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>444</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="9" t="s">
         <v>445</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="D14" s="10" t="s">
         <v>446</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="E14" s="5" t="s">
         <v>447</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="F14" s="3" t="s">
         <v>448</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="3" t="s">
         <v>449</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="H14" s="3" t="s">
         <v>450</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="I14" s="3" t="s">
         <v>451</v>
       </c>
-      <c r="I14" s="3" t="s">
+      <c r="J14" s="3" t="s">
         <v>452</v>
       </c>
-      <c r="J14" s="3" t="s">
+      <c r="K14" s="3" t="s">
         <v>453</v>
       </c>
-      <c r="K14" s="3" t="s">
+      <c r="L14" s="3" t="s">
         <v>454</v>
       </c>
-      <c r="L14" s="3" t="s">
+      <c r="M14" s="11" t="s">
         <v>455</v>
       </c>
-      <c r="M14" s="11" t="s">
+      <c r="N14" s="3" t="s">
+        <v>864</v>
+      </c>
+      <c r="O14" s="3" t="s">
+        <v>879</v>
+      </c>
+      <c r="P14" s="3" t="s">
         <v>456</v>
-      </c>
-      <c r="N14" s="3" t="s">
-        <v>865</v>
-      </c>
-      <c r="O14" s="3" t="s">
-        <v>880</v>
-      </c>
-      <c r="P14" s="3" t="s">
-        <v>457</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
+        <v>457</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>458</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="9" t="s">
         <v>459</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>460</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>206</v>
@@ -12084,7 +12159,7 @@
         <v>245</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>256</v>
@@ -12093,189 +12168,189 @@
         <v>131</v>
       </c>
       <c r="I15" s="3" t="s">
+        <v>461</v>
+      </c>
+      <c r="J15" s="3" t="s">
         <v>462</v>
       </c>
-      <c r="J15" s="3" t="s">
+      <c r="K15" s="3" t="s">
         <v>463</v>
       </c>
-      <c r="K15" s="3" t="s">
+      <c r="L15" s="3" t="s">
         <v>464</v>
       </c>
-      <c r="L15" s="3" t="s">
+      <c r="M15" s="11" t="s">
         <v>465</v>
       </c>
-      <c r="M15" s="11" t="s">
+      <c r="N15" s="3" t="s">
+        <v>865</v>
+      </c>
+      <c r="O15" s="3" t="s">
+        <v>880</v>
+      </c>
+      <c r="P15" s="3" t="s">
         <v>466</v>
-      </c>
-      <c r="N15" s="3" t="s">
-        <v>866</v>
-      </c>
-      <c r="O15" s="3" t="s">
-        <v>881</v>
-      </c>
-      <c r="P15" s="3" t="s">
-        <v>467</v>
       </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>468</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="9" t="s">
         <v>469</v>
       </c>
-      <c r="C16" s="9" t="s">
-        <v>470</v>
-      </c>
       <c r="D16" s="10" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>186</v>
       </c>
       <c r="F16" s="3" t="s">
+        <v>472</v>
+      </c>
+      <c r="G16" s="3" t="s">
         <v>473</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>474</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>221</v>
       </c>
       <c r="I16" s="3" t="s">
+        <v>474</v>
+      </c>
+      <c r="J16" s="3" t="s">
         <v>475</v>
       </c>
-      <c r="J16" s="3" t="s">
+      <c r="K16" s="3" t="s">
         <v>476</v>
       </c>
-      <c r="K16" s="3" t="s">
+      <c r="L16" s="3" t="s">
         <v>477</v>
       </c>
-      <c r="L16" s="3" t="s">
+      <c r="M16" s="11" t="s">
         <v>478</v>
       </c>
-      <c r="M16" s="11" t="s">
+      <c r="N16" s="3" t="s">
+        <v>866</v>
+      </c>
+      <c r="O16" s="3" t="s">
+        <v>881</v>
+      </c>
+      <c r="P16" s="3" t="s">
         <v>479</v>
-      </c>
-      <c r="N16" s="3" t="s">
-        <v>867</v>
-      </c>
-      <c r="O16" s="3" t="s">
-        <v>882</v>
-      </c>
-      <c r="P16" s="3" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="17" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>481</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="9" t="s">
         <v>482</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>483</v>
       </c>
       <c r="D17" s="10" t="s">
         <v>213</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="F17" s="3" t="s">
         <v>194</v>
       </c>
       <c r="G17" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="H17" s="3" t="s">
         <v>484</v>
       </c>
-      <c r="H17" s="3" t="s">
+      <c r="I17" s="3" t="s">
         <v>485</v>
       </c>
-      <c r="I17" s="3" t="s">
+      <c r="J17" s="3" t="s">
         <v>486</v>
       </c>
-      <c r="J17" s="3" t="s">
+      <c r="K17" s="3" t="s">
         <v>487</v>
       </c>
-      <c r="K17" s="3" t="s">
+      <c r="L17" s="3" t="s">
         <v>488</v>
       </c>
-      <c r="L17" s="3" t="s">
+      <c r="M17" s="11" t="s">
         <v>489</v>
       </c>
-      <c r="M17" s="11" t="s">
+      <c r="N17" s="3" t="s">
         <v>490</v>
       </c>
-      <c r="N17" s="3" t="s">
+      <c r="O17" s="3" t="s">
+        <v>882</v>
+      </c>
+      <c r="P17" s="3" t="s">
         <v>491</v>
-      </c>
-      <c r="O17" s="3" t="s">
-        <v>883</v>
-      </c>
-      <c r="P17" s="3" t="s">
-        <v>492</v>
       </c>
     </row>
     <row r="18" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
+        <v>492</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>493</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>494</v>
       </c>
       <c r="C18" s="9" t="s">
         <v>253</v>
       </c>
       <c r="D18" s="10" t="s">
+        <v>494</v>
+      </c>
+      <c r="E18" s="5" t="s">
         <v>495</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>496</v>
       </c>
       <c r="F18" s="3" t="s">
         <v>252</v>
       </c>
       <c r="G18" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="H18" s="3" t="s">
         <v>497</v>
       </c>
-      <c r="H18" s="3" t="s">
+      <c r="I18" s="3" t="s">
         <v>498</v>
       </c>
-      <c r="I18" s="3" t="s">
+      <c r="J18" s="3" t="s">
         <v>499</v>
       </c>
-      <c r="J18" s="3" t="s">
+      <c r="K18" s="3" t="s">
+        <v>315</v>
+      </c>
+      <c r="L18" s="3" t="s">
         <v>500</v>
       </c>
-      <c r="K18" s="3" t="s">
-        <v>316</v>
-      </c>
-      <c r="L18" s="3" t="s">
+      <c r="M18" s="11" t="s">
         <v>501</v>
       </c>
-      <c r="M18" s="11" t="s">
+      <c r="N18" s="3" t="s">
         <v>502</v>
       </c>
-      <c r="N18" s="3" t="s">
+      <c r="O18" s="3" t="s">
+        <v>883</v>
+      </c>
+      <c r="P18" s="3" t="s">
         <v>503</v>
-      </c>
-      <c r="O18" s="3" t="s">
-        <v>884</v>
-      </c>
-      <c r="P18" s="3" t="s">
-        <v>504</v>
       </c>
     </row>
     <row r="19" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>184</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="D19" s="10" t="s">
         <v>178</v>
@@ -12287,45 +12362,45 @@
         <v>219</v>
       </c>
       <c r="G19" s="3" t="s">
+        <v>506</v>
+      </c>
+      <c r="H19" s="3" t="s">
         <v>507</v>
       </c>
-      <c r="H19" s="3" t="s">
+      <c r="I19" s="3" t="s">
         <v>508</v>
       </c>
-      <c r="I19" s="3" t="s">
+      <c r="J19" s="3" t="s">
         <v>509</v>
-      </c>
-      <c r="J19" s="3" t="s">
-        <v>510</v>
       </c>
       <c r="K19" s="3" t="s">
         <v>254</v>
       </c>
       <c r="L19" s="3" t="s">
+        <v>510</v>
+      </c>
+      <c r="M19" s="11" t="s">
         <v>511</v>
       </c>
-      <c r="M19" s="11" t="s">
+      <c r="N19" s="3" t="s">
         <v>512</v>
       </c>
-      <c r="N19" s="3" t="s">
+      <c r="O19" s="3" t="s">
+        <v>884</v>
+      </c>
+      <c r="P19" s="3" t="s">
         <v>513</v>
-      </c>
-      <c r="O19" s="3" t="s">
-        <v>885</v>
-      </c>
-      <c r="P19" s="3" t="s">
-        <v>514</v>
       </c>
     </row>
     <row r="20" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
+        <v>514</v>
+      </c>
+      <c r="B20" s="5" t="s">
         <v>515</v>
       </c>
-      <c r="B20" s="5" t="s">
-        <v>516</v>
-      </c>
       <c r="C20" s="9" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>214</v>
@@ -12334,19 +12409,19 @@
         <v>116</v>
       </c>
       <c r="F20" s="3" t="s">
+        <v>516</v>
+      </c>
+      <c r="G20" s="3" t="s">
         <v>517</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>518</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>218</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="K20" s="3" t="s">
         <v>160</v>
@@ -12355,96 +12430,96 @@
         <v>220</v>
       </c>
       <c r="M20" s="11" t="s">
+        <v>519</v>
+      </c>
+      <c r="N20" s="3" t="s">
+        <v>856</v>
+      </c>
+      <c r="O20" s="3" t="s">
+        <v>885</v>
+      </c>
+      <c r="P20" s="3" t="s">
         <v>520</v>
-      </c>
-      <c r="N20" s="3" t="s">
-        <v>857</v>
-      </c>
-      <c r="O20" s="3" t="s">
-        <v>886</v>
-      </c>
-      <c r="P20" s="3" t="s">
-        <v>521</v>
       </c>
     </row>
     <row r="21" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>113</v>
       </c>
       <c r="C21" s="9" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="E21" s="5" t="s">
         <v>114</v>
       </c>
       <c r="F21" s="3" t="s">
+        <v>523</v>
+      </c>
+      <c r="G21" s="3" t="s">
         <v>524</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>525</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>156</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="L21" s="3" t="s">
         <v>192</v>
       </c>
       <c r="M21" s="11" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="N21" s="3" t="s">
-        <v>858</v>
+        <v>857</v>
       </c>
       <c r="O21" s="3"/>
       <c r="P21" s="3" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
     </row>
     <row r="22" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
+        <v>528</v>
+      </c>
+      <c r="B22" s="5" t="s">
         <v>529</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="C22" s="9" t="s">
         <v>530</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="D22" s="10" t="s">
         <v>531</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>532</v>
       </c>
       <c r="E22" s="5" t="s">
         <v>176</v>
       </c>
       <c r="F22" s="3" t="s">
+        <v>532</v>
+      </c>
+      <c r="G22" s="3" t="s">
         <v>533</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>534</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>173</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="K22" s="3" t="s">
         <v>232</v>
@@ -12453,62 +12528,62 @@
         <v>88</v>
       </c>
       <c r="M22" s="11" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="N22" s="3" t="s">
-        <v>859</v>
+        <v>858</v>
       </c>
       <c r="O22" s="3"/>
       <c r="P22" s="3" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
     </row>
     <row r="23" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
+        <v>536</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>537</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="C23" s="9" t="s">
+        <v>307</v>
+      </c>
+      <c r="D23" s="10" t="s">
         <v>538</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>308</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>539</v>
       </c>
       <c r="E23" s="5" t="s">
         <v>112</v>
       </c>
       <c r="F23" s="3" t="s">
+        <v>539</v>
+      </c>
+      <c r="G23" s="3" t="s">
         <v>540</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>541</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>255</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="J23" s="3" t="s">
         <v>111</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="L23" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="M23" s="11" t="s">
         <v>543</v>
       </c>
-      <c r="M23" s="11" t="s">
-        <v>544</v>
-      </c>
       <c r="N23" s="3" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="O23" s="3"/>
       <c r="P23" s="3" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
     </row>
     <row r="24" spans="1:16" x14ac:dyDescent="0.3">
@@ -12516,7 +12591,7 @@
         <v>177</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>142</v>
@@ -12528,10 +12603,10 @@
         <v>222</v>
       </c>
       <c r="F24" s="3" t="s">
+        <v>546</v>
+      </c>
+      <c r="G24" s="3" t="s">
         <v>547</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>548</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>170</v>
@@ -12540,21 +12615,21 @@
         <v>238</v>
       </c>
       <c r="J24" s="3" t="s">
+        <v>548</v>
+      </c>
+      <c r="K24" s="3" t="s">
         <v>549</v>
-      </c>
-      <c r="K24" s="3" t="s">
-        <v>550</v>
       </c>
       <c r="L24" s="3" t="s">
         <v>250</v>
       </c>
       <c r="M24" s="11" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="N24" s="3"/>
       <c r="O24" s="3"/>
       <c r="P24" s="3" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
     </row>
   </sheetData>
@@ -12631,1213 +12706,1253 @@
         <v>71</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="P1" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="Q1" s="3"/>
+      <c r="Q1" s="3" t="s">
+        <v>955</v>
+      </c>
       <c r="R1" s="3"/>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
+        <v>552</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>553</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>554</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>555</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>556</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>557</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>558</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>559</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
+        <v>935</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>901</v>
+      </c>
+      <c r="K2" s="3" t="s">
         <v>560</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>937</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>903</v>
-      </c>
-      <c r="K2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>561</v>
       </c>
-      <c r="L2" s="3" t="s">
+      <c r="M2" s="3" t="s">
         <v>562</v>
       </c>
-      <c r="M2" s="3" t="s">
+      <c r="N2" s="3" t="s">
         <v>563</v>
       </c>
-      <c r="N2" s="3" t="s">
+      <c r="O2" s="3" t="s">
+        <v>915</v>
+      </c>
+      <c r="P2" s="3" t="s">
         <v>564</v>
       </c>
-      <c r="O2" s="3" t="s">
-        <v>917</v>
-      </c>
-      <c r="P2" s="3" t="s">
-        <v>565</v>
-      </c>
-      <c r="Q2" s="3"/>
+      <c r="Q2" s="3" t="s">
+        <v>956</v>
+      </c>
       <c r="R2" s="3"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
+        <v>565</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>566</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>567</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>568</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>569</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>570</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>571</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>572</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
+        <v>891</v>
+      </c>
+      <c r="J3" s="3" t="s">
         <v>573</v>
       </c>
-      <c r="I3" s="3" t="s">
-        <v>893</v>
-      </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="3" t="s">
         <v>574</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="L3" s="3" t="s">
         <v>575</v>
       </c>
-      <c r="L3" s="3" t="s">
+      <c r="M3" s="3" t="s">
         <v>576</v>
       </c>
-      <c r="M3" s="3" t="s">
+      <c r="N3" s="3" t="s">
         <v>577</v>
       </c>
-      <c r="N3" s="3" t="s">
+      <c r="O3" s="3" t="s">
+        <v>916</v>
+      </c>
+      <c r="P3" s="3" t="s">
         <v>578</v>
       </c>
-      <c r="O3" s="3" t="s">
-        <v>918</v>
-      </c>
-      <c r="P3" s="3" t="s">
-        <v>579</v>
-      </c>
-      <c r="Q3" s="3"/>
+      <c r="Q3" s="3" t="s">
+        <v>957</v>
+      </c>
       <c r="R3" s="3"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
+        <v>579</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>580</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>581</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>582</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="E4" s="3" t="s">
         <v>583</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="3" t="s">
         <v>584</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>585</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>586</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="I4" s="3" t="s">
+        <v>936</v>
+      </c>
+      <c r="J4" s="3" t="s">
         <v>587</v>
       </c>
-      <c r="I4" s="3" t="s">
-        <v>938</v>
-      </c>
-      <c r="J4" s="3" t="s">
+      <c r="K4" s="3" t="s">
         <v>588</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="L4" s="3" t="s">
         <v>589</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="M4" s="3" t="s">
         <v>590</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="N4" s="3" t="s">
         <v>591</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="O4" s="3" t="s">
+        <v>917</v>
+      </c>
+      <c r="P4" s="3" t="s">
         <v>592</v>
       </c>
-      <c r="O4" s="3" t="s">
-        <v>919</v>
-      </c>
-      <c r="P4" s="3" t="s">
-        <v>593</v>
-      </c>
-      <c r="Q4" s="3"/>
+      <c r="Q4" s="3" t="s">
+        <v>958</v>
+      </c>
       <c r="R4" s="3"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
+        <v>593</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>594</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>595</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>596</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>597</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>598</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>599</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="H5" s="3" t="s">
         <v>600</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="I5" s="3" t="s">
+        <v>937</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>902</v>
+      </c>
+      <c r="K5" s="3" t="s">
         <v>601</v>
       </c>
-      <c r="I5" s="3" t="s">
-        <v>939</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>904</v>
-      </c>
-      <c r="K5" s="3" t="s">
+      <c r="L5" s="3" t="s">
         <v>602</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="M5" s="3" t="s">
         <v>603</v>
       </c>
-      <c r="M5" s="3" t="s">
+      <c r="N5" s="3" t="s">
         <v>604</v>
       </c>
-      <c r="N5" s="3" t="s">
+      <c r="O5" s="3" t="s">
+        <v>888</v>
+      </c>
+      <c r="P5" s="3" t="s">
         <v>605</v>
       </c>
-      <c r="O5" s="3" t="s">
-        <v>889</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>606</v>
-      </c>
-      <c r="Q5" s="3"/>
+      <c r="Q5" s="3" t="s">
+        <v>959</v>
+      </c>
       <c r="R5" s="3"/>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
+        <v>606</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>607</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>608</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>609</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="E6" s="3" t="s">
         <v>610</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>611</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>612</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="H6" s="3" t="s">
         <v>613</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="I6" s="3" t="s">
+        <v>938</v>
+      </c>
+      <c r="J6" s="3" t="s">
         <v>614</v>
       </c>
-      <c r="I6" s="3" t="s">
-        <v>940</v>
-      </c>
-      <c r="J6" s="3" t="s">
+      <c r="K6" s="3" t="s">
         <v>615</v>
       </c>
-      <c r="K6" s="3" t="s">
+      <c r="L6" s="3" t="s">
         <v>616</v>
       </c>
-      <c r="L6" s="3" t="s">
+      <c r="M6" s="3" t="s">
+        <v>906</v>
+      </c>
+      <c r="N6" s="3" t="s">
         <v>617</v>
       </c>
-      <c r="M6" s="3" t="s">
-        <v>908</v>
-      </c>
-      <c r="N6" s="3" t="s">
+      <c r="O6" s="3" t="s">
+        <v>918</v>
+      </c>
+      <c r="P6" s="3" t="s">
         <v>618</v>
       </c>
-      <c r="O6" s="3" t="s">
-        <v>920</v>
-      </c>
-      <c r="P6" s="3" t="s">
-        <v>619</v>
-      </c>
-      <c r="Q6" s="3"/>
+      <c r="Q6" s="3" t="s">
+        <v>960</v>
+      </c>
       <c r="R6" s="3"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
+        <v>619</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>620</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>621</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>622</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>623</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="3" t="s">
         <v>624</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
         <v>625</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>626</v>
-      </c>
       <c r="H7" s="3" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>941</v>
+        <v>939</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>905</v>
+        <v>903</v>
       </c>
       <c r="K7" s="3" t="s">
+        <v>627</v>
+      </c>
+      <c r="L7" s="3" t="s">
         <v>628</v>
       </c>
-      <c r="L7" s="3" t="s">
+      <c r="M7" s="3" t="s">
         <v>629</v>
       </c>
-      <c r="M7" s="3" t="s">
+      <c r="N7" s="3" t="s">
         <v>630</v>
       </c>
-      <c r="N7" s="3" t="s">
+      <c r="O7" s="3" t="s">
+        <v>919</v>
+      </c>
+      <c r="P7" s="3" t="s">
         <v>631</v>
       </c>
-      <c r="O7" s="3" t="s">
-        <v>921</v>
-      </c>
-      <c r="P7" s="3" t="s">
-        <v>632</v>
-      </c>
-      <c r="Q7" s="3"/>
+      <c r="Q7" s="3" t="s">
+        <v>961</v>
+      </c>
       <c r="R7" s="3"/>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
+        <v>632</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>633</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>634</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>635</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3" t="s">
+        <v>897</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>636</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>899</v>
-      </c>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>637</v>
       </c>
-      <c r="G8" s="3" t="s">
+      <c r="H8" s="3" t="s">
         <v>638</v>
       </c>
-      <c r="H8" s="3" t="s">
+      <c r="I8" s="3" t="s">
+        <v>940</v>
+      </c>
+      <c r="J8" s="3" t="s">
         <v>639</v>
       </c>
-      <c r="I8" s="3" t="s">
-        <v>942</v>
-      </c>
-      <c r="J8" s="3" t="s">
+      <c r="K8" s="3" t="s">
         <v>640</v>
       </c>
-      <c r="K8" s="3" t="s">
+      <c r="L8" s="3" t="s">
         <v>641</v>
       </c>
-      <c r="L8" s="3" t="s">
+      <c r="M8" s="3" t="s">
         <v>642</v>
       </c>
-      <c r="M8" s="3" t="s">
+      <c r="N8" s="3" t="s">
         <v>643</v>
       </c>
-      <c r="N8" s="3" t="s">
+      <c r="O8" s="3" t="s">
+        <v>920</v>
+      </c>
+      <c r="P8" s="3" t="s">
         <v>644</v>
       </c>
-      <c r="O8" s="3" t="s">
-        <v>922</v>
-      </c>
-      <c r="P8" s="3" t="s">
-        <v>645</v>
-      </c>
-      <c r="Q8" s="3"/>
+      <c r="Q8" s="3" t="s">
+        <v>962</v>
+      </c>
       <c r="R8" s="3"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
+        <v>645</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>646</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>647</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>648</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="3" t="s">
         <v>649</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="F9" s="3" t="s">
         <v>650</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
         <v>651</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="H9" s="3" t="s">
         <v>652</v>
       </c>
-      <c r="H9" s="3" t="s">
+      <c r="I9" s="3" t="s">
+        <v>941</v>
+      </c>
+      <c r="J9" s="3" t="s">
         <v>653</v>
       </c>
-      <c r="I9" s="3" t="s">
-        <v>943</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>654</v>
-      </c>
       <c r="K9" s="3" t="s">
+        <v>655</v>
+      </c>
+      <c r="L9" s="3" t="s">
         <v>656</v>
       </c>
-      <c r="L9" s="3" t="s">
+      <c r="M9" s="3" t="s">
         <v>657</v>
       </c>
-      <c r="M9" s="3" t="s">
+      <c r="N9" s="3" t="s">
         <v>658</v>
       </c>
-      <c r="N9" s="3" t="s">
+      <c r="O9" s="3" t="s">
+        <v>921</v>
+      </c>
+      <c r="P9" s="3" t="s">
         <v>659</v>
       </c>
-      <c r="O9" s="3" t="s">
-        <v>923</v>
-      </c>
-      <c r="P9" s="3" t="s">
-        <v>660</v>
-      </c>
-      <c r="Q9" s="3"/>
+      <c r="Q9" s="3" t="s">
+        <v>963</v>
+      </c>
       <c r="R9" s="3"/>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
+        <v>660</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>661</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>662</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
         <v>663</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="E10" s="3" t="s">
         <v>664</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="F10" s="3" t="s">
         <v>665</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="G10" s="3" t="s">
         <v>666</v>
       </c>
-      <c r="G10" s="3" t="s">
+      <c r="H10" s="3" t="s">
         <v>667</v>
       </c>
-      <c r="H10" s="3" t="s">
+      <c r="I10" s="3" t="s">
+        <v>942</v>
+      </c>
+      <c r="J10" s="3" t="s">
         <v>668</v>
       </c>
-      <c r="I10" s="3" t="s">
-        <v>944</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>669</v>
-      </c>
       <c r="K10" s="3" t="s">
-        <v>906</v>
+        <v>904</v>
       </c>
       <c r="L10" s="3" t="s">
+        <v>670</v>
+      </c>
+      <c r="M10" s="3" t="s">
+        <v>907</v>
+      </c>
+      <c r="N10" s="3" t="s">
         <v>671</v>
       </c>
-      <c r="M10" s="3" t="s">
-        <v>909</v>
-      </c>
-      <c r="N10" s="3" t="s">
+      <c r="O10" s="3" t="s">
+        <v>922</v>
+      </c>
+      <c r="P10" s="3" t="s">
         <v>672</v>
       </c>
-      <c r="O10" s="3" t="s">
-        <v>924</v>
-      </c>
-      <c r="P10" s="3" t="s">
-        <v>673</v>
-      </c>
-      <c r="Q10" s="3"/>
+      <c r="Q10" s="3" t="s">
+        <v>964</v>
+      </c>
       <c r="R10" s="3"/>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
+        <v>673</v>
+      </c>
+      <c r="B11" s="3" t="s">
         <v>674</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="C11" s="3" t="s">
+        <v>896</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>675</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>898</v>
-      </c>
-      <c r="D11" s="3" t="s">
+      <c r="E11" s="3" t="s">
         <v>676</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="F11" s="3" t="s">
         <v>677</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="G11" s="3" t="s">
         <v>678</v>
       </c>
-      <c r="G11" s="3" t="s">
+      <c r="H11" s="3" t="s">
         <v>679</v>
       </c>
-      <c r="H11" s="3" t="s">
+      <c r="I11" s="3" t="s">
+        <v>943</v>
+      </c>
+      <c r="J11" s="3" t="s">
         <v>680</v>
       </c>
-      <c r="I11" s="3" t="s">
-        <v>945</v>
-      </c>
-      <c r="J11" s="3" t="s">
+      <c r="K11" s="3" t="s">
         <v>681</v>
       </c>
-      <c r="K11" s="3" t="s">
+      <c r="L11" s="3" t="s">
         <v>682</v>
       </c>
-      <c r="L11" s="3" t="s">
+      <c r="M11" s="3" t="s">
         <v>683</v>
       </c>
-      <c r="M11" s="3" t="s">
+      <c r="N11" s="3" t="s">
         <v>684</v>
       </c>
-      <c r="N11" s="3" t="s">
-        <v>685</v>
-      </c>
       <c r="O11" s="3" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="P11" s="3" t="s">
-        <v>935</v>
-      </c>
-      <c r="Q11" s="3"/>
+        <v>933</v>
+      </c>
+      <c r="Q11" s="3" t="s">
+        <v>965</v>
+      </c>
       <c r="R11" s="3"/>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
+        <v>685</v>
+      </c>
+      <c r="B12" s="3" t="s">
         <v>686</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C12" s="3" t="s">
         <v>687</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="D12" s="3" t="s">
         <v>688</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="E12" s="3" t="s">
         <v>689</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="F12" s="3" t="s">
         <v>690</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="G12" s="3" t="s">
         <v>691</v>
       </c>
-      <c r="G12" s="3" t="s">
+      <c r="H12" s="3" t="s">
         <v>692</v>
       </c>
-      <c r="H12" s="3" t="s">
+      <c r="I12" s="3" t="s">
+        <v>944</v>
+      </c>
+      <c r="J12" s="3" t="s">
         <v>693</v>
       </c>
-      <c r="I12" s="3" t="s">
-        <v>946</v>
-      </c>
-      <c r="J12" s="3" t="s">
+      <c r="K12" s="3" t="s">
         <v>694</v>
       </c>
-      <c r="K12" s="3" t="s">
+      <c r="L12" s="3" t="s">
         <v>695</v>
       </c>
-      <c r="L12" s="3" t="s">
+      <c r="M12" s="3" t="s">
         <v>696</v>
       </c>
-      <c r="M12" s="3" t="s">
+      <c r="N12" s="3" t="s">
         <v>697</v>
       </c>
-      <c r="N12" s="3" t="s">
+      <c r="O12" s="3" t="s">
+        <v>923</v>
+      </c>
+      <c r="P12" s="3" t="s">
         <v>698</v>
       </c>
-      <c r="O12" s="3" t="s">
-        <v>925</v>
-      </c>
-      <c r="P12" s="3" t="s">
-        <v>699</v>
-      </c>
-      <c r="Q12" s="3"/>
+      <c r="Q12" s="3" t="s">
+        <v>966</v>
+      </c>
       <c r="R12" s="3"/>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
+        <v>699</v>
+      </c>
+      <c r="B13" s="3" t="s">
         <v>700</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="C13" s="3" t="s">
         <v>701</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="D13" s="3" t="s">
         <v>702</v>
       </c>
-      <c r="D13" s="3" t="s">
+      <c r="E13" s="3" t="s">
         <v>703</v>
       </c>
-      <c r="E13" s="3" t="s">
+      <c r="F13" s="3" t="s">
         <v>704</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="G13" s="3" t="s">
         <v>705</v>
       </c>
-      <c r="G13" s="3" t="s">
+      <c r="H13" s="3" t="s">
         <v>706</v>
       </c>
-      <c r="H13" s="3" t="s">
+      <c r="I13" s="3" t="s">
+        <v>945</v>
+      </c>
+      <c r="J13" s="3" t="s">
         <v>707</v>
       </c>
-      <c r="I13" s="3" t="s">
-        <v>947</v>
-      </c>
-      <c r="J13" s="3" t="s">
+      <c r="K13" s="3" t="s">
         <v>708</v>
       </c>
-      <c r="K13" s="3" t="s">
+      <c r="L13" s="3" t="s">
         <v>709</v>
       </c>
-      <c r="L13" s="3" t="s">
+      <c r="M13" s="3" t="s">
         <v>710</v>
       </c>
-      <c r="M13" s="3" t="s">
+      <c r="N13" s="3" t="s">
         <v>711</v>
       </c>
-      <c r="N13" s="3" t="s">
+      <c r="O13" s="3" t="s">
+        <v>669</v>
+      </c>
+      <c r="P13" s="3" t="s">
         <v>712</v>
       </c>
-      <c r="O13" s="3" t="s">
-        <v>670</v>
-      </c>
-      <c r="P13" s="3" t="s">
-        <v>713</v>
-      </c>
-      <c r="Q13" s="3"/>
+      <c r="Q13" s="3" t="s">
+        <v>967</v>
+      </c>
       <c r="R13" s="3"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
+        <v>713</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>714</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="C14" s="3" t="s">
         <v>715</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="D14" s="3" t="s">
         <v>716</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="E14" s="3" t="s">
         <v>717</v>
       </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="3" t="s">
         <v>718</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="3" t="s">
         <v>719</v>
       </c>
-      <c r="G14" s="3" t="s">
+      <c r="H14" s="3" t="s">
         <v>720</v>
       </c>
-      <c r="H14" s="3" t="s">
+      <c r="I14" s="3" t="s">
+        <v>946</v>
+      </c>
+      <c r="J14" s="3" t="s">
         <v>721</v>
       </c>
-      <c r="I14" s="3" t="s">
-        <v>948</v>
-      </c>
-      <c r="J14" s="3" t="s">
+      <c r="K14" s="3" t="s">
         <v>722</v>
       </c>
-      <c r="K14" s="3" t="s">
+      <c r="L14" s="3" t="s">
         <v>723</v>
       </c>
-      <c r="L14" s="3" t="s">
+      <c r="M14" s="3" t="s">
+        <v>908</v>
+      </c>
+      <c r="N14" s="3" t="s">
         <v>724</v>
       </c>
-      <c r="M14" s="3" t="s">
-        <v>910</v>
-      </c>
-      <c r="N14" s="3" t="s">
+      <c r="O14" s="3" t="s">
+        <v>924</v>
+      </c>
+      <c r="P14" s="3" t="s">
         <v>725</v>
       </c>
-      <c r="O14" s="3" t="s">
-        <v>926</v>
-      </c>
-      <c r="P14" s="3" t="s">
-        <v>726</v>
-      </c>
-      <c r="Q14" s="3"/>
+      <c r="Q14" s="3" t="s">
+        <v>968</v>
+      </c>
       <c r="R14" s="3"/>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
+        <v>726</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>727</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="C15" s="3" t="s">
         <v>728</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="D15" s="3" t="s">
         <v>729</v>
       </c>
-      <c r="D15" s="3" t="s">
+      <c r="E15" s="3" t="s">
         <v>730</v>
       </c>
-      <c r="E15" s="3" t="s">
+      <c r="F15" s="3" t="s">
         <v>731</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="G15" s="3" t="s">
         <v>732</v>
       </c>
-      <c r="G15" s="3" t="s">
+      <c r="H15" s="3" t="s">
         <v>733</v>
       </c>
-      <c r="H15" s="3" t="s">
+      <c r="I15" s="3" t="s">
+        <v>947</v>
+      </c>
+      <c r="J15" s="3" t="s">
         <v>734</v>
       </c>
-      <c r="I15" s="3" t="s">
-        <v>949</v>
-      </c>
-      <c r="J15" s="3" t="s">
+      <c r="K15" s="3" t="s">
         <v>735</v>
       </c>
-      <c r="K15" s="3" t="s">
+      <c r="L15" s="3" t="s">
         <v>736</v>
       </c>
-      <c r="L15" s="3" t="s">
+      <c r="M15" s="3" t="s">
         <v>737</v>
       </c>
-      <c r="M15" s="3" t="s">
+      <c r="N15" s="3" t="s">
         <v>738</v>
       </c>
-      <c r="N15" s="3" t="s">
+      <c r="O15" s="3" t="s">
+        <v>925</v>
+      </c>
+      <c r="P15" s="3" t="s">
         <v>739</v>
       </c>
-      <c r="O15" s="3" t="s">
-        <v>927</v>
-      </c>
-      <c r="P15" s="3" t="s">
-        <v>740</v>
-      </c>
-      <c r="Q15" s="3"/>
+      <c r="Q15" s="3" t="s">
+        <v>969</v>
+      </c>
       <c r="R15" s="3"/>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
+        <v>740</v>
+      </c>
+      <c r="B16" s="3" t="s">
         <v>741</v>
       </c>
-      <c r="B16" s="3" t="s">
+      <c r="C16" s="3" t="s">
         <v>742</v>
       </c>
-      <c r="C16" s="3" t="s">
+      <c r="D16" s="3" t="s">
         <v>743</v>
       </c>
-      <c r="D16" s="3" t="s">
+      <c r="E16" s="3" t="s">
         <v>744</v>
       </c>
-      <c r="E16" s="3" t="s">
+      <c r="F16" s="3" t="s">
         <v>745</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="G16" s="3" t="s">
         <v>746</v>
       </c>
-      <c r="G16" s="3" t="s">
+      <c r="H16" s="3" t="s">
         <v>747</v>
       </c>
-      <c r="H16" s="3" t="s">
+      <c r="I16" s="3" t="s">
+        <v>948</v>
+      </c>
+      <c r="J16" s="3" t="s">
         <v>748</v>
       </c>
-      <c r="I16" s="3" t="s">
-        <v>950</v>
-      </c>
-      <c r="J16" s="3" t="s">
+      <c r="K16" s="3" t="s">
         <v>749</v>
       </c>
-      <c r="K16" s="3" t="s">
+      <c r="L16" s="3" t="s">
         <v>750</v>
       </c>
-      <c r="L16" s="3" t="s">
+      <c r="M16" s="3" t="s">
         <v>751</v>
       </c>
-      <c r="M16" s="3" t="s">
+      <c r="N16" s="3" t="s">
         <v>752</v>
       </c>
-      <c r="N16" s="3" t="s">
+      <c r="O16" s="3" t="s">
+        <v>926</v>
+      </c>
+      <c r="P16" s="3" t="s">
         <v>753</v>
       </c>
-      <c r="O16" s="3" t="s">
-        <v>928</v>
-      </c>
-      <c r="P16" s="3" t="s">
-        <v>754</v>
-      </c>
-      <c r="Q16" s="3"/>
+      <c r="Q16" s="3" t="s">
+        <v>970</v>
+      </c>
       <c r="R16" s="3"/>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
+        <v>754</v>
+      </c>
+      <c r="B17" s="3" t="s">
         <v>755</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="C17" s="3" t="s">
         <v>756</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="D17" s="3" t="s">
         <v>757</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="E17" s="3" t="s">
         <v>758</v>
       </c>
-      <c r="E17" s="3" t="s">
+      <c r="F17" s="3" t="s">
         <v>759</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="G17" s="3" t="s">
         <v>760</v>
       </c>
-      <c r="G17" s="3" t="s">
+      <c r="H17" s="3" t="s">
         <v>761</v>
       </c>
-      <c r="H17" s="3" t="s">
+      <c r="I17" s="3" t="s">
+        <v>949</v>
+      </c>
+      <c r="J17" s="3" t="s">
         <v>762</v>
       </c>
-      <c r="I17" s="3" t="s">
-        <v>951</v>
-      </c>
-      <c r="J17" s="3" t="s">
+      <c r="K17" s="3" t="s">
         <v>763</v>
       </c>
-      <c r="K17" s="3" t="s">
+      <c r="L17" s="3" t="s">
         <v>764</v>
       </c>
-      <c r="L17" s="3" t="s">
+      <c r="M17" s="3" t="s">
         <v>765</v>
       </c>
-      <c r="M17" s="3" t="s">
+      <c r="N17" s="3" t="s">
         <v>766</v>
       </c>
-      <c r="N17" s="3" t="s">
+      <c r="O17" s="3" t="s">
+        <v>927</v>
+      </c>
+      <c r="P17" s="3" t="s">
         <v>767</v>
       </c>
-      <c r="O17" s="3" t="s">
-        <v>929</v>
-      </c>
-      <c r="P17" s="3" t="s">
-        <v>768</v>
-      </c>
-      <c r="Q17" s="3"/>
+      <c r="Q17" s="3" t="s">
+        <v>971</v>
+      </c>
       <c r="R17" s="3"/>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
+        <v>768</v>
+      </c>
+      <c r="B18" s="3" t="s">
         <v>769</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="C18" s="3" t="s">
         <v>770</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="D18" s="3" t="s">
         <v>771</v>
       </c>
-      <c r="D18" s="3" t="s">
+      <c r="E18" s="3" t="s">
         <v>772</v>
       </c>
-      <c r="E18" s="3" t="s">
+      <c r="F18" s="3" t="s">
         <v>773</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="G18" s="3" t="s">
         <v>774</v>
       </c>
-      <c r="G18" s="3" t="s">
+      <c r="H18" s="3" t="s">
         <v>775</v>
       </c>
-      <c r="H18" s="3" t="s">
+      <c r="I18" s="3" t="s">
+        <v>654</v>
+      </c>
+      <c r="J18" s="3" t="s">
         <v>776</v>
       </c>
-      <c r="I18" s="3" t="s">
-        <v>655</v>
-      </c>
-      <c r="J18" s="3" t="s">
+      <c r="K18" s="3" t="s">
         <v>777</v>
       </c>
-      <c r="K18" s="3" t="s">
+      <c r="L18" s="3" t="s">
         <v>778</v>
       </c>
-      <c r="L18" s="3" t="s">
+      <c r="M18" s="3" t="s">
+        <v>909</v>
+      </c>
+      <c r="N18" s="3" t="s">
         <v>779</v>
       </c>
-      <c r="M18" s="3" t="s">
-        <v>911</v>
-      </c>
-      <c r="N18" s="3" t="s">
+      <c r="O18" s="3" t="s">
+        <v>928</v>
+      </c>
+      <c r="P18" s="3" t="s">
         <v>780</v>
       </c>
-      <c r="O18" s="3" t="s">
-        <v>930</v>
-      </c>
-      <c r="P18" s="3" t="s">
-        <v>781</v>
-      </c>
-      <c r="Q18" s="3"/>
+      <c r="Q18" s="3" t="s">
+        <v>972</v>
+      </c>
       <c r="R18" s="3"/>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
+        <v>781</v>
+      </c>
+      <c r="B19" s="3" t="s">
         <v>782</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="C19" s="3" t="s">
         <v>783</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="D19" s="3" t="s">
         <v>784</v>
       </c>
-      <c r="D19" s="3" t="s">
+      <c r="E19" s="3" t="s">
         <v>785</v>
       </c>
-      <c r="E19" s="3" t="s">
+      <c r="F19" s="3" t="s">
         <v>786</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="G19" s="3" t="s">
         <v>787</v>
       </c>
-      <c r="G19" s="3" t="s">
+      <c r="H19" s="3" t="s">
         <v>788</v>
       </c>
-      <c r="H19" s="3" t="s">
+      <c r="I19" s="3" t="s">
+        <v>950</v>
+      </c>
+      <c r="J19" s="3" t="s">
         <v>789</v>
       </c>
-      <c r="I19" s="3" t="s">
-        <v>952</v>
-      </c>
-      <c r="J19" s="3" t="s">
+      <c r="K19" s="3" t="s">
         <v>790</v>
       </c>
-      <c r="K19" s="3" t="s">
+      <c r="L19" s="3" t="s">
         <v>791</v>
       </c>
-      <c r="L19" s="3" t="s">
+      <c r="M19" s="3" t="s">
+        <v>912</v>
+      </c>
+      <c r="N19" s="3" t="s">
         <v>792</v>
       </c>
-      <c r="M19" s="3" t="s">
-        <v>914</v>
-      </c>
-      <c r="N19" s="3" t="s">
+      <c r="O19" s="3" t="s">
+        <v>929</v>
+      </c>
+      <c r="P19" s="3" t="s">
         <v>793</v>
       </c>
-      <c r="O19" s="3" t="s">
-        <v>931</v>
-      </c>
-      <c r="P19" s="3" t="s">
-        <v>794</v>
-      </c>
-      <c r="Q19" s="3"/>
+      <c r="Q19" s="3" t="s">
+        <v>973</v>
+      </c>
       <c r="R19" s="3"/>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
+        <v>794</v>
+      </c>
+      <c r="B20" s="3" t="s">
         <v>795</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="C20" s="3" t="s">
         <v>796</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="D20" s="3" t="s">
         <v>797</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="E20" s="3" t="s">
         <v>798</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="F20" s="3" t="s">
         <v>799</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="G20" s="3" t="s">
         <v>800</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="H20" s="3" t="s">
         <v>801</v>
       </c>
-      <c r="H20" s="3" t="s">
+      <c r="I20" s="3" t="s">
+        <v>951</v>
+      </c>
+      <c r="J20" s="3" t="s">
         <v>802</v>
       </c>
-      <c r="I20" s="3" t="s">
-        <v>953</v>
-      </c>
-      <c r="J20" s="3" t="s">
+      <c r="K20" s="3" t="s">
         <v>803</v>
       </c>
-      <c r="K20" s="3" t="s">
+      <c r="L20" s="3" t="s">
         <v>804</v>
       </c>
-      <c r="L20" s="3" t="s">
+      <c r="M20" s="3" t="s">
         <v>805</v>
       </c>
-      <c r="M20" s="3" t="s">
+      <c r="N20" s="3" t="s">
         <v>806</v>
       </c>
-      <c r="N20" s="3" t="s">
+      <c r="O20" s="3" t="s">
+        <v>930</v>
+      </c>
+      <c r="P20" s="1" t="s">
         <v>807</v>
       </c>
-      <c r="O20" s="3" t="s">
-        <v>932</v>
-      </c>
-      <c r="P20" s="1" t="s">
-        <v>808</v>
-      </c>
-      <c r="Q20" s="3"/>
+      <c r="Q20" s="3" t="s">
+        <v>974</v>
+      </c>
       <c r="R20" s="3"/>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
+        <v>808</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>809</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="C21" s="3" t="s">
         <v>810</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="D21" s="3" t="s">
         <v>811</v>
       </c>
-      <c r="D21" s="3" t="s">
+      <c r="E21" s="3" t="s">
         <v>812</v>
       </c>
-      <c r="E21" s="3" t="s">
+      <c r="F21" s="3" t="s">
+        <v>898</v>
+      </c>
+      <c r="G21" s="3" t="s">
         <v>813</v>
       </c>
-      <c r="F21" s="3" t="s">
-        <v>900</v>
-      </c>
-      <c r="G21" s="3" t="s">
+      <c r="H21" s="3" t="s">
         <v>814</v>
       </c>
-      <c r="H21" s="3" t="s">
+      <c r="I21" s="3" t="s">
+        <v>952</v>
+      </c>
+      <c r="J21" s="3" t="s">
         <v>815</v>
       </c>
-      <c r="I21" s="3" t="s">
-        <v>954</v>
-      </c>
-      <c r="J21" s="3" t="s">
+      <c r="K21" s="3" t="s">
         <v>816</v>
       </c>
-      <c r="K21" s="3" t="s">
+      <c r="L21" s="3" t="s">
+        <v>905</v>
+      </c>
+      <c r="M21" s="3" t="s">
         <v>817</v>
       </c>
-      <c r="L21" s="3" t="s">
-        <v>907</v>
-      </c>
-      <c r="M21" s="3" t="s">
+      <c r="N21" s="3" t="s">
+        <v>913</v>
+      </c>
+      <c r="O21" s="3" t="s">
+        <v>931</v>
+      </c>
+      <c r="P21" s="3" t="s">
         <v>818</v>
-      </c>
-      <c r="N21" s="3" t="s">
-        <v>915</v>
-      </c>
-      <c r="O21" s="3" t="s">
-        <v>933</v>
-      </c>
-      <c r="P21" s="3" t="s">
-        <v>819</v>
       </c>
       <c r="Q21" s="3"/>
       <c r="R21" s="3"/>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
+        <v>819</v>
+      </c>
+      <c r="B22" s="3" t="s">
         <v>820</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="C22" s="3" t="s">
         <v>821</v>
       </c>
-      <c r="C22" s="3" t="s">
+      <c r="D22" s="3" t="s">
         <v>822</v>
       </c>
-      <c r="D22" s="3" t="s">
+      <c r="E22" s="3" t="s">
         <v>823</v>
       </c>
-      <c r="E22" s="3" t="s">
+      <c r="F22" s="3" t="s">
         <v>824</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="G22" s="3" t="s">
         <v>825</v>
       </c>
-      <c r="G22" s="3" t="s">
+      <c r="H22" s="3" t="s">
         <v>826</v>
       </c>
-      <c r="H22" s="3" t="s">
+      <c r="I22" s="3" t="s">
+        <v>828</v>
+      </c>
+      <c r="J22" s="3" t="s">
         <v>827</v>
       </c>
-      <c r="I22" s="3" t="s">
+      <c r="K22" s="3" t="s">
         <v>829</v>
       </c>
-      <c r="J22" s="3" t="s">
-        <v>828</v>
-      </c>
-      <c r="K22" s="3" t="s">
+      <c r="L22" s="3" t="s">
         <v>830</v>
       </c>
-      <c r="L22" s="3" t="s">
+      <c r="M22" s="3" t="s">
+        <v>910</v>
+      </c>
+      <c r="N22" s="3" t="s">
         <v>831</v>
       </c>
-      <c r="M22" s="3" t="s">
-        <v>912</v>
-      </c>
-      <c r="N22" s="3" t="s">
+      <c r="O22" s="3" t="s">
+        <v>894</v>
+      </c>
+      <c r="P22" s="3" t="s">
         <v>832</v>
-      </c>
-      <c r="O22" s="3" t="s">
-        <v>896</v>
-      </c>
-      <c r="P22" s="3" t="s">
-        <v>833</v>
       </c>
       <c r="Q22" s="3"/>
       <c r="R22" s="3"/>
     </row>
     <row r="23" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
+        <v>833</v>
+      </c>
+      <c r="B23" s="3" t="s">
         <v>834</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="C23" s="3" t="s">
         <v>835</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="D23" s="3" t="s">
         <v>836</v>
       </c>
-      <c r="D23" s="3" t="s">
+      <c r="E23" s="3" t="s">
         <v>837</v>
       </c>
-      <c r="E23" s="3" t="s">
+      <c r="F23" s="3" t="s">
         <v>838</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="G23" s="3" t="s">
         <v>839</v>
       </c>
-      <c r="G23" s="3" t="s">
+      <c r="H23" s="3" t="s">
         <v>840</v>
       </c>
-      <c r="H23" s="3" t="s">
+      <c r="I23" s="3" t="s">
+        <v>953</v>
+      </c>
+      <c r="J23" s="3" t="s">
         <v>841</v>
       </c>
-      <c r="I23" s="3" t="s">
-        <v>955</v>
-      </c>
-      <c r="J23" s="3" t="s">
+      <c r="K23" s="3" t="s">
         <v>842</v>
       </c>
-      <c r="K23" s="3" t="s">
+      <c r="L23" s="3" t="s">
         <v>843</v>
       </c>
-      <c r="L23" s="3" t="s">
-        <v>844</v>
-      </c>
       <c r="M23" s="3" t="s">
-        <v>913</v>
+        <v>911</v>
       </c>
       <c r="N23" s="3" t="s">
-        <v>895</v>
+        <v>893</v>
       </c>
       <c r="O23" s="3" t="s">
-        <v>894</v>
+        <v>892</v>
       </c>
       <c r="P23" s="3" t="s">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="Q23" s="3"/>
       <c r="R23" s="3"/>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
+        <v>844</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>895</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>845</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>897</v>
-      </c>
-      <c r="C24" s="3" t="s">
+      <c r="D24" s="3" t="s">
         <v>846</v>
       </c>
-      <c r="D24" s="3" t="s">
+      <c r="E24" s="3" t="s">
         <v>847</v>
       </c>
-      <c r="E24" s="3" t="s">
+      <c r="F24" s="3" t="s">
+        <v>899</v>
+      </c>
+      <c r="G24" s="3" t="s">
         <v>848</v>
       </c>
-      <c r="F24" s="3" t="s">
-        <v>901</v>
-      </c>
-      <c r="G24" s="3" t="s">
+      <c r="H24" s="3" t="s">
         <v>849</v>
       </c>
-      <c r="H24" s="3" t="s">
+      <c r="I24" s="3" t="s">
+        <v>954</v>
+      </c>
+      <c r="J24" s="3" t="s">
         <v>850</v>
       </c>
-      <c r="I24" s="3" t="s">
-        <v>956</v>
-      </c>
-      <c r="J24" s="3" t="s">
+      <c r="K24" s="3" t="s">
         <v>851</v>
       </c>
-      <c r="K24" s="3" t="s">
+      <c r="L24" s="3" t="s">
         <v>852</v>
       </c>
-      <c r="L24" s="3" t="s">
+      <c r="M24" s="3" t="s">
         <v>853</v>
       </c>
-      <c r="M24" s="3" t="s">
+      <c r="N24" s="3" t="s">
+        <v>914</v>
+      </c>
+      <c r="O24" s="3" t="s">
+        <v>932</v>
+      </c>
+      <c r="P24" s="3" t="s">
         <v>854</v>
-      </c>
-      <c r="N24" s="3" t="s">
-        <v>916</v>
-      </c>
-      <c r="O24" s="3" t="s">
-        <v>934</v>
-      </c>
-      <c r="P24" s="3" t="s">
-        <v>855</v>
       </c>
       <c r="Q24" s="3"/>
       <c r="R24" s="3"/>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
     </row>
   </sheetData>
@@ -13847,7 +13962,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.44140625" bestFit="1" customWidth="1"/>
@@ -13965,13 +14080,13 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>887</v>
+        <v>886</v>
       </c>
       <c r="B5" t="s">
+        <v>889</v>
+      </c>
+      <c r="C5" t="s">
         <v>890</v>
-      </c>
-      <c r="C5" t="s">
-        <v>891</v>
       </c>
       <c r="D5" t="s">
         <v>23</v>
@@ -13983,7 +14098,7 @@
         <v>300000000</v>
       </c>
       <c r="G5" t="s">
-        <v>892</v>
+        <v>978</v>
       </c>
       <c r="H5">
         <v>14</v>
@@ -14136,7 +14251,7 @@
         <v>100000000</v>
       </c>
       <c r="F11" s="12">
-        <v>1123000000</v>
+        <v>1000000000</v>
       </c>
       <c r="G11" t="s">
         <v>51</v>
@@ -14299,6 +14414,32 @@
       </c>
       <c r="H17">
         <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>955</v>
+      </c>
+      <c r="B18" t="s">
+        <v>975</v>
+      </c>
+      <c r="C18" t="s">
+        <v>976</v>
+      </c>
+      <c r="D18" t="s">
+        <v>977</v>
+      </c>
+      <c r="E18">
+        <v>100000000</v>
+      </c>
+      <c r="F18" s="12">
+        <v>300000000</v>
+      </c>
+      <c r="G18" t="s">
+        <v>979</v>
+      </c>
+      <c r="H18">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajustes en PDF y Excel, control de duplicados y manejo de errores en mercado
</commit_message>
<xml_diff>
--- a/lmi temp 9.xlsx
+++ b/lmi temp 9.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alex1\Downloads\LMI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{520C08AE-A86C-4BB7-8B4E-A80D2952339A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91A99464-2C4F-4C1C-A5E3-256A37D38EAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="2" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1473" uniqueCount="996">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1652" uniqueCount="1014">
   <si>
     <t>Equipo</t>
   </si>
@@ -3071,6 +3071,60 @@
   </si>
   <si>
     <t>Intercambio de Jugadores</t>
+  </si>
+  <si>
+    <t>Compra</t>
+  </si>
+  <si>
+    <t>Benjamin Sesko</t>
+  </si>
+  <si>
+    <t>T. Alexander-Arnold</t>
+  </si>
+  <si>
+    <t>James Rodriguez</t>
+  </si>
+  <si>
+    <t>Joan Garcia</t>
+  </si>
+  <si>
+    <t>Pedro Porro</t>
+  </si>
+  <si>
+    <t>Fc Barcelona</t>
+  </si>
+  <si>
+    <t>Jules Kounde</t>
+  </si>
+  <si>
+    <t>Joao Pedro</t>
+  </si>
+  <si>
+    <t>Joao Neves</t>
+  </si>
+  <si>
+    <t>Ac Milan</t>
+  </si>
+  <si>
+    <t>David Raya</t>
+  </si>
+  <si>
+    <t>Son Heung Min</t>
+  </si>
+  <si>
+    <t>Leandro Trossard</t>
+  </si>
+  <si>
+    <t>Estevao</t>
+  </si>
+  <si>
+    <t>Prestamo</t>
+  </si>
+  <si>
+    <t>Prestamo de jugadores</t>
+  </si>
+  <si>
+    <t>Luka Modric</t>
   </si>
 </sst>
 </file>
@@ -14196,7 +14250,7 @@
         <v>100000000</v>
       </c>
       <c r="F7" s="12">
-        <v>1752000000</v>
+        <v>2152000000</v>
       </c>
       <c r="G7" t="s">
         <v>36</v>
@@ -14352,7 +14406,7 @@
         <v>100000000</v>
       </c>
       <c r="F13" s="12">
-        <v>2390000000</v>
+        <v>2690000000</v>
       </c>
       <c r="G13" t="s">
         <v>64</v>
@@ -14498,7 +14552,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
@@ -14550,6 +14604,9 @@
       <c r="E2">
         <v>25</v>
       </c>
+      <c r="F2" t="s">
+        <v>994</v>
+      </c>
       <c r="G2" t="s">
         <v>989</v>
       </c>
@@ -14570,6 +14627,9 @@
       <c r="E3">
         <v>50</v>
       </c>
+      <c r="F3" t="s">
+        <v>994</v>
+      </c>
       <c r="G3" t="s">
         <v>989</v>
       </c>
@@ -14590,6 +14650,9 @@
       <c r="E4">
         <v>120</v>
       </c>
+      <c r="F4" t="s">
+        <v>994</v>
+      </c>
       <c r="G4" t="s">
         <v>989</v>
       </c>
@@ -14610,6 +14673,9 @@
       <c r="E5">
         <v>65</v>
       </c>
+      <c r="F5" t="s">
+        <v>994</v>
+      </c>
       <c r="G5" t="s">
         <v>989</v>
       </c>
@@ -14630,6 +14696,9 @@
       <c r="E6">
         <v>90</v>
       </c>
+      <c r="F6" t="s">
+        <v>994</v>
+      </c>
       <c r="G6" t="s">
         <v>989</v>
       </c>
@@ -14650,6 +14719,9 @@
       <c r="E7">
         <v>170</v>
       </c>
+      <c r="F7" t="s">
+        <v>994</v>
+      </c>
       <c r="G7" t="s">
         <v>989</v>
       </c>
@@ -14697,6 +14769,673 @@
         <v>994</v>
       </c>
       <c r="G9" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>131</v>
+      </c>
+      <c r="B10" t="s">
+        <v>996</v>
+      </c>
+      <c r="C10" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" t="s">
+        <v>75</v>
+      </c>
+      <c r="E10">
+        <v>68</v>
+      </c>
+      <c r="F10" t="s">
+        <v>994</v>
+      </c>
+      <c r="G10" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>558</v>
+      </c>
+      <c r="B11" t="s">
+        <v>996</v>
+      </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" t="s">
+        <v>75</v>
+      </c>
+      <c r="E11">
+        <v>65</v>
+      </c>
+      <c r="F11" t="s">
+        <v>994</v>
+      </c>
+      <c r="G11" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>997</v>
+      </c>
+      <c r="B12" t="s">
+        <v>988</v>
+      </c>
+      <c r="C12" t="s">
+        <v>75</v>
+      </c>
+      <c r="D12" t="s">
+        <v>60</v>
+      </c>
+      <c r="E12">
+        <v>100</v>
+      </c>
+      <c r="F12" t="s">
+        <v>994</v>
+      </c>
+      <c r="G12" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>998</v>
+      </c>
+      <c r="B13" t="s">
+        <v>988</v>
+      </c>
+      <c r="C13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" t="s">
+        <v>70</v>
+      </c>
+      <c r="E13">
+        <v>90</v>
+      </c>
+      <c r="F13" t="s">
+        <v>994</v>
+      </c>
+      <c r="G13" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>260</v>
+      </c>
+      <c r="B14" t="s">
+        <v>986</v>
+      </c>
+      <c r="C14" t="s">
+        <v>75</v>
+      </c>
+      <c r="D14" t="s">
+        <v>65</v>
+      </c>
+      <c r="E14">
+        <v>0</v>
+      </c>
+      <c r="F14" t="s">
+        <v>994</v>
+      </c>
+      <c r="G14" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>999</v>
+      </c>
+      <c r="B15" t="s">
+        <v>986</v>
+      </c>
+      <c r="C15" t="s">
+        <v>65</v>
+      </c>
+      <c r="D15" t="s">
+        <v>75</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15" t="s">
+        <v>994</v>
+      </c>
+      <c r="G15" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>1000</v>
+      </c>
+      <c r="B16" t="s">
+        <v>996</v>
+      </c>
+      <c r="C16" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" t="s">
+        <v>70</v>
+      </c>
+      <c r="E16">
+        <v>75</v>
+      </c>
+      <c r="F16" t="s">
+        <v>994</v>
+      </c>
+      <c r="G16" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>1001</v>
+      </c>
+      <c r="B17" t="s">
+        <v>996</v>
+      </c>
+      <c r="C17" t="s">
+        <v>56</v>
+      </c>
+      <c r="D17" t="s">
+        <v>70</v>
+      </c>
+      <c r="E17">
+        <v>60</v>
+      </c>
+      <c r="F17" t="s">
+        <v>994</v>
+      </c>
+      <c r="G17" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>590</v>
+      </c>
+      <c r="B18" t="s">
+        <v>988</v>
+      </c>
+      <c r="C18" t="s">
+        <v>70</v>
+      </c>
+      <c r="D18" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18">
+        <v>20</v>
+      </c>
+      <c r="F18" t="s">
+        <v>994</v>
+      </c>
+      <c r="G18" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>293</v>
+      </c>
+      <c r="B19" t="s">
+        <v>996</v>
+      </c>
+      <c r="C19" t="s">
+        <v>1002</v>
+      </c>
+      <c r="D19" t="s">
+        <v>42</v>
+      </c>
+      <c r="E19">
+        <v>130</v>
+      </c>
+      <c r="F19" t="s">
+        <v>994</v>
+      </c>
+      <c r="G19" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>1003</v>
+      </c>
+      <c r="B20" t="s">
+        <v>986</v>
+      </c>
+      <c r="C20" t="s">
+        <v>1002</v>
+      </c>
+      <c r="D20" t="s">
+        <v>42</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20" t="s">
+        <v>994</v>
+      </c>
+      <c r="G20" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>363</v>
+      </c>
+      <c r="B21" t="s">
+        <v>986</v>
+      </c>
+      <c r="C21" t="s">
+        <v>42</v>
+      </c>
+      <c r="D21" t="s">
+        <v>1002</v>
+      </c>
+      <c r="E21">
+        <v>0</v>
+      </c>
+      <c r="F21" t="s">
+        <v>994</v>
+      </c>
+      <c r="G21" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>1004</v>
+      </c>
+      <c r="B22" t="s">
+        <v>996</v>
+      </c>
+      <c r="C22" t="s">
+        <v>13</v>
+      </c>
+      <c r="D22" t="s">
+        <v>1002</v>
+      </c>
+      <c r="E22">
+        <v>136</v>
+      </c>
+      <c r="F22" t="s">
+        <v>994</v>
+      </c>
+      <c r="G22" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B23" t="s">
+        <v>986</v>
+      </c>
+      <c r="C23" t="s">
+        <v>32</v>
+      </c>
+      <c r="D23" t="s">
+        <v>1002</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23" t="s">
+        <v>994</v>
+      </c>
+      <c r="G23" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>294</v>
+      </c>
+      <c r="B24" t="s">
+        <v>986</v>
+      </c>
+      <c r="C24" t="s">
+        <v>1002</v>
+      </c>
+      <c r="D24" t="s">
+        <v>32</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24" t="s">
+        <v>994</v>
+      </c>
+      <c r="G24" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>195</v>
+      </c>
+      <c r="B25" t="s">
+        <v>986</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1006</v>
+      </c>
+      <c r="D25" t="s">
+        <v>1002</v>
+      </c>
+      <c r="E25">
+        <v>0</v>
+      </c>
+      <c r="F25" t="s">
+        <v>994</v>
+      </c>
+      <c r="G25" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>299</v>
+      </c>
+      <c r="B26" t="s">
+        <v>986</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1002</v>
+      </c>
+      <c r="D26" t="s">
+        <v>1006</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26" t="s">
+        <v>994</v>
+      </c>
+      <c r="G26" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>1007</v>
+      </c>
+      <c r="B27" t="s">
+        <v>996</v>
+      </c>
+      <c r="C27" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" t="s">
+        <v>47</v>
+      </c>
+      <c r="E27">
+        <v>50</v>
+      </c>
+      <c r="F27" t="s">
+        <v>994</v>
+      </c>
+      <c r="G27" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>188</v>
+      </c>
+      <c r="B28" t="s">
+        <v>988</v>
+      </c>
+      <c r="C28" t="s">
+        <v>47</v>
+      </c>
+      <c r="D28" t="s">
+        <v>85</v>
+      </c>
+      <c r="E28">
+        <v>25</v>
+      </c>
+      <c r="F28" t="s">
+        <v>994</v>
+      </c>
+      <c r="G28" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>1008</v>
+      </c>
+      <c r="B29" t="s">
+        <v>986</v>
+      </c>
+      <c r="C29" t="s">
+        <v>23</v>
+      </c>
+      <c r="D29" t="s">
+        <v>47</v>
+      </c>
+      <c r="E29">
+        <v>0</v>
+      </c>
+      <c r="F29" t="s">
+        <v>994</v>
+      </c>
+      <c r="G29" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>422</v>
+      </c>
+      <c r="B30" t="s">
+        <v>986</v>
+      </c>
+      <c r="C30" t="s">
+        <v>47</v>
+      </c>
+      <c r="D30" t="s">
+        <v>23</v>
+      </c>
+      <c r="E30">
+        <v>0</v>
+      </c>
+      <c r="F30" t="s">
+        <v>994</v>
+      </c>
+      <c r="G30" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>503</v>
+      </c>
+      <c r="B31" t="s">
+        <v>996</v>
+      </c>
+      <c r="C31" t="s">
+        <v>42</v>
+      </c>
+      <c r="D31" t="s">
+        <v>13</v>
+      </c>
+      <c r="E31">
+        <v>80</v>
+      </c>
+      <c r="F31" t="s">
+        <v>994</v>
+      </c>
+      <c r="G31" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B32" t="s">
+        <v>996</v>
+      </c>
+      <c r="C32" t="s">
+        <v>56</v>
+      </c>
+      <c r="D32" t="s">
+        <v>13</v>
+      </c>
+      <c r="E32">
+        <v>20</v>
+      </c>
+      <c r="F32" t="s">
+        <v>994</v>
+      </c>
+      <c r="G32" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>121</v>
+      </c>
+      <c r="B33" t="s">
+        <v>988</v>
+      </c>
+      <c r="C33" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" t="s">
+        <v>85</v>
+      </c>
+      <c r="E33">
+        <v>20</v>
+      </c>
+      <c r="F33" t="s">
+        <v>994</v>
+      </c>
+      <c r="G33" t="s">
+        <v>989</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>585</v>
+      </c>
+      <c r="B34" t="s">
+        <v>986</v>
+      </c>
+      <c r="C34" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" t="s">
+        <v>56</v>
+      </c>
+      <c r="E34">
+        <v>60</v>
+      </c>
+      <c r="F34" t="s">
+        <v>994</v>
+      </c>
+      <c r="G34" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>1010</v>
+      </c>
+      <c r="B35" t="s">
+        <v>986</v>
+      </c>
+      <c r="C35" t="s">
+        <v>56</v>
+      </c>
+      <c r="D35" t="s">
+        <v>13</v>
+      </c>
+      <c r="E35">
+        <v>60</v>
+      </c>
+      <c r="F35" t="s">
+        <v>994</v>
+      </c>
+      <c r="G35" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>264</v>
+      </c>
+      <c r="B36" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C36" t="s">
+        <v>60</v>
+      </c>
+      <c r="D36" t="s">
+        <v>37</v>
+      </c>
+      <c r="E36">
+        <v>60</v>
+      </c>
+      <c r="F36">
+        <v>2</v>
+      </c>
+      <c r="G36" t="s">
+        <v>1012</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>480</v>
+      </c>
+      <c r="B37" t="s">
+        <v>986</v>
+      </c>
+      <c r="C37" t="s">
+        <v>60</v>
+      </c>
+      <c r="D37" t="s">
+        <v>23</v>
+      </c>
+      <c r="E37">
+        <v>20</v>
+      </c>
+      <c r="F37" t="s">
+        <v>994</v>
+      </c>
+      <c r="G37" t="s">
+        <v>995</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>1013</v>
+      </c>
+      <c r="B38" t="s">
+        <v>986</v>
+      </c>
+      <c r="C38" t="s">
+        <v>23</v>
+      </c>
+      <c r="D38" t="s">
+        <v>60</v>
+      </c>
+      <c r="E38">
+        <v>20</v>
+      </c>
+      <c r="F38" t="s">
+        <v>994</v>
+      </c>
+      <c r="G38" t="s">
         <v>995</v>
       </c>
     </row>

</xml_diff>